<commit_message>
docs: add Testing Plan sheet (unit through GA) to the SaaS tracker
New tab covers every test type needed before going live: automated
(unit/integration/regression), multi-tenant isolation matrix, security/
pentest, load & performance (baseline/concurrency/spike/soak/DB volume),
resilience (multi-replica/chaos), migration & backup/DR drills, then the
Alpha -> Closed Beta -> Staged Open Beta -> GA rollout milestones with
entry/exit criteria and tenant counts for each stage. Wired into the
Dashboard (testing sign-off KPI) and Go-Live Checklist (new gate item).
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Task Backlog" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Kanban Board" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Go-Live Checklist" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Testing Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Go-Live Checklist" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="45">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -238,6 +239,18 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
     </font>
@@ -266,8 +279,13 @@
       <color rgb="0038761D"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -354,6 +372,26 @@
         <fgColor rgb="001155CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00990000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00666666"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B5394"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00134F5C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -381,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -522,18 +560,86 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1003,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1046,7 +1152,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Dashboard — live rollup of every sprint: task counts, % complete, and the overall go-live gate status. All formulas — edit Status on Task Backlog and this updates itself.</t>
+          <t>Dashboard — live rollup of every sprint AND the Testing Plan: task counts, % complete, open P0s, and the overall go-live gate status. All formulas — edit Status on Task Backlog / Testing Plan and this updates itself.</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1164,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Task Backlog — the single source of truth. One row per task. Change the Status dropdown as work moves; this drives the Dashboard and is the sortable/filterable 'sprint sheet.'</t>
+          <t>Task Backlog — the single source of truth for engineering work. One row per fix. Change the Status dropdown as work moves; this drives the Dashboard and is the sortable/filterable 'sprint sheet.'</t>
         </is>
       </c>
     </row>
@@ -1082,119 +1188,131 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Go-Live Checklist — the final gate. Every row must be checked TRUE before opening self-serve signup or onboarding client #1 at scale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+          <t>Testing Plan — every test type required before going live (automated, multi-tenant isolation, security, load/performance, resilience, migration/backup) PLUS the Alpha -&gt; Closed Beta -&gt; Staged Beta -&gt; GA rollout milestones with entry/exit criteria for each stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Go-Live Checklist — the final gate. Every row must be checked TRUE before opening self-serve signup or onboarding client #1 at scale — includes a line item confirming every Testing Plan phase passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Legend — Priority</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Ship-blocker — must close before the next tenant / go-live gate it sits in</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Fix before selling to a real customer — not an immediate blocker but close soon</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Quality/hardening — schedule once P0/P1 are clear</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Legend — Status</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>In Review</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Cells to edit</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>On Task Backlog: Status, Owner, Start Date, Due Date, and Notes are yours to fill in / update (shown with a light yellow fill on the header). Everything else documents the finding and should not need editing.</t>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>On Task Backlog: Status, Owner, Start Date, Due Date, and Notes are yours to fill in / update. On Testing Plan: Status and Owner are yours to update. On Go-Live Checklist: set Done? to TRUE only once verified. All editable columns are shown with a gold header fill. Everything else documents the finding and should not need editing.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
@@ -1290,14 +1408,25 @@
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="4" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Testing Plan phases not yet Passed</t>
+        </is>
+      </c>
+      <c r="C10" s="17">
+        <f>COUNTIF('Testing Plan'!I13:I33,"&lt;&gt;Passed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>READY FOR 100-CLIENT SaaS?</t>
         </is>
       </c>
-      <c r="C11" s="19">
-        <f>IF(C9=0,"READY — all go-live blockers closed","NOT READY — "&amp;C9&amp;" blocker(s) still open")</f>
+      <c r="C12" s="19">
+        <f>IF(AND(C9=0,C10=0),"READY — all go-live blockers closed and every testing phase passed","NOT READY — "&amp;C9&amp;" blocker(s) open, "&amp;C10&amp;" testing phase(s) not yet Passed")</f>
         <v/>
       </c>
     </row>
@@ -1538,15 +1667,15 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="C12:H12"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="C11:H11"/>
   </mergeCells>
-  <conditionalFormatting sqref="C11">
+  <conditionalFormatting sqref="C12">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$C$9=0</formula>
+      <formula>AND($C$9=0,$C$10=0)</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$C$9&gt;0</formula>
+      <formula>OR($C$9&gt;0,$C$10&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5379,7 +5508,1419 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Testing Plan — from automated tests through Alpha, Beta, and GA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Every test type required before going live, sequenced by phase, plus the Alpha -&gt; Closed Beta -&gt; Staged Beta -&gt; GA rollout milestones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Rollout Milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Tenant Count</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Entry Criteria</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Exit Criteria / Pass Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Internal Alpha</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>0 (internal only)</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>1-2 weeks</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 0 + 1 P0 Done, automated suite green</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>Zero open P0/P1 after full manual walkthrough of every module + baseline load test</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Closed Beta</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>3-5 design partners</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>2-4 weeks</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Alpha exit met + Sprint 2 + 3 Done + backup/restore drill passed</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>No P0 incidents, daily active usage from most partners, isolation matrix 100% pass, 1+ non-textile tenant validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Staged Open Beta</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>10 -&gt; 30 -&gt; 50 tenants</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>3-6 weeks (tiered)</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>Closed Beta exit met + Sprint 5 Done</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>SLO held at every tier, zero scheduler/cross-tenant incidents, support load manageable</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>General Availability</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>100+ / self-serve</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>Staged Beta exit met + Go-Live Checklist 100% + go/no-go held</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Sustained SLA at target traffic, zero open P0s for a full monitoring cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Detailed Test Plan — by phase</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="62" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B12" s="62" t="inlineStr">
+        <is>
+          <t>Test Type</t>
+        </is>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>What It Verifies</t>
+        </is>
+      </c>
+      <c r="D12" s="62" t="inlineStr">
+        <is>
+          <t>Scope / Method</t>
+        </is>
+      </c>
+      <c r="E12" s="62" t="inlineStr">
+        <is>
+          <t>Entry Criteria</t>
+        </is>
+      </c>
+      <c r="F12" s="62" t="inlineStr">
+        <is>
+          <t>Exit Criteria / Pass Bar</t>
+        </is>
+      </c>
+      <c r="G12" s="62" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="H12" s="62" t="inlineStr">
+        <is>
+          <t>Linked Sprint</t>
+        </is>
+      </c>
+      <c r="I12" s="63" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J12" s="63" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="64" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>Unit Testing</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Individual functions/handlers behave correctly in isolation (auth, RBAC, compute handlers, operating-model resolver, etc.)</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>pytest, run on every PR (backend/pytest.ini, backend/tests/)</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Code written</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>100% of new/changed code has a passing unit test; suite green in CI</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>Dev / CI</t>
+        </is>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 0-5 (continuous)</t>
+        </is>
+      </c>
+      <c r="I13" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J13" s="34" t="inlineStr"/>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="64" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>Integration Testing</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Full request/response flow across routers + DB for each domain (auth, tasks, decisions, workflows, brain, ledger)</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>pytest against a real test Mongo instance, one suite per router domain</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>Unit suite green</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>Every endpoint touched by Sprints 0-3 has at least one integration test; suite green</t>
+        </is>
+      </c>
+      <c r="G14" s="34" t="inlineStr">
+        <is>
+          <t>Dev / CI</t>
+        </is>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 0-3</t>
+        </is>
+      </c>
+      <c r="I14" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J14" s="34" t="inlineStr"/>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>Regression Testing</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Nothing that used to work broke as a result of this round of fixes</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Full automated suite re-run after each sprint merges to the branch</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>Each sprint's tasks marked Done</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Zero net-new failures vs. the pre-sprint baseline run</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>Every sprint</t>
+        </is>
+      </c>
+      <c r="I15" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J15" s="34" t="inlineStr"/>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="65" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>Multi-Tenant Isolation Test Matrix</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>No cross-tenant read/write is possible on ANY collection, endpoint, or background job</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>Scripted test: create 2+ tenants with overlapping data (incl. same phone number per S2-03), attempt cross-tenant read/write/delete on every collection + every _ensure_owned call site from S2-01</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 2 tasks Done</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>100% pass — zero cross-tenant access possible, incl. OTP/WhatsApp phone routing and tenant deletion completeness</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I16" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="inlineStr"/>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="65" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="inlineStr">
+        <is>
+          <t>Dynamic-Workflow Multi-Tenant Test</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>A NON-textile tenant (e.g. restaurant/clinic) gets a correctly working approval + payment-tracking loop, not just the textile demo</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>Onboard a synthetic non-textile tenant, run its AI-designed pipeline end to end incl. owner approval + dashboard KPIs</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>S1-06 Done</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>Approval gate, pending-purchases dashboard, and payment-overdue alerts all fire correctly for the non-textile pipeline</t>
+        </is>
+      </c>
+      <c r="G17" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I17" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J17" s="34" t="inlineStr"/>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="66" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B18" s="34" t="inlineStr">
+        <is>
+          <t>Security / Penetration Testing</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Every Sprint 0 vulnerability is actually closed, not just patched in one spot</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>Manual + tool-assisted (OWASP ZAP or similar): CORS/CSRF exploit attempt, unauth file access, JWT tampering, WhatsApp signature bypass, brute-force login, superadmin default creds</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 0 tasks Done</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>Zero exploitable findings on the Sprint 0 issue list; independent reviewer (or external pentest) sign-off</t>
+        </is>
+      </c>
+      <c r="G18" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="I18" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J18" s="34" t="inlineStr"/>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="66" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>RBAC / Permission Audit</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Every role sees exactly what it should and nothing more (finance data, admin routes, brain visibility rules)</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>Scripted test matrix: role x endpoint x expected access, incl. brain_rbac intents and document visibility rules</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 0-2 Done</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>100% pass on the role x endpoint matrix</t>
+        </is>
+      </c>
+      <c r="G19" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 0-2</t>
+        </is>
+      </c>
+      <c r="I19" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J19" s="34" t="inlineStr"/>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t>Load / Performance Testing — Baseline</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Normal-traffic response times meet SLO before adding concurrency</t>
+        </is>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>k6 or Locust against staging, single-tenant, ramping requests per endpoint</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 1 Done, staging live (S5-01)</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>P95 latency within target (e.g. &lt;500ms for reads, &lt;3s for AI-backed endpoints) at expected steady load</t>
+        </is>
+      </c>
+      <c r="G20" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I20" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J20" s="34" t="inlineStr"/>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>Load Testing — Multi-Tenant Concurrency</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>The system holds up with ~100 tenants' worth of simultaneous traffic, not just one tenant at a time</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>k6/Locust simulating 100 tenants concurrently hitting dashboards, /ask, and voice-capture together (S5-02)</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>Baseline load test passed</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>No error-rate spike, no shared-LLM-key 429 cascade (validates S1-05), DB pool holds under SUMMED load</t>
+        </is>
+      </c>
+      <c r="G21" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I21" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J21" s="34" t="inlineStr"/>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="67" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="inlineStr">
+        <is>
+          <t>Spike / Burst Testing</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>A sudden burst (e.g. many tenants' morning login + voice-capture rush) doesn't cascade into an outage</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Short high-intensity burst against the follow-up-scheduler window and login/OTP path</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Multi-tenant load test passed</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>System recovers within target time with no dropped requests beyond configured rate limits</t>
+        </is>
+      </c>
+      <c r="G22" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I22" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J22" s="34" t="inlineStr"/>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>Soak / Endurance Testing</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>No slow memory leak, connection-pool exhaustion, or gradual degradation over sustained runtime</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Run realistic traffic continuously for 24-48h on staging</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>Spike test passed</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>No degradation in latency/error-rate/memory over the full run</t>
+        </is>
+      </c>
+      <c r="G23" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I23" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J23" s="34" t="inlineStr"/>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="67" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t>Database Query Performance at Volume</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>Indexes actually get used and stay fast as data grows, not just at demo-tenant scale</t>
+        </is>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Seed staging with ~50k tasks / 10k contacts / 20k invoices across many tenants; profile the hot dashboard + /ask queries</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Schema fixes (S2-08, SCALE items) Done</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>No full-collection scans on hot paths; dashboard/brief load within SLO at seeded volume</t>
+        </is>
+      </c>
+      <c r="G24" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 1-2</t>
+        </is>
+      </c>
+      <c r="I24" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J24" s="34" t="inlineStr"/>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="68" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B25" s="34" t="inlineStr">
+        <is>
+          <t>Multi-Replica / Concurrency Testing</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>Running 3+ app replicas doesn't duplicate scheduled work or race on startup</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Deploy 3 replicas on staging; verify the follow-up scheduler fires exactly once per interval, not 3x (validates S1-01); verify index/migration bootstrap doesn't race</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 1 Done, real deploy config (S1-04) exists</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>Zero duplicate escalation emails/alerts observed across a full scheduler interval with 3 replicas running</t>
+        </is>
+      </c>
+      <c r="G25" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="I25" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J25" s="34" t="inlineStr"/>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="68" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>Failure-Injection / Chaos Testing</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>The system degrades gracefully, not catastrophically, when a dependency fails</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Kill a replica mid-request, simulate the LLM provider timing out/erroring, simulate a DB connection drop</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>Multi-replica test passed</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>In-flight requests fail cleanly with a user-visible error, no data corruption, service recovers automatically</t>
+        </is>
+      </c>
+      <c r="G26" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I26" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J26" s="34" t="inlineStr"/>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="69" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>Data Migration Dry-Run</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>Every schema change introduced by Sprints 0-3 applies cleanly to real-shaped data with no loss</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Run the migration plan (S5-05) against a full staging copy of realistic seeded data; diff before/after</t>
+        </is>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>All schema-changing tasks (S1-02, S2-01/02/08, S3-02) Done</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>Migration completes with zero data loss and a documented rollback path; re-run is idempotent</t>
+        </is>
+      </c>
+      <c r="G27" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I27" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J27" s="34" t="inlineStr"/>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="69" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B28" s="34" t="inlineStr">
+        <is>
+          <t>Backup &amp; Disaster-Recovery Drill</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>A real restore works within the defined RPO/RTO, not just a backup file existing</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>Actually delete/corrupt a staging DB copy and restore from the S5-04 backup process, timed</t>
+        </is>
+      </c>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>S5-04 backup runbook written</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>Restore completes within the target RTO with data loss within the target RPO</t>
+        </is>
+      </c>
+      <c r="G28" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I28" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J28" s="34" t="inlineStr"/>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="69" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B29" s="34" t="inlineStr">
+        <is>
+          <t>Tenant-Deletion Completeness Test</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>Deleting a tenant removes 100% of their data (DB + files), nothing orphaned</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Create a tenant with data in every collection incl. brain_context/brain_documents/files, delete it, verify zero remaining rows/files</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>S2-02 Done</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>Zero rows or files remain referencing the deleted tenant_id anywhere</t>
+        </is>
+      </c>
+      <c r="G29" s="34" t="inlineStr">
+        <is>
+          <t>Staging</t>
+        </is>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="I29" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J29" s="34" t="inlineStr"/>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="70" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B30" s="34" t="inlineStr">
+        <is>
+          <t>Internal Alpha Testing</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>The team itself can run real day-to-day operations on the product without a P0/P1 bug surfacing</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Internal team + demo data, every module used daily for the alpha window</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>Sprint 0 + Sprint 1 P0 all Done; automated suite green</t>
+        </is>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>Zero open P0/P1 bugs after the alpha window; baseline load test passed</t>
+        </is>
+      </c>
+      <c r="G30" s="34" t="inlineStr">
+        <is>
+          <t>Staging (alpha)</t>
+        </is>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>After Sprint 1</t>
+        </is>
+      </c>
+      <c r="I30" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J30" s="34" t="inlineStr"/>
+    </row>
+    <row r="31" ht="58" customHeight="1">
+      <c r="A31" s="71" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>Closed Beta — Design Partners</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>A small set of REAL external tenants (ideally incl. a non-textile business) run real operations and the product holds up without hand-holding beyond normal support</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>3-5 hand-picked design-partner tenants, high-touch support, 2-4 weeks, daily monitoring</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>Alpha exit criteria met; Sprint 2 + Sprint 3 Done; backup/restore drill passed</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>No P0 incidents; majority of design partners show daily active usage; tenant isolation matrix 100% pass with real data; at least 1 non-textile tenant validates the workflow fix</t>
+        </is>
+      </c>
+      <c r="G31" s="34" t="inlineStr">
+        <is>
+          <t>Production (limited)</t>
+        </is>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>After Sprint 3</t>
+        </is>
+      </c>
+      <c r="I31" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J31" s="34" t="inlineStr"/>
+    </row>
+    <row r="32" ht="58" customHeight="1">
+      <c r="A32" s="72" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B32" s="34" t="inlineStr">
+        <is>
+          <t>Staged Open Beta</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>Controlled expansion in tiers with a monitoring checkpoint before each step, so a problem is caught at 10 tenants, not 100</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Expand 10 -&gt; 30 -&gt; 50 tenants; hold at each tier for a monitoring window before advancing (ties to S5-09)</t>
+        </is>
+      </c>
+      <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>Closed Beta exit criteria met; Sprint 5 Done (load test, observability, migration dry-run)</t>
+        </is>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>Error rate + latency within SLO at every tier; no scheduler double-fire or cross-tenant incident observed; support volume stays manageable</t>
+        </is>
+      </c>
+      <c r="G32" s="34" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I32" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J32" s="34" t="inlineStr"/>
+    </row>
+    <row r="33" ht="58" customHeight="1">
+      <c r="A33" s="73" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>General Availability / Self-Serve Launch</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>The product is ready for unassisted signup at the full target scale</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Open self-serve signup; remove any beta gating</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t>Staged Beta exit criteria met; Go-Live Checklist 100% TRUE; final go/no-go held (S5-10)</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>Sustained SLA at ~100-tenant traffic with no open P0s for a full monitoring cycle</t>
+        </is>
+      </c>
+      <c r="G33" s="34" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>After Sprint 5</t>
+        </is>
+      </c>
+      <c r="I33" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J33" s="34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="57" t="inlineStr">
+        <is>
+          <t>Phase key:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B36" s="75" t="inlineStr">
+        <is>
+          <t>Automated (Unit/Integration/Regression)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="76" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B37" s="75" t="inlineStr">
+        <is>
+          <t>Multi-Tenant Isolation</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="77" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B38" s="75" t="inlineStr">
+        <is>
+          <t>Security / Pentest</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="78" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B39" s="75" t="inlineStr">
+        <is>
+          <t>Load &amp; Performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="79" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B40" s="75" t="inlineStr">
+        <is>
+          <t>Resilience / Concurrency / Chaos</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="80" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B41" s="75" t="inlineStr">
+        <is>
+          <t>Migration &amp; Backup/DR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="81" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B42" s="75" t="inlineStr">
+        <is>
+          <t>Internal Alpha</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="82" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B43" s="75" t="inlineStr">
+        <is>
+          <t>Closed Beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="83" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B44" s="75" t="inlineStr">
+        <is>
+          <t>Staged Open Beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="84" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B45" s="75" t="inlineStr">
+        <is>
+          <t>General Availability</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B38:D38"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I13:I33">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"Not Started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="7">
+      <formula>"Passed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="5">
+      <formula>"Failed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5">
+      <formula>"Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="I13:I33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not Started,In Progress,Passed,Failed,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5403,29 +6944,29 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="62" t="inlineStr">
+      <c r="A4" s="85" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="B4" s="62" t="inlineStr">
+      <c r="B4" s="85" t="inlineStr">
         <is>
           <t>Checklist item</t>
         </is>
       </c>
-      <c r="C4" s="62" t="inlineStr">
+      <c r="C4" s="85" t="inlineStr">
         <is>
           <t>Verified in</t>
         </is>
       </c>
-      <c r="D4" s="62" t="inlineStr">
+      <c r="D4" s="85" t="inlineStr">
         <is>
           <t>Done?</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="63" t="inlineStr">
+      <c r="A5" s="86" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
@@ -5435,19 +6976,19 @@
           <t>All Sprint 0 P0 items closed and verified (not just coded)</t>
         </is>
       </c>
-      <c r="C5" s="64" t="inlineStr">
+      <c r="C5" s="87" t="inlineStr">
         <is>
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="D5" s="65" t="inlineStr">
+      <c r="D5" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="63" t="inlineStr">
+      <c r="A6" s="86" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
@@ -5457,19 +6998,19 @@
           <t>Secrets rotated out of .env into a real secrets manager</t>
         </is>
       </c>
-      <c r="C6" s="66" t="inlineStr">
+      <c r="C6" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D6" s="65" t="inlineStr">
+      <c r="D6" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="86" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
@@ -5479,19 +7020,19 @@
           <t>Follow-up scheduler runs as a single external job, not in-process</t>
         </is>
       </c>
-      <c r="C7" s="67" t="inlineStr">
+      <c r="C7" s="90" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D7" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="63" t="inlineStr">
+      <c r="A8" s="86" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
@@ -5501,19 +7042,19 @@
           <t>All file uploads route through obj_store; local-disk path removed</t>
         </is>
       </c>
-      <c r="C8" s="67" t="inlineStr">
+      <c r="C8" s="90" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D8" s="65" t="inlineStr">
+      <c r="D8" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="86" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
@@ -5523,19 +7064,19 @@
           <t>Real Dockerfile/Procfile committed with pinned worker count</t>
         </is>
       </c>
-      <c r="C9" s="67" t="inlineStr">
+      <c r="C9" s="90" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D9" s="65" t="inlineStr">
+      <c r="D9" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="63" t="inlineStr">
+      <c r="A10" s="86" t="inlineStr">
         <is>
           <t>Scale</t>
         </is>
@@ -5545,19 +7086,19 @@
           <t>LLM calls have timeouts + a concurrency limit</t>
         </is>
       </c>
-      <c r="C10" s="67" t="inlineStr">
+      <c r="C10" s="90" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D10" s="65" t="inlineStr">
+      <c r="D10" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="63" t="inlineStr">
+      <c r="A11" s="86" t="inlineStr">
         <is>
           <t>Multi-tenant</t>
         </is>
@@ -5567,19 +7108,19 @@
           <t>Dynamic workflow approval loop works for a non-textile tenant</t>
         </is>
       </c>
-      <c r="C11" s="67" t="inlineStr">
+      <c r="C11" s="90" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D11" s="65" t="inlineStr">
+      <c r="D11" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="63" t="inlineStr">
+      <c r="A12" s="86" t="inlineStr">
         <is>
           <t>Multi-tenant</t>
         </is>
@@ -5589,19 +7130,19 @@
           <t>OTP login + WhatsApp routing are tenant-scoped</t>
         </is>
       </c>
-      <c r="C12" s="68" t="inlineStr">
+      <c r="C12" s="91" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="D12" s="65" t="inlineStr">
+      <c r="D12" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="63" t="inlineStr">
+      <c r="A13" s="86" t="inlineStr">
         <is>
           <t>Multi-tenant</t>
         </is>
@@ -5611,19 +7152,19 @@
           <t>Tenant deletion removes ALL tenant data incl. files</t>
         </is>
       </c>
-      <c r="C13" s="68" t="inlineStr">
+      <c r="C13" s="91" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="D13" s="65" t="inlineStr">
+      <c r="D13" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="63" t="inlineStr">
+      <c r="A14" s="86" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
@@ -5633,19 +7174,19 @@
           <t>Real payment provider integrated (Stripe/Razorpay)</t>
         </is>
       </c>
-      <c r="C14" s="69" t="inlineStr">
+      <c r="C14" s="92" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="D14" s="65" t="inlineStr">
+      <c r="D14" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="63" t="inlineStr">
+      <c r="A15" s="86" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
@@ -5655,19 +7196,19 @@
           <t>Per-tenant AI key isolation with usage quota enforcement</t>
         </is>
       </c>
-      <c r="C15" s="69" t="inlineStr">
+      <c r="C15" s="92" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="D15" s="65" t="inlineStr">
+      <c r="D15" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="63" t="inlineStr">
+      <c r="A16" s="86" t="inlineStr">
         <is>
           <t>Billing</t>
         </is>
@@ -5677,19 +7218,19 @@
           <t>Plan / entitlement fields exist on every tenant</t>
         </is>
       </c>
-      <c r="C16" s="69" t="inlineStr">
+      <c r="C16" s="92" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="D16" s="65" t="inlineStr">
+      <c r="D16" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="63" t="inlineStr">
+      <c r="A17" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5699,19 +7240,19 @@
           <t>Staging environment mirrors production</t>
         </is>
       </c>
-      <c r="C17" s="66" t="inlineStr">
+      <c r="C17" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D17" s="65" t="inlineStr">
+      <c r="D17" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="63" t="inlineStr">
+      <c r="A18" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5721,19 +7262,19 @@
           <t>Load test completed at ~100-tenant equivalent traffic</t>
         </is>
       </c>
-      <c r="C18" s="66" t="inlineStr">
+      <c r="C18" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D18" s="65" t="inlineStr">
+      <c r="D18" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="63" t="inlineStr">
+      <c r="A19" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5743,19 +7284,19 @@
           <t>Sentry / error tracking is live in production</t>
         </is>
       </c>
-      <c r="C19" s="66" t="inlineStr">
+      <c r="C19" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D19" s="65" t="inlineStr">
+      <c r="D19" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="63" t="inlineStr">
+      <c r="A20" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5765,19 +7306,19 @@
           <t>Backup restore has been TESTED, not just documented</t>
         </is>
       </c>
-      <c r="C20" s="66" t="inlineStr">
+      <c r="C20" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D20" s="65" t="inlineStr">
+      <c r="D20" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="63" t="inlineStr">
+      <c r="A21" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5787,19 +7328,19 @@
           <t>Data migration for all schema changes dry-run on staging</t>
         </is>
       </c>
-      <c r="C21" s="66" t="inlineStr">
+      <c r="C21" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D21" s="65" t="inlineStr">
+      <c r="D21" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="63" t="inlineStr">
+      <c r="A22" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5809,19 +7350,19 @@
           <t>Rollback procedure written and rehearsed</t>
         </is>
       </c>
-      <c r="C22" s="66" t="inlineStr">
+      <c r="C22" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D22" s="65" t="inlineStr">
+      <c r="D22" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="63" t="inlineStr">
+      <c r="A23" s="86" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
@@ -5831,57 +7372,79 @@
           <t>Staged rollout plan approved (5-&gt;20-&gt;50-&gt;100)</t>
         </is>
       </c>
-      <c r="C23" s="66" t="inlineStr">
+      <c r="C23" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D23" s="65" t="inlineStr">
+      <c r="D23" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="63" t="inlineStr">
+      <c r="A24" s="86" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Every Testing Plan phase (A-J) hit its exit criteria, incl. Closed + Staged Beta</t>
+        </is>
+      </c>
+      <c r="C24" s="93" t="inlineStr">
+        <is>
+          <t>Testing Plan</t>
+        </is>
+      </c>
+      <c r="D24" s="88" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="86" t="inlineStr">
         <is>
           <t>Sign-off</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>Final go/no-go review held with the full team</t>
         </is>
       </c>
-      <c r="C24" s="66" t="inlineStr">
+      <c r="C25" s="89" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D24" s="65" t="inlineStr">
+      <c r="D25" s="88" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>VERDICT</t>
         </is>
       </c>
-      <c r="B26" s="19">
-        <f>IF(COUNTIF(D5:D24,"TRUE")=COUNTA(D5:D24),"GO — cleared to sell as SaaS at scale","NOT YET — "&amp;(COUNTA(D5:D24)-COUNTIF(D5:D24,"TRUE"))&amp;" item(s) still open")</f>
+      <c r="B27" s="19">
+        <f>IF(COUNTIF(D5:D25,"TRUE")=COUNTA(D5:D25),"GO — cleared to sell as SaaS at scale","NOT YET — "&amp;(COUNTA(D5:D25)-COUNTIF(D5:D25,"TRUE"))&amp;" item(s) still open")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B26:D26"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:D24">
+  <conditionalFormatting sqref="D5:D25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"TRUE"</formula>
     </cfRule>
@@ -5889,16 +7452,16 @@
       <formula>"FALSE"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B26">
+  <conditionalFormatting sqref="B27">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>COUNTIF($D$5:$D$24,"TRUE")=COUNTA($D$5:$D$24)</formula>
+      <formula>COUNTIF($D$5:$D$25,"TRUE")=COUNTA($D$5:$D$25)</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="1">
-      <formula>COUNTIF($D$5:$D$24,"TRUE")&lt;COUNTA($D$5:$D$24)</formula>
+      <formula>COUNTIF($D$5:$D$25,"TRUE")&lt;COUNTA($D$5:$D$25)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D5:D25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: add Fix Log tab to the SaaS tracker
Running record of every code change: which finding it closes, files
touched, tests, current status, dates, PR/commit link, gotchas. Pre-seeded
with Fix #1 as two parts: (A) kill the purchase_payment textile hardcode
so any tenant's approval loop + dashboard work, and (B) wire workflow
advance -> auto-create Finance expense (surfaced when the founder asked
whether purchases go to Finance directly - today they don't, which is a
real product gap worth closing alongside 1A).
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -10,9 +10,10 @@
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Task Backlog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Kanban Board" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Testing Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Go-Live Checklist" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fix Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Kanban Board" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Testing Plan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Go-Live Checklist" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="45">
+  <fonts count="46">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -284,6 +285,12 @@
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="22">
     <fill>
@@ -419,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -640,11 +647,35 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -744,6 +775,19 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00D9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00351C75"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E4D7F5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5060,6 +5104,443 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t>Fix Log — every change we make, in order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>The running record of code changes: which finding it closes, what files it touches, which tests cover it, current status, and any gotchas. Grows as we ship fixes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Module in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>What it delivers</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Related Backlog / Test Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="94" t="inlineStr">
+        <is>
+          <t>Module 1</t>
+        </is>
+      </c>
+      <c r="B6" s="95" t="inlineStr">
+        <is>
+          <t>Multi-tenant / Dynamic Workflows</t>
+        </is>
+      </c>
+      <c r="C6" s="95" t="inlineStr">
+        <is>
+          <t>Make the product actually work for any small business (bakery, salon, boutique, clinic, workshop), not just the textile demo tenant. Unblocks Day-1 onboarding for non-textile pilots.</t>
+        </is>
+      </c>
+      <c r="D6" s="95" t="inlineStr">
+        <is>
+          <t>P0 — the product's core 'shaped around your workflow' promise doesn't deliver without this.</t>
+        </is>
+      </c>
+      <c r="E6" s="95" t="inlineStr">
+        <is>
+          <t>Sprint 1 (WF-1, WF-2, WF-3, WF-4 in Testing Plan) + Sprint 2 (S2-01, S2-02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Fix Log entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="62" t="inlineStr">
+        <is>
+          <t>Fix ID</t>
+        </is>
+      </c>
+      <c r="B9" s="62" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t>Backlog ID</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F9" s="62" t="inlineStr">
+        <is>
+          <t>Files touched</t>
+        </is>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Related tests</t>
+        </is>
+      </c>
+      <c r="H9" s="63" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I9" s="62" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="J9" s="63" t="inlineStr">
+        <is>
+          <t>Started</t>
+        </is>
+      </c>
+      <c r="K9" s="63" t="inlineStr">
+        <is>
+          <t>Finished</t>
+        </is>
+      </c>
+      <c r="L9" s="63" t="inlineStr">
+        <is>
+          <t>PR / Commit</t>
+        </is>
+      </c>
+      <c r="M9" s="63" t="inlineStr">
+        <is>
+          <t>Notes / gotchas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="105" customHeight="1">
+      <c r="A10" s="96" t="inlineStr">
+        <is>
+          <t>FIX-001-A</t>
+        </is>
+      </c>
+      <c r="B10" s="96" t="inlineStr">
+        <is>
+          <t>Multi-tenant / Dynamic Workflows</t>
+        </is>
+      </c>
+      <c r="C10" s="96" t="inlineStr">
+        <is>
+          <t>S1-06</t>
+        </is>
+      </c>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>Kill purchase_payment textile hardcode</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>Owner-approval loop + 'pending purchases' dashboard + payment-overdue alerts currently only fire when a workflow's type equals the literal string 'purchase_payment' (the textile demo pipeline key). For any AI-designed pipeline (e.g. 'procurement', 'ingredient_purchase', 'salon_restock'), these features silently break. Replace the hardcode with per-tenant pipeline lookup via the tenant's operating_model.</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>routers/decisions.py:166; server.py:2429; routers/brief.py:95,98,238,262</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>tests/test_workflows_dynamic.py (new) — non-textile approval loop, dashboard, brief</t>
+        </is>
+      </c>
+      <c r="H10" s="37" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="I10" s="42" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J10" s="96" t="inlineStr"/>
+      <c r="K10" s="96" t="inlineStr"/>
+      <c r="L10" s="96" t="inlineStr"/>
+      <c r="M10" s="22" t="inlineStr">
+        <is>
+          <t>Discovered as WF-1 in AI/Brain/Agentic review. Founder confirmed the target market is any small business (bakery, salon, boutique, clinic, workshop) not just textile manufacturers — so this is a Day-1 unblock for any non-textile pilot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" s="96" t="inlineStr">
+        <is>
+          <t>FIX-001-B</t>
+        </is>
+      </c>
+      <c r="B11" s="96" t="inlineStr">
+        <is>
+          <t>Multi-tenant / Dynamic Workflows</t>
+        </is>
+      </c>
+      <c r="C11" s="96" t="inlineStr">
+        <is>
+          <t>(newly discovered)</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>Wire workflow-advance to auto-create Finance expense on final stage</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="inlineStr">
+        <is>
+          <t>When a workflow card advances to its final 'paid' stage (or the dynamic equivalent), auto-create an Expense in db.expenses via create_expense() with the workflow's amount + counterparty, and store a workflow_id link on the expense so the two records are traceable. Currently the workflow-advance handler (server.py:2236) only updates the card's stage — Finance never learns about the purchase, so the founder has to record it twice.</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>server.py:2236 (advance_workflow); routers/ledger.py:222 (create_expense)</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>tests/test_workflow_finance_link.py (new) — advance to paid -&gt; expense created + linked</t>
+        </is>
+      </c>
+      <c r="H11" s="37" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="I11" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J11" s="96" t="inlineStr"/>
+      <c r="K11" s="96" t="inlineStr"/>
+      <c r="L11" s="96" t="inlineStr"/>
+      <c r="M11" s="22" t="inlineStr">
+        <is>
+          <t>Not in the original audit. Surfaced when the founder asked 'will it go to Finance directly?' Genuine product gap: today the workflow board and Finance are two parallel systems that don't communicate. Fix makes the loop honest so P&amp;L and CEO Brief reflect real spend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="57" t="inlineStr">
+        <is>
+          <t>Status legend:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="B15" s="97" t="inlineStr">
+        <is>
+          <t>In the backlog, no work yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="98" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="B16" s="97" t="inlineStr">
+        <is>
+          <t>Reading code, scoping the fix, drafting the approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="99" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="B17" s="97" t="inlineStr">
+        <is>
+          <t>Writing the fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>Code Review</t>
+        </is>
+      </c>
+      <c r="B18" s="97" t="inlineStr">
+        <is>
+          <t>Fix written, awaiting review / self-review</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="100" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B19" s="97" t="inlineStr">
+        <is>
+          <t>Tests running (unit + integration + manual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="101" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B20" s="97" t="inlineStr">
+        <is>
+          <t>Merged + tests green + verified on staging</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="36" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="97" t="inlineStr">
+        <is>
+          <t>Waiting on an external dependency or decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36" t="inlineStr">
+        <is>
+          <t>Rolled Back</t>
+        </is>
+      </c>
+      <c r="B22" s="97" t="inlineStr">
+        <is>
+          <t>Shipped, broke something, reverted (record it, don't hide it)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="B22:E22"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H10:H500">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"Not Started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+      <formula>"Planning"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4">
+      <formula>"In Progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
+      <formula>"Code Review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="8">
+      <formula>"Testing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="7">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="5">
+      <formula>"Blocked"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="5">
+      <formula>"Rolled Back"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="H10:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not Started,Planning,In Progress,Code Review,Testing,Done,Blocked,Rolled Back"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I10:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"P0,P1,P2"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5502,7 +5983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6914,7 +7395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(tracker): mark FIX-002-C Done, Sprint 1 = 3/6 shipped
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -1836,7 +1836,7 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="102" t="inlineStr">
+      <c r="A2" s="103" t="inlineStr">
         <is>
           <t>S0-01</t>
         </is>
@@ -1846,7 +1846,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C2" s="102" t="inlineStr">
+      <c r="C2" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -1866,17 +1866,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G2" s="102" t="inlineStr">
+      <c r="G2" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H2" s="102" t="inlineStr">
+      <c r="H2" s="103" t="inlineStr">
         <is>
           <t>server.py:4925-4937</t>
         </is>
       </c>
-      <c r="I2" s="102" t="inlineStr">
+      <c r="I2" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -1886,9 +1886,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K2" s="102" t="inlineStr"/>
-      <c r="L2" s="102" t="inlineStr"/>
-      <c r="M2" s="102" t="inlineStr"/>
+      <c r="K2" s="103" t="inlineStr"/>
+      <c r="L2" s="103" t="inlineStr"/>
+      <c r="M2" s="103" t="inlineStr"/>
       <c r="N2" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1897,7 +1897,7 @@
       <c r="O2" s="22" t="inlineStr"/>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="102" t="inlineStr">
+      <c r="A3" s="103" t="inlineStr">
         <is>
           <t>S0-02</t>
         </is>
@@ -1907,7 +1907,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C3" s="102" t="inlineStr">
+      <c r="C3" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -1927,17 +1927,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G3" s="102" t="inlineStr">
+      <c r="G3" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H3" s="102" t="inlineStr">
+      <c r="H3" s="103" t="inlineStr">
         <is>
           <t>server.py:4994-5001, core.py:218-222</t>
         </is>
       </c>
-      <c r="I3" s="102" t="inlineStr">
+      <c r="I3" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -1947,9 +1947,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K3" s="102" t="inlineStr"/>
-      <c r="L3" s="102" t="inlineStr"/>
-      <c r="M3" s="102" t="inlineStr"/>
+      <c r="K3" s="103" t="inlineStr"/>
+      <c r="L3" s="103" t="inlineStr"/>
+      <c r="M3" s="103" t="inlineStr"/>
       <c r="N3" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1958,7 +1958,7 @@
       <c r="O3" s="22" t="inlineStr"/>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="102" t="inlineStr">
+      <c r="A4" s="103" t="inlineStr">
         <is>
           <t>S0-03</t>
         </is>
@@ -1968,7 +1968,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C4" s="102" t="inlineStr">
+      <c r="C4" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -1988,17 +1988,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G4" s="102" t="inlineStr">
+      <c r="G4" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H4" s="102" t="inlineStr">
+      <c r="H4" s="103" t="inlineStr">
         <is>
           <t>server.py:3032-3038</t>
         </is>
       </c>
-      <c r="I4" s="102" t="inlineStr">
+      <c r="I4" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2008,9 +2008,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K4" s="102" t="inlineStr"/>
-      <c r="L4" s="102" t="inlineStr"/>
-      <c r="M4" s="102" t="inlineStr"/>
+      <c r="K4" s="103" t="inlineStr"/>
+      <c r="L4" s="103" t="inlineStr"/>
+      <c r="M4" s="103" t="inlineStr"/>
       <c r="N4" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2019,7 +2019,7 @@
       <c r="O4" s="22" t="inlineStr"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="102" t="inlineStr">
+      <c r="A5" s="103" t="inlineStr">
         <is>
           <t>S0-04</t>
         </is>
@@ -2029,7 +2029,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C5" s="102" t="inlineStr">
+      <c r="C5" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2049,17 +2049,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G5" s="102" t="inlineStr">
+      <c r="G5" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H5" s="102" t="inlineStr">
+      <c r="H5" s="103" t="inlineStr">
         <is>
           <t>server.py:1345-1347</t>
         </is>
       </c>
-      <c r="I5" s="102" t="inlineStr">
+      <c r="I5" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2069,9 +2069,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K5" s="102" t="inlineStr"/>
-      <c r="L5" s="102" t="inlineStr"/>
-      <c r="M5" s="102" t="inlineStr"/>
+      <c r="K5" s="103" t="inlineStr"/>
+      <c r="L5" s="103" t="inlineStr"/>
+      <c r="M5" s="103" t="inlineStr"/>
       <c r="N5" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2080,7 +2080,7 @@
       <c r="O5" s="22" t="inlineStr"/>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="102" t="inlineStr">
+      <c r="A6" s="103" t="inlineStr">
         <is>
           <t>S0-05</t>
         </is>
@@ -2090,7 +2090,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C6" s="102" t="inlineStr">
+      <c r="C6" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2110,17 +2110,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G6" s="102" t="inlineStr">
+      <c r="G6" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H6" s="102" t="inlineStr">
+      <c r="H6" s="103" t="inlineStr">
         <is>
           <t>server.py:3919-3933</t>
         </is>
       </c>
-      <c r="I6" s="102" t="inlineStr">
+      <c r="I6" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2130,9 +2130,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K6" s="102" t="inlineStr"/>
-      <c r="L6" s="102" t="inlineStr"/>
-      <c r="M6" s="102" t="inlineStr"/>
+      <c r="K6" s="103" t="inlineStr"/>
+      <c r="L6" s="103" t="inlineStr"/>
+      <c r="M6" s="103" t="inlineStr"/>
       <c r="N6" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2141,7 +2141,7 @@
       <c r="O6" s="22" t="inlineStr"/>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="102" t="inlineStr">
+      <c r="A7" s="103" t="inlineStr">
         <is>
           <t>S0-06</t>
         </is>
@@ -2151,7 +2151,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C7" s="102" t="inlineStr">
+      <c r="C7" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2171,17 +2171,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G7" s="102" t="inlineStr">
+      <c r="G7" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H7" s="102" t="inlineStr">
+      <c r="H7" s="103" t="inlineStr">
         <is>
           <t>routers/signup.py, routers/onboarding.py:39,73</t>
         </is>
       </c>
-      <c r="I7" s="102" t="inlineStr">
+      <c r="I7" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2191,9 +2191,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K7" s="102" t="inlineStr"/>
-      <c r="L7" s="102" t="inlineStr"/>
-      <c r="M7" s="102" t="inlineStr"/>
+      <c r="K7" s="103" t="inlineStr"/>
+      <c r="L7" s="103" t="inlineStr"/>
+      <c r="M7" s="103" t="inlineStr"/>
       <c r="N7" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2202,7 +2202,7 @@
       <c r="O7" s="22" t="inlineStr"/>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="102" t="inlineStr">
+      <c r="A8" s="103" t="inlineStr">
         <is>
           <t>S0-07</t>
         </is>
@@ -2212,7 +2212,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C8" s="102" t="inlineStr">
+      <c r="C8" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2232,17 +2232,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G8" s="102" t="inlineStr">
+      <c r="G8" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H8" s="102" t="inlineStr">
+      <c r="H8" s="103" t="inlineStr">
         <is>
           <t>routers/auth.py:151-162</t>
         </is>
       </c>
-      <c r="I8" s="102" t="inlineStr">
+      <c r="I8" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2252,9 +2252,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K8" s="102" t="inlineStr"/>
-      <c r="L8" s="102" t="inlineStr"/>
-      <c r="M8" s="102" t="inlineStr"/>
+      <c r="K8" s="103" t="inlineStr"/>
+      <c r="L8" s="103" t="inlineStr"/>
+      <c r="M8" s="103" t="inlineStr"/>
       <c r="N8" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2263,7 +2263,7 @@
       <c r="O8" s="22" t="inlineStr"/>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="102" t="inlineStr">
+      <c r="A9" s="103" t="inlineStr">
         <is>
           <t>S0-08</t>
         </is>
@@ -2273,7 +2273,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C9" s="102" t="inlineStr">
+      <c r="C9" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2293,17 +2293,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G9" s="102" t="inlineStr">
+      <c r="G9" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H9" s="102" t="inlineStr">
+      <c r="H9" s="103" t="inlineStr">
         <is>
           <t>routers/auth.py:148,162</t>
         </is>
       </c>
-      <c r="I9" s="102" t="inlineStr">
+      <c r="I9" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2313,9 +2313,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K9" s="102" t="inlineStr"/>
-      <c r="L9" s="102" t="inlineStr"/>
-      <c r="M9" s="102" t="inlineStr"/>
+      <c r="K9" s="103" t="inlineStr"/>
+      <c r="L9" s="103" t="inlineStr"/>
+      <c r="M9" s="103" t="inlineStr"/>
       <c r="N9" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2324,7 +2324,7 @@
       <c r="O9" s="22" t="inlineStr"/>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="102" t="inlineStr">
+      <c r="A10" s="103" t="inlineStr">
         <is>
           <t>S0-09</t>
         </is>
@@ -2334,7 +2334,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C10" s="102" t="inlineStr">
+      <c r="C10" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2354,17 +2354,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G10" s="102" t="inlineStr">
+      <c r="G10" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H10" s="102" t="inlineStr">
+      <c r="H10" s="103" t="inlineStr">
         <is>
           <t>core.py:237,297</t>
         </is>
       </c>
-      <c r="I10" s="102" t="inlineStr">
+      <c r="I10" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2374,9 +2374,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K10" s="102" t="inlineStr"/>
-      <c r="L10" s="102" t="inlineStr"/>
-      <c r="M10" s="102" t="inlineStr"/>
+      <c r="K10" s="103" t="inlineStr"/>
+      <c r="L10" s="103" t="inlineStr"/>
+      <c r="M10" s="103" t="inlineStr"/>
       <c r="N10" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2385,7 +2385,7 @@
       <c r="O10" s="22" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="102" t="inlineStr">
+      <c r="A11" s="103" t="inlineStr">
         <is>
           <t>S0-10</t>
         </is>
@@ -2395,7 +2395,7 @@
           <t>Sprint 0</t>
         </is>
       </c>
-      <c r="C11" s="102" t="inlineStr">
+      <c r="C11" s="103" t="inlineStr">
         <is>
           <t>Security/Auth</t>
         </is>
@@ -2415,17 +2415,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G11" s="102" t="inlineStr">
+      <c r="G11" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H11" s="102" t="inlineStr">
+      <c r="H11" s="103" t="inlineStr">
         <is>
           <t>server.py:1372,1386,1396,1397</t>
         </is>
       </c>
-      <c r="I11" s="102" t="inlineStr">
+      <c r="I11" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2435,9 +2435,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K11" s="102" t="inlineStr"/>
-      <c r="L11" s="102" t="inlineStr"/>
-      <c r="M11" s="102" t="inlineStr"/>
+      <c r="K11" s="103" t="inlineStr"/>
+      <c r="L11" s="103" t="inlineStr"/>
+      <c r="M11" s="103" t="inlineStr"/>
       <c r="N11" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2446,7 +2446,7 @@
       <c r="O11" s="22" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="102" t="inlineStr">
+      <c r="A12" s="103" t="inlineStr">
         <is>
           <t>S1-01</t>
         </is>
@@ -2456,7 +2456,7 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C12" s="102" t="inlineStr">
+      <c r="C12" s="103" t="inlineStr">
         <is>
           <t>Scale/Ops</t>
         </is>
@@ -2476,17 +2476,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G12" s="102" t="inlineStr">
+      <c r="G12" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H12" s="102" t="inlineStr">
+      <c r="H12" s="103" t="inlineStr">
         <is>
           <t>server.py:2765, 4946</t>
         </is>
       </c>
-      <c r="I12" s="102" t="inlineStr">
+      <c r="I12" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2496,9 +2496,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K12" s="102" t="inlineStr"/>
-      <c r="L12" s="102" t="inlineStr"/>
-      <c r="M12" s="102" t="inlineStr"/>
+      <c r="K12" s="103" t="inlineStr"/>
+      <c r="L12" s="103" t="inlineStr"/>
+      <c r="M12" s="103" t="inlineStr"/>
       <c r="N12" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2507,7 +2507,7 @@
       <c r="O12" s="22" t="inlineStr"/>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="102" t="inlineStr">
+      <c r="A13" s="103" t="inlineStr">
         <is>
           <t>S1-02</t>
         </is>
@@ -2517,7 +2517,7 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C13" s="102" t="inlineStr">
+      <c r="C13" s="103" t="inlineStr">
         <is>
           <t>Scale/Ops</t>
         </is>
@@ -2537,17 +2537,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G13" s="102" t="inlineStr">
+      <c r="G13" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H13" s="102" t="inlineStr">
+      <c r="H13" s="103" t="inlineStr">
         <is>
           <t>server.py:1357,1419,4004</t>
         </is>
       </c>
-      <c r="I13" s="102" t="inlineStr">
+      <c r="I13" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2557,9 +2557,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K13" s="102" t="inlineStr"/>
-      <c r="L13" s="102" t="inlineStr"/>
-      <c r="M13" s="102" t="inlineStr"/>
+      <c r="K13" s="103" t="inlineStr"/>
+      <c r="L13" s="103" t="inlineStr"/>
+      <c r="M13" s="103" t="inlineStr"/>
       <c r="N13" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2568,7 +2568,7 @@
       <c r="O13" s="22" t="inlineStr"/>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="102" t="inlineStr">
+      <c r="A14" s="103" t="inlineStr">
         <is>
           <t>S1-03</t>
         </is>
@@ -2578,7 +2578,7 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C14" s="102" t="inlineStr">
+      <c r="C14" s="103" t="inlineStr">
         <is>
           <t>Scale/Ops</t>
         </is>
@@ -2598,17 +2598,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G14" s="102" t="inlineStr">
+      <c r="G14" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H14" s="102" t="inlineStr">
+      <c r="H14" s="103" t="inlineStr">
         <is>
           <t>server.py:1739,1902,3032; ledger.py:146</t>
         </is>
       </c>
-      <c r="I14" s="102" t="inlineStr">
+      <c r="I14" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2618,9 +2618,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K14" s="102" t="inlineStr"/>
-      <c r="L14" s="102" t="inlineStr"/>
-      <c r="M14" s="102" t="inlineStr"/>
+      <c r="K14" s="103" t="inlineStr"/>
+      <c r="L14" s="103" t="inlineStr"/>
+      <c r="M14" s="103" t="inlineStr"/>
       <c r="N14" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2629,7 +2629,7 @@
       <c r="O14" s="22" t="inlineStr"/>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="102" t="inlineStr">
+      <c r="A15" s="103" t="inlineStr">
         <is>
           <t>S1-04</t>
         </is>
@@ -2639,7 +2639,7 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C15" s="102" t="inlineStr">
+      <c r="C15" s="103" t="inlineStr">
         <is>
           <t>Scale/Ops</t>
         </is>
@@ -2659,17 +2659,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G15" s="102" t="inlineStr">
+      <c r="G15" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H15" s="102" t="inlineStr">
+      <c r="H15" s="103" t="inlineStr">
         <is>
           <t>(missing — new file)</t>
         </is>
       </c>
-      <c r="I15" s="102" t="inlineStr">
+      <c r="I15" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2679,9 +2679,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K15" s="102" t="inlineStr"/>
-      <c r="L15" s="102" t="inlineStr"/>
-      <c r="M15" s="102" t="inlineStr"/>
+      <c r="K15" s="103" t="inlineStr"/>
+      <c r="L15" s="103" t="inlineStr"/>
+      <c r="M15" s="103" t="inlineStr"/>
       <c r="N15" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2690,7 +2690,7 @@
       <c r="O15" s="22" t="inlineStr"/>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="102" t="inlineStr">
+      <c r="A16" s="103" t="inlineStr">
         <is>
           <t>S1-05</t>
         </is>
@@ -2700,7 +2700,7 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C16" s="102" t="inlineStr">
+      <c r="C16" s="103" t="inlineStr">
         <is>
           <t>Scale/Ops</t>
         </is>
@@ -2720,17 +2720,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G16" s="102" t="inlineStr">
+      <c r="G16" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H16" s="102" t="inlineStr">
+      <c r="H16" s="103" t="inlineStr">
         <is>
           <t>core.py:177</t>
         </is>
       </c>
-      <c r="I16" s="102" t="inlineStr">
+      <c r="I16" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2740,9 +2740,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K16" s="102" t="inlineStr"/>
-      <c r="L16" s="102" t="inlineStr"/>
-      <c r="M16" s="102" t="inlineStr"/>
+      <c r="K16" s="103" t="inlineStr"/>
+      <c r="L16" s="103" t="inlineStr"/>
+      <c r="M16" s="103" t="inlineStr"/>
       <c r="N16" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2751,7 +2751,7 @@
       <c r="O16" s="22" t="inlineStr"/>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="102" t="inlineStr">
+      <c r="A17" s="103" t="inlineStr">
         <is>
           <t>S1-06</t>
         </is>
@@ -2761,7 +2761,7 @@
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C17" s="102" t="inlineStr">
+      <c r="C17" s="103" t="inlineStr">
         <is>
           <t>Scale/Ops</t>
         </is>
@@ -2781,17 +2781,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G17" s="102" t="inlineStr">
+      <c r="G17" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H17" s="102" t="inlineStr">
+      <c r="H17" s="103" t="inlineStr">
         <is>
           <t>routers/decisions.py:166; server.py:2429; routers/brief.py:95,98,238,262</t>
         </is>
       </c>
-      <c r="I17" s="102" t="inlineStr">
+      <c r="I17" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2801,9 +2801,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K17" s="102" t="inlineStr"/>
-      <c r="L17" s="102" t="inlineStr"/>
-      <c r="M17" s="102" t="inlineStr"/>
+      <c r="K17" s="103" t="inlineStr"/>
+      <c r="L17" s="103" t="inlineStr"/>
+      <c r="M17" s="103" t="inlineStr"/>
       <c r="N17" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2812,7 +2812,7 @@
       <c r="O17" s="22" t="inlineStr"/>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="102" t="inlineStr">
+      <c r="A18" s="103" t="inlineStr">
         <is>
           <t>S2-01</t>
         </is>
@@ -2822,7 +2822,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C18" s="102" t="inlineStr">
+      <c r="C18" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -2842,17 +2842,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G18" s="102" t="inlineStr">
+      <c r="G18" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H18" s="102" t="inlineStr">
+      <c r="H18" s="103" t="inlineStr">
         <is>
           <t>routers/tasks.py:317,360,395; decisions.py:144-227; brain_docs.py:320,329; ledger.py:585,638,684</t>
         </is>
       </c>
-      <c r="I18" s="102" t="inlineStr">
+      <c r="I18" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2862,9 +2862,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K18" s="102" t="inlineStr"/>
-      <c r="L18" s="102" t="inlineStr"/>
-      <c r="M18" s="102" t="inlineStr"/>
+      <c r="K18" s="103" t="inlineStr"/>
+      <c r="L18" s="103" t="inlineStr"/>
+      <c r="M18" s="103" t="inlineStr"/>
       <c r="N18" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -2873,7 +2873,7 @@
       <c r="O18" s="22" t="inlineStr"/>
     </row>
     <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="102" t="inlineStr">
+      <c r="A19" s="103" t="inlineStr">
         <is>
           <t>S2-02</t>
         </is>
@@ -2883,7 +2883,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C19" s="102" t="inlineStr">
+      <c r="C19" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -2903,17 +2903,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G19" s="102" t="inlineStr">
+      <c r="G19" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H19" s="102" t="inlineStr">
+      <c r="H19" s="103" t="inlineStr">
         <is>
           <t>routers/admin.py:161-186</t>
         </is>
       </c>
-      <c r="I19" s="102" t="inlineStr">
+      <c r="I19" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -2923,9 +2923,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K19" s="102" t="inlineStr"/>
-      <c r="L19" s="102" t="inlineStr"/>
-      <c r="M19" s="102" t="inlineStr"/>
+      <c r="K19" s="103" t="inlineStr"/>
+      <c r="L19" s="103" t="inlineStr"/>
+      <c r="M19" s="103" t="inlineStr"/>
       <c r="N19" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -2934,7 +2934,7 @@
       <c r="O19" s="22" t="inlineStr"/>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="102" t="inlineStr">
+      <c r="A20" s="103" t="inlineStr">
         <is>
           <t>S2-03</t>
         </is>
@@ -2944,7 +2944,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C20" s="102" t="inlineStr">
+      <c r="C20" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -2964,17 +2964,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G20" s="102" t="inlineStr">
+      <c r="G20" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H20" s="102" t="inlineStr">
+      <c r="H20" s="103" t="inlineStr">
         <is>
           <t>server.py:1418-1428,1357; 3999-4028</t>
         </is>
       </c>
-      <c r="I20" s="102" t="inlineStr">
+      <c r="I20" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -2984,9 +2984,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K20" s="102" t="inlineStr"/>
-      <c r="L20" s="102" t="inlineStr"/>
-      <c r="M20" s="102" t="inlineStr"/>
+      <c r="K20" s="103" t="inlineStr"/>
+      <c r="L20" s="103" t="inlineStr"/>
+      <c r="M20" s="103" t="inlineStr"/>
       <c r="N20" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2995,7 +2995,7 @@
       <c r="O20" s="22" t="inlineStr"/>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="102" t="inlineStr">
+      <c r="A21" s="103" t="inlineStr">
         <is>
           <t>S2-04</t>
         </is>
@@ -3005,7 +3005,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C21" s="102" t="inlineStr">
+      <c r="C21" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3025,17 +3025,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G21" s="102" t="inlineStr">
+      <c r="G21" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H21" s="102" t="inlineStr">
+      <c r="H21" s="103" t="inlineStr">
         <is>
           <t>server.py:3993-3995</t>
         </is>
       </c>
-      <c r="I21" s="102" t="inlineStr">
+      <c r="I21" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3045,9 +3045,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K21" s="102" t="inlineStr"/>
-      <c r="L21" s="102" t="inlineStr"/>
-      <c r="M21" s="102" t="inlineStr"/>
+      <c r="K21" s="103" t="inlineStr"/>
+      <c r="L21" s="103" t="inlineStr"/>
+      <c r="M21" s="103" t="inlineStr"/>
       <c r="N21" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3056,7 +3056,7 @@
       <c r="O21" s="22" t="inlineStr"/>
     </row>
     <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="102" t="inlineStr">
+      <c r="A22" s="103" t="inlineStr">
         <is>
           <t>S2-05</t>
         </is>
@@ -3066,7 +3066,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C22" s="102" t="inlineStr">
+      <c r="C22" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3086,17 +3086,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G22" s="102" t="inlineStr">
+      <c r="G22" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H22" s="102" t="inlineStr">
+      <c r="H22" s="103" t="inlineStr">
         <is>
           <t>server.py:2142-2158; routers/decisions.py:44,172-175</t>
         </is>
       </c>
-      <c r="I22" s="102" t="inlineStr">
+      <c r="I22" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3106,9 +3106,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K22" s="102" t="inlineStr"/>
-      <c r="L22" s="102" t="inlineStr"/>
-      <c r="M22" s="102" t="inlineStr"/>
+      <c r="K22" s="103" t="inlineStr"/>
+      <c r="L22" s="103" t="inlineStr"/>
+      <c r="M22" s="103" t="inlineStr"/>
       <c r="N22" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3117,7 +3117,7 @@
       <c r="O22" s="22" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="102" t="inlineStr">
+      <c r="A23" s="103" t="inlineStr">
         <is>
           <t>S2-06</t>
         </is>
@@ -3127,7 +3127,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C23" s="102" t="inlineStr">
+      <c r="C23" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3147,17 +3147,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G23" s="102" t="inlineStr">
+      <c r="G23" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H23" s="102" t="inlineStr">
+      <c r="H23" s="103" t="inlineStr">
         <is>
           <t>core.py:225-226</t>
         </is>
       </c>
-      <c r="I23" s="102" t="inlineStr">
+      <c r="I23" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3167,9 +3167,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K23" s="102" t="inlineStr"/>
-      <c r="L23" s="102" t="inlineStr"/>
-      <c r="M23" s="102" t="inlineStr"/>
+      <c r="K23" s="103" t="inlineStr"/>
+      <c r="L23" s="103" t="inlineStr"/>
+      <c r="M23" s="103" t="inlineStr"/>
       <c r="N23" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3178,7 +3178,7 @@
       <c r="O23" s="22" t="inlineStr"/>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="102" t="inlineStr">
+      <c r="A24" s="103" t="inlineStr">
         <is>
           <t>S2-07</t>
         </is>
@@ -3188,7 +3188,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C24" s="102" t="inlineStr">
+      <c r="C24" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3208,17 +3208,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G24" s="102" t="inlineStr">
+      <c r="G24" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H24" s="102" t="inlineStr">
+      <c r="H24" s="103" t="inlineStr">
         <is>
           <t>routers/auth.py</t>
         </is>
       </c>
-      <c r="I24" s="102" t="inlineStr">
+      <c r="I24" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3228,9 +3228,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K24" s="102" t="inlineStr"/>
-      <c r="L24" s="102" t="inlineStr"/>
-      <c r="M24" s="102" t="inlineStr"/>
+      <c r="K24" s="103" t="inlineStr"/>
+      <c r="L24" s="103" t="inlineStr"/>
+      <c r="M24" s="103" t="inlineStr"/>
       <c r="N24" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3239,7 +3239,7 @@
       <c r="O24" s="22" t="inlineStr"/>
     </row>
     <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="102" t="inlineStr">
+      <c r="A25" s="103" t="inlineStr">
         <is>
           <t>S2-08</t>
         </is>
@@ -3249,7 +3249,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C25" s="102" t="inlineStr">
+      <c r="C25" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3269,17 +3269,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G25" s="102" t="inlineStr">
+      <c r="G25" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H25" s="102" t="inlineStr">
+      <c r="H25" s="103" t="inlineStr">
         <is>
           <t>server.py:4865</t>
         </is>
       </c>
-      <c r="I25" s="102" t="inlineStr">
+      <c r="I25" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3289,9 +3289,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K25" s="102" t="inlineStr"/>
-      <c r="L25" s="102" t="inlineStr"/>
-      <c r="M25" s="102" t="inlineStr"/>
+      <c r="K25" s="103" t="inlineStr"/>
+      <c r="L25" s="103" t="inlineStr"/>
+      <c r="M25" s="103" t="inlineStr"/>
       <c r="N25" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3300,7 +3300,7 @@
       <c r="O25" s="22" t="inlineStr"/>
     </row>
     <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="102" t="inlineStr">
+      <c r="A26" s="103" t="inlineStr">
         <is>
           <t>S2-09</t>
         </is>
@@ -3310,7 +3310,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C26" s="102" t="inlineStr">
+      <c r="C26" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3330,17 +3330,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G26" s="102" t="inlineStr">
+      <c r="G26" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H26" s="102" t="inlineStr">
+      <c r="H26" s="103" t="inlineStr">
         <is>
           <t>routers/tasks.py; server.py:3326</t>
         </is>
       </c>
-      <c r="I26" s="102" t="inlineStr">
+      <c r="I26" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3350,9 +3350,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K26" s="102" t="inlineStr"/>
-      <c r="L26" s="102" t="inlineStr"/>
-      <c r="M26" s="102" t="inlineStr"/>
+      <c r="K26" s="103" t="inlineStr"/>
+      <c r="L26" s="103" t="inlineStr"/>
+      <c r="M26" s="103" t="inlineStr"/>
       <c r="N26" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3361,7 +3361,7 @@
       <c r="O26" s="22" t="inlineStr"/>
     </row>
     <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="102" t="inlineStr">
+      <c r="A27" s="103" t="inlineStr">
         <is>
           <t>S2-10</t>
         </is>
@@ -3371,7 +3371,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C27" s="102" t="inlineStr">
+      <c r="C27" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3391,17 +3391,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G27" s="102" t="inlineStr">
+      <c r="G27" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H27" s="102" t="inlineStr">
+      <c r="H27" s="103" t="inlineStr">
         <is>
           <t>routers/auth.py:92-93</t>
         </is>
       </c>
-      <c r="I27" s="102" t="inlineStr">
+      <c r="I27" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3411,9 +3411,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K27" s="102" t="inlineStr"/>
-      <c r="L27" s="102" t="inlineStr"/>
-      <c r="M27" s="102" t="inlineStr"/>
+      <c r="K27" s="103" t="inlineStr"/>
+      <c r="L27" s="103" t="inlineStr"/>
+      <c r="M27" s="103" t="inlineStr"/>
       <c r="N27" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3422,7 +3422,7 @@
       <c r="O27" s="22" t="inlineStr"/>
     </row>
     <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="102" t="inlineStr">
+      <c r="A28" s="103" t="inlineStr">
         <is>
           <t>S2-11</t>
         </is>
@@ -3432,7 +3432,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C28" s="102" t="inlineStr">
+      <c r="C28" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3452,17 +3452,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G28" s="102" t="inlineStr">
+      <c r="G28" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H28" s="102" t="inlineStr">
+      <c r="H28" s="103" t="inlineStr">
         <is>
           <t>server.py:1154-1160</t>
         </is>
       </c>
-      <c r="I28" s="102" t="inlineStr">
+      <c r="I28" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3472,9 +3472,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K28" s="102" t="inlineStr"/>
-      <c r="L28" s="102" t="inlineStr"/>
-      <c r="M28" s="102" t="inlineStr"/>
+      <c r="K28" s="103" t="inlineStr"/>
+      <c r="L28" s="103" t="inlineStr"/>
+      <c r="M28" s="103" t="inlineStr"/>
       <c r="N28" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3483,7 +3483,7 @@
       <c r="O28" s="22" t="inlineStr"/>
     </row>
     <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="102" t="inlineStr">
+      <c r="A29" s="103" t="inlineStr">
         <is>
           <t>S2-12</t>
         </is>
@@ -3493,7 +3493,7 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C29" s="102" t="inlineStr">
+      <c r="C29" s="103" t="inlineStr">
         <is>
           <t>Tenancy/Data</t>
         </is>
@@ -3513,17 +3513,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G29" s="102" t="inlineStr">
+      <c r="G29" s="103" t="inlineStr">
         <is>
           <t>Schema/Scale/Go-Live Review</t>
         </is>
       </c>
-      <c r="H29" s="102" t="inlineStr">
+      <c r="H29" s="103" t="inlineStr">
         <is>
           <t>server.py:2433</t>
         </is>
       </c>
-      <c r="I29" s="102" t="inlineStr">
+      <c r="I29" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3533,9 +3533,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K29" s="102" t="inlineStr"/>
-      <c r="L29" s="102" t="inlineStr"/>
-      <c r="M29" s="102" t="inlineStr"/>
+      <c r="K29" s="103" t="inlineStr"/>
+      <c r="L29" s="103" t="inlineStr"/>
+      <c r="M29" s="103" t="inlineStr"/>
       <c r="N29" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3544,7 +3544,7 @@
       <c r="O29" s="22" t="inlineStr"/>
     </row>
     <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="102" t="inlineStr">
+      <c r="A30" s="103" t="inlineStr">
         <is>
           <t>S3-01</t>
         </is>
@@ -3554,7 +3554,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C30" s="102" t="inlineStr">
+      <c r="C30" s="103" t="inlineStr">
         <is>
           <t>Billing/AI-Keys</t>
         </is>
@@ -3574,17 +3574,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G30" s="102" t="inlineStr">
+      <c r="G30" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H30" s="102" t="inlineStr">
+      <c r="H30" s="103" t="inlineStr">
         <is>
           <t>requirements.txt:129</t>
         </is>
       </c>
-      <c r="I30" s="102" t="inlineStr">
+      <c r="I30" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -3594,9 +3594,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K30" s="102" t="inlineStr"/>
-      <c r="L30" s="102" t="inlineStr"/>
-      <c r="M30" s="102" t="inlineStr"/>
+      <c r="K30" s="103" t="inlineStr"/>
+      <c r="L30" s="103" t="inlineStr"/>
+      <c r="M30" s="103" t="inlineStr"/>
       <c r="N30" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3605,7 +3605,7 @@
       <c r="O30" s="22" t="inlineStr"/>
     </row>
     <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="102" t="inlineStr">
+      <c r="A31" s="103" t="inlineStr">
         <is>
           <t>S3-02</t>
         </is>
@@ -3615,7 +3615,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C31" s="102" t="inlineStr">
+      <c r="C31" s="103" t="inlineStr">
         <is>
           <t>Billing/AI-Keys</t>
         </is>
@@ -3635,17 +3635,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G31" s="102" t="inlineStr">
+      <c r="G31" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H31" s="102" t="inlineStr">
+      <c r="H31" s="103" t="inlineStr">
         <is>
           <t>tenant document schema</t>
         </is>
       </c>
-      <c r="I31" s="102" t="inlineStr">
+      <c r="I31" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3655,9 +3655,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K31" s="102" t="inlineStr"/>
-      <c r="L31" s="102" t="inlineStr"/>
-      <c r="M31" s="102" t="inlineStr"/>
+      <c r="K31" s="103" t="inlineStr"/>
+      <c r="L31" s="103" t="inlineStr"/>
+      <c r="M31" s="103" t="inlineStr"/>
       <c r="N31" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3666,7 +3666,7 @@
       <c r="O31" s="22" t="inlineStr"/>
     </row>
     <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="102" t="inlineStr">
+      <c r="A32" s="103" t="inlineStr">
         <is>
           <t>S3-03</t>
         </is>
@@ -3676,7 +3676,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C32" s="102" t="inlineStr">
+      <c r="C32" s="103" t="inlineStr">
         <is>
           <t>Billing/AI-Keys</t>
         </is>
@@ -3696,17 +3696,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G32" s="102" t="inlineStr">
+      <c r="G32" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H32" s="102" t="inlineStr">
+      <c r="H32" s="103" t="inlineStr">
         <is>
           <t>config.py:53-60; core.py:177-205; routers/admin.py:335-348</t>
         </is>
       </c>
-      <c r="I32" s="102" t="inlineStr">
+      <c r="I32" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -3716,9 +3716,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K32" s="102" t="inlineStr"/>
-      <c r="L32" s="102" t="inlineStr"/>
-      <c r="M32" s="102" t="inlineStr"/>
+      <c r="K32" s="103" t="inlineStr"/>
+      <c r="L32" s="103" t="inlineStr"/>
+      <c r="M32" s="103" t="inlineStr"/>
       <c r="N32" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3727,7 +3727,7 @@
       <c r="O32" s="22" t="inlineStr"/>
     </row>
     <row r="33" ht="32" customHeight="1">
-      <c r="A33" s="102" t="inlineStr">
+      <c r="A33" s="103" t="inlineStr">
         <is>
           <t>S3-04</t>
         </is>
@@ -3737,7 +3737,7 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C33" s="102" t="inlineStr">
+      <c r="C33" s="103" t="inlineStr">
         <is>
           <t>Billing/AI-Keys</t>
         </is>
@@ -3757,17 +3757,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G33" s="102" t="inlineStr">
+      <c r="G33" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H33" s="102" t="inlineStr">
+      <c r="H33" s="103" t="inlineStr">
         <is>
           <t>services/usage.py</t>
         </is>
       </c>
-      <c r="I33" s="102" t="inlineStr">
+      <c r="I33" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3777,9 +3777,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K33" s="102" t="inlineStr"/>
-      <c r="L33" s="102" t="inlineStr"/>
-      <c r="M33" s="102" t="inlineStr"/>
+      <c r="K33" s="103" t="inlineStr"/>
+      <c r="L33" s="103" t="inlineStr"/>
+      <c r="M33" s="103" t="inlineStr"/>
       <c r="N33" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3788,7 +3788,7 @@
       <c r="O33" s="22" t="inlineStr"/>
     </row>
     <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="102" t="inlineStr">
+      <c r="A34" s="103" t="inlineStr">
         <is>
           <t>S4-01</t>
         </is>
@@ -3798,7 +3798,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C34" s="102" t="inlineStr">
+      <c r="C34" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -3818,17 +3818,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G34" s="102" t="inlineStr">
+      <c r="G34" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H34" s="102" t="inlineStr">
+      <c r="H34" s="103" t="inlineStr">
         <is>
           <t>server.py:4894; brain.py:250-255</t>
         </is>
       </c>
-      <c r="I34" s="102" t="inlineStr">
+      <c r="I34" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3838,9 +3838,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K34" s="102" t="inlineStr"/>
-      <c r="L34" s="102" t="inlineStr"/>
-      <c r="M34" s="102" t="inlineStr"/>
+      <c r="K34" s="103" t="inlineStr"/>
+      <c r="L34" s="103" t="inlineStr"/>
+      <c r="M34" s="103" t="inlineStr"/>
       <c r="N34" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3849,7 +3849,7 @@
       <c r="O34" s="22" t="inlineStr"/>
     </row>
     <row r="35" ht="32" customHeight="1">
-      <c r="A35" s="102" t="inlineStr">
+      <c r="A35" s="103" t="inlineStr">
         <is>
           <t>S4-02</t>
         </is>
@@ -3859,7 +3859,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C35" s="102" t="inlineStr">
+      <c r="C35" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -3879,17 +3879,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G35" s="102" t="inlineStr">
+      <c r="G35" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H35" s="102" t="inlineStr">
+      <c r="H35" s="103" t="inlineStr">
         <is>
           <t>tasks.py:507; services/brain_context.py</t>
         </is>
       </c>
-      <c r="I35" s="102" t="inlineStr">
+      <c r="I35" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -3899,9 +3899,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K35" s="102" t="inlineStr"/>
-      <c r="L35" s="102" t="inlineStr"/>
-      <c r="M35" s="102" t="inlineStr"/>
+      <c r="K35" s="103" t="inlineStr"/>
+      <c r="L35" s="103" t="inlineStr"/>
+      <c r="M35" s="103" t="inlineStr"/>
       <c r="N35" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3910,7 +3910,7 @@
       <c r="O35" s="22" t="inlineStr"/>
     </row>
     <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="102" t="inlineStr">
+      <c r="A36" s="103" t="inlineStr">
         <is>
           <t>S4-03</t>
         </is>
@@ -3920,7 +3920,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C36" s="102" t="inlineStr">
+      <c r="C36" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -3940,17 +3940,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G36" s="102" t="inlineStr">
+      <c r="G36" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H36" s="102" t="inlineStr">
+      <c r="H36" s="103" t="inlineStr">
         <is>
           <t>brain.py:714,752,794</t>
         </is>
       </c>
-      <c r="I36" s="102" t="inlineStr">
+      <c r="I36" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -3960,9 +3960,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K36" s="102" t="inlineStr"/>
-      <c r="L36" s="102" t="inlineStr"/>
-      <c r="M36" s="102" t="inlineStr"/>
+      <c r="K36" s="103" t="inlineStr"/>
+      <c r="L36" s="103" t="inlineStr"/>
+      <c r="M36" s="103" t="inlineStr"/>
       <c r="N36" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -3971,7 +3971,7 @@
       <c r="O36" s="22" t="inlineStr"/>
     </row>
     <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="102" t="inlineStr">
+      <c r="A37" s="103" t="inlineStr">
         <is>
           <t>S4-04</t>
         </is>
@@ -3981,7 +3981,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C37" s="102" t="inlineStr">
+      <c r="C37" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4001,17 +4001,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G37" s="102" t="inlineStr">
+      <c r="G37" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H37" s="102" t="inlineStr">
+      <c r="H37" s="103" t="inlineStr">
         <is>
           <t>routers/brain.py:52,205</t>
         </is>
       </c>
-      <c r="I37" s="102" t="inlineStr">
+      <c r="I37" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4021,9 +4021,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K37" s="102" t="inlineStr"/>
-      <c r="L37" s="102" t="inlineStr"/>
-      <c r="M37" s="102" t="inlineStr"/>
+      <c r="K37" s="103" t="inlineStr"/>
+      <c r="L37" s="103" t="inlineStr"/>
+      <c r="M37" s="103" t="inlineStr"/>
       <c r="N37" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4032,7 +4032,7 @@
       <c r="O37" s="22" t="inlineStr"/>
     </row>
     <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="102" t="inlineStr">
+      <c r="A38" s="103" t="inlineStr">
         <is>
           <t>S4-05</t>
         </is>
@@ -4042,7 +4042,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C38" s="102" t="inlineStr">
+      <c r="C38" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4062,17 +4062,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G38" s="102" t="inlineStr">
+      <c r="G38" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H38" s="102" t="inlineStr">
+      <c r="H38" s="103" t="inlineStr">
         <is>
           <t>routers/brain_docs.py:147-213</t>
         </is>
       </c>
-      <c r="I38" s="102" t="inlineStr">
+      <c r="I38" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -4082,9 +4082,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K38" s="102" t="inlineStr"/>
-      <c r="L38" s="102" t="inlineStr"/>
-      <c r="M38" s="102" t="inlineStr"/>
+      <c r="K38" s="103" t="inlineStr"/>
+      <c r="L38" s="103" t="inlineStr"/>
+      <c r="M38" s="103" t="inlineStr"/>
       <c r="N38" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4093,7 +4093,7 @@
       <c r="O38" s="22" t="inlineStr"/>
     </row>
     <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="102" t="inlineStr">
+      <c r="A39" s="103" t="inlineStr">
         <is>
           <t>S4-06</t>
         </is>
@@ -4103,7 +4103,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C39" s="102" t="inlineStr">
+      <c r="C39" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4123,17 +4123,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G39" s="102" t="inlineStr">
+      <c r="G39" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H39" s="102" t="inlineStr">
+      <c r="H39" s="103" t="inlineStr">
         <is>
           <t>(new infra)</t>
         </is>
       </c>
-      <c r="I39" s="102" t="inlineStr">
+      <c r="I39" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -4143,9 +4143,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K39" s="102" t="inlineStr"/>
-      <c r="L39" s="102" t="inlineStr"/>
-      <c r="M39" s="102" t="inlineStr"/>
+      <c r="K39" s="103" t="inlineStr"/>
+      <c r="L39" s="103" t="inlineStr"/>
+      <c r="M39" s="103" t="inlineStr"/>
       <c r="N39" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4154,7 +4154,7 @@
       <c r="O39" s="22" t="inlineStr"/>
     </row>
     <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="102" t="inlineStr">
+      <c r="A40" s="103" t="inlineStr">
         <is>
           <t>S4-07</t>
         </is>
@@ -4164,7 +4164,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C40" s="102" t="inlineStr">
+      <c r="C40" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4184,17 +4184,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G40" s="102" t="inlineStr">
+      <c r="G40" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H40" s="102" t="inlineStr">
+      <c r="H40" s="103" t="inlineStr">
         <is>
           <t>routers/brain.py; routers/brain_router.py</t>
         </is>
       </c>
-      <c r="I40" s="102" t="inlineStr">
+      <c r="I40" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4204,9 +4204,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K40" s="102" t="inlineStr"/>
-      <c r="L40" s="102" t="inlineStr"/>
-      <c r="M40" s="102" t="inlineStr"/>
+      <c r="K40" s="103" t="inlineStr"/>
+      <c r="L40" s="103" t="inlineStr"/>
+      <c r="M40" s="103" t="inlineStr"/>
       <c r="N40" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4215,7 +4215,7 @@
       <c r="O40" s="22" t="inlineStr"/>
     </row>
     <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="102" t="inlineStr">
+      <c r="A41" s="103" t="inlineStr">
         <is>
           <t>S4-08</t>
         </is>
@@ -4225,7 +4225,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C41" s="102" t="inlineStr">
+      <c r="C41" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4245,17 +4245,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G41" s="102" t="inlineStr">
+      <c r="G41" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H41" s="102" t="inlineStr">
+      <c r="H41" s="103" t="inlineStr">
         <is>
           <t>routers/brain_router.py:266-277,481-482</t>
         </is>
       </c>
-      <c r="I41" s="102" t="inlineStr">
+      <c r="I41" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -4265,9 +4265,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K41" s="102" t="inlineStr"/>
-      <c r="L41" s="102" t="inlineStr"/>
-      <c r="M41" s="102" t="inlineStr"/>
+      <c r="K41" s="103" t="inlineStr"/>
+      <c r="L41" s="103" t="inlineStr"/>
+      <c r="M41" s="103" t="inlineStr"/>
       <c r="N41" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4276,7 +4276,7 @@
       <c r="O41" s="22" t="inlineStr"/>
     </row>
     <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="102" t="inlineStr">
+      <c r="A42" s="103" t="inlineStr">
         <is>
           <t>S4-09</t>
         </is>
@@ -4286,7 +4286,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C42" s="102" t="inlineStr">
+      <c r="C42" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4306,17 +4306,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G42" s="102" t="inlineStr">
+      <c r="G42" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H42" s="102" t="inlineStr">
+      <c r="H42" s="103" t="inlineStr">
         <is>
           <t>routers/brain_router.py:95,353</t>
         </is>
       </c>
-      <c r="I42" s="102" t="inlineStr">
+      <c r="I42" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4326,9 +4326,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K42" s="102" t="inlineStr"/>
-      <c r="L42" s="102" t="inlineStr"/>
-      <c r="M42" s="102" t="inlineStr"/>
+      <c r="K42" s="103" t="inlineStr"/>
+      <c r="L42" s="103" t="inlineStr"/>
+      <c r="M42" s="103" t="inlineStr"/>
       <c r="N42" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4337,7 +4337,7 @@
       <c r="O42" s="22" t="inlineStr"/>
     </row>
     <row r="43" ht="32" customHeight="1">
-      <c r="A43" s="102" t="inlineStr">
+      <c r="A43" s="103" t="inlineStr">
         <is>
           <t>S4-10</t>
         </is>
@@ -4347,7 +4347,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C43" s="102" t="inlineStr">
+      <c r="C43" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4367,17 +4367,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G43" s="102" t="inlineStr">
+      <c r="G43" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H43" s="102" t="inlineStr">
+      <c r="H43" s="103" t="inlineStr">
         <is>
           <t>ledger.py:521-838; server.py (workflow advance, meetings)</t>
         </is>
       </c>
-      <c r="I43" s="102" t="inlineStr">
+      <c r="I43" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -4387,9 +4387,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K43" s="102" t="inlineStr"/>
-      <c r="L43" s="102" t="inlineStr"/>
-      <c r="M43" s="102" t="inlineStr"/>
+      <c r="K43" s="103" t="inlineStr"/>
+      <c r="L43" s="103" t="inlineStr"/>
+      <c r="M43" s="103" t="inlineStr"/>
       <c r="N43" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4398,7 +4398,7 @@
       <c r="O43" s="22" t="inlineStr"/>
     </row>
     <row r="44" ht="32" customHeight="1">
-      <c r="A44" s="102" t="inlineStr">
+      <c r="A44" s="103" t="inlineStr">
         <is>
           <t>S4-11</t>
         </is>
@@ -4408,7 +4408,7 @@
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C44" s="102" t="inlineStr">
+      <c r="C44" s="103" t="inlineStr">
         <is>
           <t>AI/Brain</t>
         </is>
@@ -4428,17 +4428,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="G44" s="102" t="inlineStr">
+      <c r="G44" s="103" t="inlineStr">
         <is>
           <t>AI/Brain/Agentic Review</t>
         </is>
       </c>
-      <c r="H44" s="102" t="inlineStr">
+      <c r="H44" s="103" t="inlineStr">
         <is>
           <t>services/brain_context.py:36-47</t>
         </is>
       </c>
-      <c r="I44" s="102" t="inlineStr">
+      <c r="I44" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4448,9 +4448,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K44" s="102" t="inlineStr"/>
-      <c r="L44" s="102" t="inlineStr"/>
-      <c r="M44" s="102" t="inlineStr"/>
+      <c r="K44" s="103" t="inlineStr"/>
+      <c r="L44" s="103" t="inlineStr"/>
+      <c r="M44" s="103" t="inlineStr"/>
       <c r="N44" s="41" t="inlineStr">
         <is>
           <t>No</t>
@@ -4459,7 +4459,7 @@
       <c r="O44" s="22" t="inlineStr"/>
     </row>
     <row r="45" ht="32" customHeight="1">
-      <c r="A45" s="102" t="inlineStr">
+      <c r="A45" s="103" t="inlineStr">
         <is>
           <t>S5-01</t>
         </is>
@@ -4469,7 +4469,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C45" s="102" t="inlineStr">
+      <c r="C45" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4489,17 +4489,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G45" s="102" t="inlineStr">
+      <c r="G45" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H45" s="102" t="inlineStr">
+      <c r="H45" s="103" t="inlineStr">
         <is>
           <t>(infra)</t>
         </is>
       </c>
-      <c r="I45" s="102" t="inlineStr">
+      <c r="I45" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4509,9 +4509,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K45" s="102" t="inlineStr"/>
-      <c r="L45" s="102" t="inlineStr"/>
-      <c r="M45" s="102" t="inlineStr"/>
+      <c r="K45" s="103" t="inlineStr"/>
+      <c r="L45" s="103" t="inlineStr"/>
+      <c r="M45" s="103" t="inlineStr"/>
       <c r="N45" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4520,7 +4520,7 @@
       <c r="O45" s="22" t="inlineStr"/>
     </row>
     <row r="46" ht="32" customHeight="1">
-      <c r="A46" s="102" t="inlineStr">
+      <c r="A46" s="103" t="inlineStr">
         <is>
           <t>S5-02</t>
         </is>
@@ -4530,7 +4530,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C46" s="102" t="inlineStr">
+      <c r="C46" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4550,17 +4550,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G46" s="102" t="inlineStr">
+      <c r="G46" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H46" s="102" t="inlineStr">
+      <c r="H46" s="103" t="inlineStr">
         <is>
           <t>(new)</t>
         </is>
       </c>
-      <c r="I46" s="102" t="inlineStr">
+      <c r="I46" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4570,9 +4570,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K46" s="102" t="inlineStr"/>
-      <c r="L46" s="102" t="inlineStr"/>
-      <c r="M46" s="102" t="inlineStr"/>
+      <c r="K46" s="103" t="inlineStr"/>
+      <c r="L46" s="103" t="inlineStr"/>
+      <c r="M46" s="103" t="inlineStr"/>
       <c r="N46" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4581,7 +4581,7 @@
       <c r="O46" s="22" t="inlineStr"/>
     </row>
     <row r="47" ht="32" customHeight="1">
-      <c r="A47" s="102" t="inlineStr">
+      <c r="A47" s="103" t="inlineStr">
         <is>
           <t>S5-03</t>
         </is>
@@ -4591,7 +4591,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C47" s="102" t="inlineStr">
+      <c r="C47" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4611,17 +4611,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G47" s="102" t="inlineStr">
+      <c r="G47" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H47" s="102" t="inlineStr">
+      <c r="H47" s="103" t="inlineStr">
         <is>
           <t>(missing)</t>
         </is>
       </c>
-      <c r="I47" s="102" t="inlineStr">
+      <c r="I47" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4631,9 +4631,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K47" s="102" t="inlineStr"/>
-      <c r="L47" s="102" t="inlineStr"/>
-      <c r="M47" s="102" t="inlineStr"/>
+      <c r="K47" s="103" t="inlineStr"/>
+      <c r="L47" s="103" t="inlineStr"/>
+      <c r="M47" s="103" t="inlineStr"/>
       <c r="N47" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4642,7 +4642,7 @@
       <c r="O47" s="22" t="inlineStr"/>
     </row>
     <row r="48" ht="32" customHeight="1">
-      <c r="A48" s="102" t="inlineStr">
+      <c r="A48" s="103" t="inlineStr">
         <is>
           <t>S5-04</t>
         </is>
@@ -4652,7 +4652,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C48" s="102" t="inlineStr">
+      <c r="C48" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4672,17 +4672,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G48" s="102" t="inlineStr">
+      <c r="G48" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H48" s="102" t="inlineStr">
+      <c r="H48" s="103" t="inlineStr">
         <is>
           <t>(missing)</t>
         </is>
       </c>
-      <c r="I48" s="102" t="inlineStr">
+      <c r="I48" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4692,9 +4692,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K48" s="102" t="inlineStr"/>
-      <c r="L48" s="102" t="inlineStr"/>
-      <c r="M48" s="102" t="inlineStr"/>
+      <c r="K48" s="103" t="inlineStr"/>
+      <c r="L48" s="103" t="inlineStr"/>
+      <c r="M48" s="103" t="inlineStr"/>
       <c r="N48" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4703,7 +4703,7 @@
       <c r="O48" s="22" t="inlineStr"/>
     </row>
     <row r="49" ht="32" customHeight="1">
-      <c r="A49" s="102" t="inlineStr">
+      <c r="A49" s="103" t="inlineStr">
         <is>
           <t>S5-05</t>
         </is>
@@ -4713,7 +4713,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C49" s="102" t="inlineStr">
+      <c r="C49" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4733,17 +4733,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G49" s="102" t="inlineStr">
+      <c r="G49" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H49" s="102" t="inlineStr">
+      <c r="H49" s="103" t="inlineStr">
         <is>
           <t>(new)</t>
         </is>
       </c>
-      <c r="I49" s="102" t="inlineStr">
+      <c r="I49" s="103" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -4753,9 +4753,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K49" s="102" t="inlineStr"/>
-      <c r="L49" s="102" t="inlineStr"/>
-      <c r="M49" s="102" t="inlineStr"/>
+      <c r="K49" s="103" t="inlineStr"/>
+      <c r="L49" s="103" t="inlineStr"/>
+      <c r="M49" s="103" t="inlineStr"/>
       <c r="N49" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4764,7 +4764,7 @@
       <c r="O49" s="22" t="inlineStr"/>
     </row>
     <row r="50" ht="32" customHeight="1">
-      <c r="A50" s="102" t="inlineStr">
+      <c r="A50" s="103" t="inlineStr">
         <is>
           <t>S5-06</t>
         </is>
@@ -4774,7 +4774,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C50" s="102" t="inlineStr">
+      <c r="C50" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4794,17 +4794,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G50" s="102" t="inlineStr">
+      <c r="G50" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H50" s="102" t="inlineStr">
+      <c r="H50" s="103" t="inlineStr">
         <is>
           <t>backend/pytest.ini, backend/tests/</t>
         </is>
       </c>
-      <c r="I50" s="102" t="inlineStr">
+      <c r="I50" s="103" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -4814,9 +4814,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K50" s="102" t="inlineStr"/>
-      <c r="L50" s="102" t="inlineStr"/>
-      <c r="M50" s="102" t="inlineStr"/>
+      <c r="K50" s="103" t="inlineStr"/>
+      <c r="L50" s="103" t="inlineStr"/>
+      <c r="M50" s="103" t="inlineStr"/>
       <c r="N50" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4825,7 +4825,7 @@
       <c r="O50" s="22" t="inlineStr"/>
     </row>
     <row r="51" ht="32" customHeight="1">
-      <c r="A51" s="102" t="inlineStr">
+      <c r="A51" s="103" t="inlineStr">
         <is>
           <t>S5-07</t>
         </is>
@@ -4835,7 +4835,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C51" s="102" t="inlineStr">
+      <c r="C51" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4855,17 +4855,17 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="G51" s="102" t="inlineStr">
+      <c r="G51" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H51" s="102" t="inlineStr">
+      <c r="H51" s="103" t="inlineStr">
         <is>
           <t>(new)</t>
         </is>
       </c>
-      <c r="I51" s="102" t="inlineStr">
+      <c r="I51" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -4875,9 +4875,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K51" s="102" t="inlineStr"/>
-      <c r="L51" s="102" t="inlineStr"/>
-      <c r="M51" s="102" t="inlineStr"/>
+      <c r="K51" s="103" t="inlineStr"/>
+      <c r="L51" s="103" t="inlineStr"/>
+      <c r="M51" s="103" t="inlineStr"/>
       <c r="N51" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4886,7 +4886,7 @@
       <c r="O51" s="22" t="inlineStr"/>
     </row>
     <row r="52" ht="32" customHeight="1">
-      <c r="A52" s="102" t="inlineStr">
+      <c r="A52" s="103" t="inlineStr">
         <is>
           <t>S5-08</t>
         </is>
@@ -4896,7 +4896,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C52" s="102" t="inlineStr">
+      <c r="C52" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4916,17 +4916,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G52" s="102" t="inlineStr">
+      <c r="G52" s="103" t="inlineStr">
         <is>
           <t>SaaS Readiness Review</t>
         </is>
       </c>
-      <c r="H52" s="102" t="inlineStr">
+      <c r="H52" s="103" t="inlineStr">
         <is>
           <t>backend/.env, config.py</t>
         </is>
       </c>
-      <c r="I52" s="102" t="inlineStr">
+      <c r="I52" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -4936,9 +4936,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K52" s="102" t="inlineStr"/>
-      <c r="L52" s="102" t="inlineStr"/>
-      <c r="M52" s="102" t="inlineStr"/>
+      <c r="K52" s="103" t="inlineStr"/>
+      <c r="L52" s="103" t="inlineStr"/>
+      <c r="M52" s="103" t="inlineStr"/>
       <c r="N52" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4947,7 +4947,7 @@
       <c r="O52" s="22" t="inlineStr"/>
     </row>
     <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="102" t="inlineStr">
+      <c r="A53" s="103" t="inlineStr">
         <is>
           <t>S5-09</t>
         </is>
@@ -4957,7 +4957,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C53" s="102" t="inlineStr">
+      <c r="C53" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -4977,17 +4977,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G53" s="102" t="inlineStr">
+      <c r="G53" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H53" s="102" t="inlineStr">
+      <c r="H53" s="103" t="inlineStr">
         <is>
           <t>(process)</t>
         </is>
       </c>
-      <c r="I53" s="102" t="inlineStr">
+      <c r="I53" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -4997,9 +4997,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K53" s="102" t="inlineStr"/>
-      <c r="L53" s="102" t="inlineStr"/>
-      <c r="M53" s="102" t="inlineStr"/>
+      <c r="K53" s="103" t="inlineStr"/>
+      <c r="L53" s="103" t="inlineStr"/>
+      <c r="M53" s="103" t="inlineStr"/>
       <c r="N53" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5008,7 +5008,7 @@
       <c r="O53" s="22" t="inlineStr"/>
     </row>
     <row r="54" ht="32" customHeight="1">
-      <c r="A54" s="102" t="inlineStr">
+      <c r="A54" s="103" t="inlineStr">
         <is>
           <t>S5-10</t>
         </is>
@@ -5018,7 +5018,7 @@
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="C54" s="102" t="inlineStr">
+      <c r="C54" s="103" t="inlineStr">
         <is>
           <t>DevOps/Migration</t>
         </is>
@@ -5038,17 +5038,17 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="G54" s="102" t="inlineStr">
+      <c r="G54" s="103" t="inlineStr">
         <is>
           <t>Go-Live Gate</t>
         </is>
       </c>
-      <c r="H54" s="102" t="inlineStr">
+      <c r="H54" s="103" t="inlineStr">
         <is>
           <t>(process)</t>
         </is>
       </c>
-      <c r="I54" s="102" t="inlineStr">
+      <c r="I54" s="103" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -5058,9 +5058,9 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="K54" s="102" t="inlineStr"/>
-      <c r="L54" s="102" t="inlineStr"/>
-      <c r="M54" s="102" t="inlineStr"/>
+      <c r="K54" s="103" t="inlineStr"/>
+      <c r="L54" s="103" t="inlineStr"/>
+      <c r="M54" s="103" t="inlineStr"/>
       <c r="N54" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -5138,7 +5138,7 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Running record. Updated side-by-side after every shipped commit. Currently: 8 Done, 16 in backlog.</t>
+          <t>Running record. Updated side-by-side after every shipped commit. Currently: 9 Done, 15 in backlog.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="E7" s="95" t="inlineStr">
         <is>
-          <t>2/5 shipped, 3 remaining + FIX-002-C added.</t>
+          <t>3/6 shipped (FIX-002-C added migration ledger).</t>
         </is>
       </c>
     </row>
@@ -5876,9 +5876,9 @@
           <t>tests/test_migrations.py — helper contract + idempotency</t>
         </is>
       </c>
-      <c r="H19" s="37" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H19" s="101" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I19" s="38" t="inlineStr">
@@ -5886,9 +5886,21 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J19" s="103" t="inlineStr"/>
-      <c r="K19" s="103" t="inlineStr"/>
-      <c r="L19" s="103" t="inlineStr"/>
+      <c r="J19" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="K19" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="L19" s="103" t="inlineStr">
+        <is>
+          <t>(this commit)</t>
+        </is>
+      </c>
       <c r="M19" s="22" t="inlineStr">
         <is>
           <t>Prerequisite for S1-03 (uploads migration). MongoDB doesn't need Alembic (no DDL) but does need this ledger discipline.</t>
@@ -6720,6 +6732,8 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="57" t="inlineStr">
         <is>
@@ -7564,7 +7578,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B13" s="102" t="inlineStr">
+      <c r="B13" s="103" t="inlineStr">
         <is>
           <t>Unit Testing</t>
         </is>
@@ -7589,12 +7603,12 @@
           <t>100% of new/changed code has a passing unit test; suite green in CI</t>
         </is>
       </c>
-      <c r="G13" s="102" t="inlineStr">
+      <c r="G13" s="103" t="inlineStr">
         <is>
           <t>Dev / CI</t>
         </is>
       </c>
-      <c r="H13" s="102" t="inlineStr">
+      <c r="H13" s="103" t="inlineStr">
         <is>
           <t>Sprint 0-5 (continuous)</t>
         </is>
@@ -7604,7 +7618,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J13" s="102" t="inlineStr"/>
+      <c r="J13" s="103" t="inlineStr"/>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="64" t="inlineStr">
@@ -7612,7 +7626,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B14" s="102" t="inlineStr">
+      <c r="B14" s="103" t="inlineStr">
         <is>
           <t>Integration Testing</t>
         </is>
@@ -7637,12 +7651,12 @@
           <t>Every endpoint touched by Sprints 0-3 has at least one integration test; suite green</t>
         </is>
       </c>
-      <c r="G14" s="102" t="inlineStr">
+      <c r="G14" s="103" t="inlineStr">
         <is>
           <t>Dev / CI</t>
         </is>
       </c>
-      <c r="H14" s="102" t="inlineStr">
+      <c r="H14" s="103" t="inlineStr">
         <is>
           <t>Sprint 0-3</t>
         </is>
@@ -7652,7 +7666,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J14" s="102" t="inlineStr"/>
+      <c r="J14" s="103" t="inlineStr"/>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="64" t="inlineStr">
@@ -7660,7 +7674,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B15" s="102" t="inlineStr">
+      <c r="B15" s="103" t="inlineStr">
         <is>
           <t>Regression Testing</t>
         </is>
@@ -7685,12 +7699,12 @@
           <t>Zero net-new failures vs. the pre-sprint baseline run</t>
         </is>
       </c>
-      <c r="G15" s="102" t="inlineStr">
+      <c r="G15" s="103" t="inlineStr">
         <is>
           <t>CI</t>
         </is>
       </c>
-      <c r="H15" s="102" t="inlineStr">
+      <c r="H15" s="103" t="inlineStr">
         <is>
           <t>Every sprint</t>
         </is>
@@ -7700,7 +7714,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J15" s="102" t="inlineStr"/>
+      <c r="J15" s="103" t="inlineStr"/>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="65" t="inlineStr">
@@ -7708,7 +7722,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B16" s="102" t="inlineStr">
+      <c r="B16" s="103" t="inlineStr">
         <is>
           <t>Multi-Tenant Isolation Test Matrix</t>
         </is>
@@ -7733,12 +7747,12 @@
           <t>100% pass — zero cross-tenant access possible, incl. OTP/WhatsApp phone routing and tenant deletion completeness</t>
         </is>
       </c>
-      <c r="G16" s="102" t="inlineStr">
+      <c r="G16" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H16" s="102" t="inlineStr">
+      <c r="H16" s="103" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
@@ -7748,7 +7762,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J16" s="102" t="inlineStr"/>
+      <c r="J16" s="103" t="inlineStr"/>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="65" t="inlineStr">
@@ -7756,7 +7770,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B17" s="102" t="inlineStr">
+      <c r="B17" s="103" t="inlineStr">
         <is>
           <t>Dynamic-Workflow Multi-Tenant Test</t>
         </is>
@@ -7781,12 +7795,12 @@
           <t>Approval gate, pending-purchases dashboard, and payment-overdue alerts all fire correctly for the non-textile pipeline</t>
         </is>
       </c>
-      <c r="G17" s="102" t="inlineStr">
+      <c r="G17" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H17" s="102" t="inlineStr">
+      <c r="H17" s="103" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
@@ -7796,7 +7810,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J17" s="102" t="inlineStr"/>
+      <c r="J17" s="103" t="inlineStr"/>
     </row>
     <row r="18" ht="58" customHeight="1">
       <c r="A18" s="66" t="inlineStr">
@@ -7804,7 +7818,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B18" s="102" t="inlineStr">
+      <c r="B18" s="103" t="inlineStr">
         <is>
           <t>Security / Penetration Testing</t>
         </is>
@@ -7829,12 +7843,12 @@
           <t>Zero exploitable findings on the Sprint 0 issue list; independent reviewer (or external pentest) sign-off</t>
         </is>
       </c>
-      <c r="G18" s="102" t="inlineStr">
+      <c r="G18" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H18" s="102" t="inlineStr">
+      <c r="H18" s="103" t="inlineStr">
         <is>
           <t>Sprint 0</t>
         </is>
@@ -7844,7 +7858,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J18" s="102" t="inlineStr"/>
+      <c r="J18" s="103" t="inlineStr"/>
     </row>
     <row r="19" ht="58" customHeight="1">
       <c r="A19" s="66" t="inlineStr">
@@ -7852,7 +7866,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B19" s="102" t="inlineStr">
+      <c r="B19" s="103" t="inlineStr">
         <is>
           <t>RBAC / Permission Audit</t>
         </is>
@@ -7877,12 +7891,12 @@
           <t>100% pass on the role x endpoint matrix</t>
         </is>
       </c>
-      <c r="G19" s="102" t="inlineStr">
+      <c r="G19" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H19" s="102" t="inlineStr">
+      <c r="H19" s="103" t="inlineStr">
         <is>
           <t>Sprint 0-2</t>
         </is>
@@ -7892,7 +7906,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J19" s="102" t="inlineStr"/>
+      <c r="J19" s="103" t="inlineStr"/>
     </row>
     <row r="20" ht="58" customHeight="1">
       <c r="A20" s="67" t="inlineStr">
@@ -7900,7 +7914,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B20" s="102" t="inlineStr">
+      <c r="B20" s="103" t="inlineStr">
         <is>
           <t>Load / Performance Testing — Baseline</t>
         </is>
@@ -7925,12 +7939,12 @@
           <t>P95 latency within target (e.g. &lt;500ms for reads, &lt;3s for AI-backed endpoints) at expected steady load</t>
         </is>
       </c>
-      <c r="G20" s="102" t="inlineStr">
+      <c r="G20" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H20" s="102" t="inlineStr">
+      <c r="H20" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -7940,7 +7954,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J20" s="102" t="inlineStr"/>
+      <c r="J20" s="103" t="inlineStr"/>
     </row>
     <row r="21" ht="58" customHeight="1">
       <c r="A21" s="67" t="inlineStr">
@@ -7948,7 +7962,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B21" s="102" t="inlineStr">
+      <c r="B21" s="103" t="inlineStr">
         <is>
           <t>Load Testing — Multi-Tenant Concurrency</t>
         </is>
@@ -7973,12 +7987,12 @@
           <t>No error-rate spike, no shared-LLM-key 429 cascade (validates S1-05), DB pool holds under SUMMED load</t>
         </is>
       </c>
-      <c r="G21" s="102" t="inlineStr">
+      <c r="G21" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H21" s="102" t="inlineStr">
+      <c r="H21" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -7988,7 +8002,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J21" s="102" t="inlineStr"/>
+      <c r="J21" s="103" t="inlineStr"/>
     </row>
     <row r="22" ht="58" customHeight="1">
       <c r="A22" s="67" t="inlineStr">
@@ -7996,7 +8010,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B22" s="102" t="inlineStr">
+      <c r="B22" s="103" t="inlineStr">
         <is>
           <t>Spike / Burst Testing</t>
         </is>
@@ -8021,12 +8035,12 @@
           <t>System recovers within target time with no dropped requests beyond configured rate limits</t>
         </is>
       </c>
-      <c r="G22" s="102" t="inlineStr">
+      <c r="G22" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H22" s="102" t="inlineStr">
+      <c r="H22" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -8036,7 +8050,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J22" s="102" t="inlineStr"/>
+      <c r="J22" s="103" t="inlineStr"/>
     </row>
     <row r="23" ht="58" customHeight="1">
       <c r="A23" s="67" t="inlineStr">
@@ -8044,7 +8058,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B23" s="102" t="inlineStr">
+      <c r="B23" s="103" t="inlineStr">
         <is>
           <t>Soak / Endurance Testing</t>
         </is>
@@ -8069,12 +8083,12 @@
           <t>No degradation in latency/error-rate/memory over the full run</t>
         </is>
       </c>
-      <c r="G23" s="102" t="inlineStr">
+      <c r="G23" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H23" s="102" t="inlineStr">
+      <c r="H23" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -8084,7 +8098,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J23" s="102" t="inlineStr"/>
+      <c r="J23" s="103" t="inlineStr"/>
     </row>
     <row r="24" ht="58" customHeight="1">
       <c r="A24" s="67" t="inlineStr">
@@ -8092,7 +8106,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B24" s="102" t="inlineStr">
+      <c r="B24" s="103" t="inlineStr">
         <is>
           <t>Database Query Performance at Volume</t>
         </is>
@@ -8117,12 +8131,12 @@
           <t>No full-collection scans on hot paths; dashboard/brief load within SLO at seeded volume</t>
         </is>
       </c>
-      <c r="G24" s="102" t="inlineStr">
+      <c r="G24" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H24" s="102" t="inlineStr">
+      <c r="H24" s="103" t="inlineStr">
         <is>
           <t>Sprint 1-2</t>
         </is>
@@ -8132,7 +8146,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J24" s="102" t="inlineStr"/>
+      <c r="J24" s="103" t="inlineStr"/>
     </row>
     <row r="25" ht="58" customHeight="1">
       <c r="A25" s="68" t="inlineStr">
@@ -8140,7 +8154,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B25" s="102" t="inlineStr">
+      <c r="B25" s="103" t="inlineStr">
         <is>
           <t>Multi-Replica / Concurrency Testing</t>
         </is>
@@ -8165,12 +8179,12 @@
           <t>Zero duplicate escalation emails/alerts observed across a full scheduler interval with 3 replicas running</t>
         </is>
       </c>
-      <c r="G25" s="102" t="inlineStr">
+      <c r="G25" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H25" s="102" t="inlineStr">
+      <c r="H25" s="103" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
@@ -8180,7 +8194,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J25" s="102" t="inlineStr"/>
+      <c r="J25" s="103" t="inlineStr"/>
     </row>
     <row r="26" ht="58" customHeight="1">
       <c r="A26" s="68" t="inlineStr">
@@ -8188,7 +8202,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B26" s="102" t="inlineStr">
+      <c r="B26" s="103" t="inlineStr">
         <is>
           <t>Failure-Injection / Chaos Testing</t>
         </is>
@@ -8213,12 +8227,12 @@
           <t>In-flight requests fail cleanly with a user-visible error, no data corruption, service recovers automatically</t>
         </is>
       </c>
-      <c r="G26" s="102" t="inlineStr">
+      <c r="G26" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H26" s="102" t="inlineStr">
+      <c r="H26" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -8228,7 +8242,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J26" s="102" t="inlineStr"/>
+      <c r="J26" s="103" t="inlineStr"/>
     </row>
     <row r="27" ht="58" customHeight="1">
       <c r="A27" s="69" t="inlineStr">
@@ -8236,7 +8250,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B27" s="102" t="inlineStr">
+      <c r="B27" s="103" t="inlineStr">
         <is>
           <t>Data Migration Dry-Run</t>
         </is>
@@ -8261,12 +8275,12 @@
           <t>Migration completes with zero data loss and a documented rollback path; re-run is idempotent</t>
         </is>
       </c>
-      <c r="G27" s="102" t="inlineStr">
+      <c r="G27" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H27" s="102" t="inlineStr">
+      <c r="H27" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -8276,7 +8290,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J27" s="102" t="inlineStr"/>
+      <c r="J27" s="103" t="inlineStr"/>
     </row>
     <row r="28" ht="58" customHeight="1">
       <c r="A28" s="69" t="inlineStr">
@@ -8284,7 +8298,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B28" s="102" t="inlineStr">
+      <c r="B28" s="103" t="inlineStr">
         <is>
           <t>Backup &amp; Disaster-Recovery Drill</t>
         </is>
@@ -8309,12 +8323,12 @@
           <t>Restore completes within the target RTO with data loss within the target RPO</t>
         </is>
       </c>
-      <c r="G28" s="102" t="inlineStr">
+      <c r="G28" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H28" s="102" t="inlineStr">
+      <c r="H28" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -8324,7 +8338,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J28" s="102" t="inlineStr"/>
+      <c r="J28" s="103" t="inlineStr"/>
     </row>
     <row r="29" ht="58" customHeight="1">
       <c r="A29" s="69" t="inlineStr">
@@ -8332,7 +8346,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B29" s="102" t="inlineStr">
+      <c r="B29" s="103" t="inlineStr">
         <is>
           <t>Tenant-Deletion Completeness Test</t>
         </is>
@@ -8357,12 +8371,12 @@
           <t>Zero rows or files remain referencing the deleted tenant_id anywhere</t>
         </is>
       </c>
-      <c r="G29" s="102" t="inlineStr">
+      <c r="G29" s="103" t="inlineStr">
         <is>
           <t>Staging</t>
         </is>
       </c>
-      <c r="H29" s="102" t="inlineStr">
+      <c r="H29" s="103" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
@@ -8372,7 +8386,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J29" s="102" t="inlineStr"/>
+      <c r="J29" s="103" t="inlineStr"/>
     </row>
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="70" t="inlineStr">
@@ -8380,7 +8394,7 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B30" s="102" t="inlineStr">
+      <c r="B30" s="103" t="inlineStr">
         <is>
           <t>Internal Alpha Testing</t>
         </is>
@@ -8405,12 +8419,12 @@
           <t>Zero open P0/P1 bugs after the alpha window; baseline load test passed</t>
         </is>
       </c>
-      <c r="G30" s="102" t="inlineStr">
+      <c r="G30" s="103" t="inlineStr">
         <is>
           <t>Staging (alpha)</t>
         </is>
       </c>
-      <c r="H30" s="102" t="inlineStr">
+      <c r="H30" s="103" t="inlineStr">
         <is>
           <t>After Sprint 1</t>
         </is>
@@ -8420,7 +8434,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J30" s="102" t="inlineStr"/>
+      <c r="J30" s="103" t="inlineStr"/>
     </row>
     <row r="31" ht="58" customHeight="1">
       <c r="A31" s="71" t="inlineStr">
@@ -8428,7 +8442,7 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B31" s="102" t="inlineStr">
+      <c r="B31" s="103" t="inlineStr">
         <is>
           <t>Closed Beta — Design Partners</t>
         </is>
@@ -8453,12 +8467,12 @@
           <t>No P0 incidents; majority of design partners show daily active usage; tenant isolation matrix 100% pass with real data; at least 1 non-textile tenant validates the workflow fix</t>
         </is>
       </c>
-      <c r="G31" s="102" t="inlineStr">
+      <c r="G31" s="103" t="inlineStr">
         <is>
           <t>Production (limited)</t>
         </is>
       </c>
-      <c r="H31" s="102" t="inlineStr">
+      <c r="H31" s="103" t="inlineStr">
         <is>
           <t>After Sprint 3</t>
         </is>
@@ -8468,7 +8482,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J31" s="102" t="inlineStr"/>
+      <c r="J31" s="103" t="inlineStr"/>
     </row>
     <row r="32" ht="58" customHeight="1">
       <c r="A32" s="72" t="inlineStr">
@@ -8476,7 +8490,7 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B32" s="102" t="inlineStr">
+      <c r="B32" s="103" t="inlineStr">
         <is>
           <t>Staged Open Beta</t>
         </is>
@@ -8501,12 +8515,12 @@
           <t>Error rate + latency within SLO at every tier; no scheduler double-fire or cross-tenant incident observed; support volume stays manageable</t>
         </is>
       </c>
-      <c r="G32" s="102" t="inlineStr">
+      <c r="G32" s="103" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="H32" s="102" t="inlineStr">
+      <c r="H32" s="103" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
@@ -8516,7 +8530,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J32" s="102" t="inlineStr"/>
+      <c r="J32" s="103" t="inlineStr"/>
     </row>
     <row r="33" ht="58" customHeight="1">
       <c r="A33" s="73" t="inlineStr">
@@ -8524,7 +8538,7 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B33" s="102" t="inlineStr">
+      <c r="B33" s="103" t="inlineStr">
         <is>
           <t>General Availability / Self-Serve Launch</t>
         </is>
@@ -8549,12 +8563,12 @@
           <t>Sustained SLA at ~100-tenant traffic with no open P0s for a full monitoring cycle</t>
         </is>
       </c>
-      <c r="G33" s="102" t="inlineStr">
+      <c r="G33" s="103" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="H33" s="102" t="inlineStr">
+      <c r="H33" s="103" t="inlineStr">
         <is>
           <t>After Sprint 5</t>
         </is>
@@ -8564,7 +8578,7 @@
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J33" s="102" t="inlineStr"/>
+      <c r="J33" s="103" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="57" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): mark FIX-002-D Done, Sprint 1 = 4/6 shipped
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -5138,7 +5138,7 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Running record. Updated side-by-side after every shipped commit. Currently: 9 Done, 15 in backlog.</t>
+          <t>Running record. Updated side-by-side after every shipped commit. Currently: 10 Done, 14 in backlog.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="E7" s="95" t="inlineStr">
         <is>
-          <t>3/6 shipped (FIX-002-C added migration ledger).</t>
+          <t>4/6 shipped. Remaining: FIX-002-E (uploads -&gt; obj_store) and FIX-002-F (Dockerfile).</t>
         </is>
       </c>
     </row>
@@ -5943,9 +5943,9 @@
           <t>tests: single-fire under multiple simulated replicas</t>
         </is>
       </c>
-      <c r="H20" s="37" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H20" s="101" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I20" s="36" t="inlineStr">
@@ -5953,9 +5953,21 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="J20" s="103" t="inlineStr"/>
-      <c r="K20" s="103" t="inlineStr"/>
-      <c r="L20" s="103" t="inlineStr"/>
+      <c r="J20" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="K20" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="L20" s="103" t="inlineStr">
+        <is>
+          <t>(this commit)</t>
+        </is>
+      </c>
       <c r="M20" s="22" t="inlineStr">
         <is>
           <t>Half-day fix. Requires design decision on external cron vs leader election.</t>

</xml_diff>

<commit_message>
docs(tracker): mark FIX-002-E Done, Sprint 1 = 5/6 shipped
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -5138,7 +5138,7 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Running record. Updated side-by-side after every shipped commit. Currently: 10 Done, 14 in backlog.</t>
+          <t>Running record. Updated side-by-side after every shipped commit. Currently: 11 Done, 13 in backlog.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="E7" s="95" t="inlineStr">
         <is>
-          <t>4/6 shipped. Remaining: FIX-002-E (uploads -&gt; obj_store) and FIX-002-F (Dockerfile).</t>
+          <t>5/6 shipped. Remaining: FIX-002-F (Dockerfile).</t>
         </is>
       </c>
     </row>
@@ -6010,9 +6010,9 @@
           <t>tests: upload, download, cross-replica visibility, deletion</t>
         </is>
       </c>
-      <c r="H21" s="37" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="H21" s="101" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I21" s="36" t="inlineStr">
@@ -6020,9 +6020,21 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="J21" s="103" t="inlineStr"/>
-      <c r="K21" s="103" t="inlineStr"/>
-      <c r="L21" s="103" t="inlineStr"/>
+      <c r="J21" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="K21" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="L21" s="103" t="inlineStr">
+        <is>
+          <t>(this commit)</t>
+        </is>
+      </c>
       <c r="M21" s="22" t="inlineStr">
         <is>
           <t>Half-day. Depends on FIX-002-C for the migration. Also closes FIX-001-E EC8 (legacy local files for tenant deletion).</t>

</xml_diff>

<commit_message>
docs(tracker): FIX-003-B done, Sprint 2 = 8/12 shipped
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -3155,20 +3155,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J22" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J22" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K22" s="103" t="inlineStr"/>
-      <c r="L22" s="103" t="inlineStr"/>
-      <c r="M22" s="103" t="inlineStr"/>
+      <c r="L22" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M22" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N22" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O22" s="22" t="inlineStr"/>
+      <c r="O22" s="22" t="inlineStr">
+        <is>
+          <t>Shipped in FIX-003-B (f18bbc3).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="103" t="inlineStr">
@@ -3338,20 +3350,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J25" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J25" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K25" s="103" t="inlineStr"/>
-      <c r="L25" s="103" t="inlineStr"/>
-      <c r="M25" s="103" t="inlineStr"/>
+      <c r="L25" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M25" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N25" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O25" s="22" t="inlineStr"/>
+      <c r="O25" s="22" t="inlineStr">
+        <is>
+          <t>Shipped in FIX-003-B (f18bbc3).</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="103" t="inlineStr">
@@ -3460,20 +3484,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J27" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J27" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K27" s="103" t="inlineStr"/>
-      <c r="L27" s="103" t="inlineStr"/>
-      <c r="M27" s="103" t="inlineStr"/>
+      <c r="L27" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M27" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N27" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O27" s="22" t="inlineStr"/>
+      <c r="O27" s="22" t="inlineStr">
+        <is>
+          <t>Shipped in FIX-003-B (f18bbc3).</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="103" t="inlineStr">
@@ -3582,20 +3618,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J29" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J29" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K29" s="103" t="inlineStr"/>
-      <c r="L29" s="103" t="inlineStr"/>
-      <c r="M29" s="103" t="inlineStr"/>
+      <c r="L29" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M29" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N29" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O29" s="22" t="inlineStr"/>
+      <c r="O29" s="22" t="inlineStr">
+        <is>
+          <t>Already closed by FIX-001-F; regression-guarded in FIX-003-B.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="103" t="inlineStr">
@@ -5164,7 +5212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5297,7 +5345,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>IN PROGRESS. 4/12 shipped: tenant safety helpers (FIX-001-C), TENANT_COLLECTIONS wipe (FIX-001-E), tenant-scoped OTP + WhatsApp routing (FIX-003-A, folds S2-04). Remaining: 4x P1 tenancy hygiene + 4x P2 cleanup.</t>
+          <t>IN PROGRESS. 8/12 shipped: tenant helpers (FIX-001-C), TENANT_COLLECTIONS wipe (FIX-001-E), OTP+WhatsApp tenant scoping (FIX-003-A, folds S2-04), hygiene batch (FIX-003-B: enrich_decisions guard, contacts.type index, register race, active-workflow lock-in). Remaining 4: S2-06 session invalidation, S2-07 email verif + password reset, S2-09 denormalized names, S2-11 AI setup failure flag.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5307,7 +5355,7 @@
       </c>
       <c r="E8" s="106" t="inlineStr">
         <is>
-          <t>4/12 shipped.</t>
+          <t>8/12 shipped. 4 remaining (all P1 hygiene).</t>
         </is>
       </c>
     </row>
@@ -7254,9 +7302,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
           <t>Blocked on S5-01 (Stand up staging env). Single-tenant deployments unaffected.</t>
@@ -7309,12 +7354,76 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
           <t>Sprint 3 territory (S3-03 or new S3-05). Removes the whole class of cross-tenant WhatsApp collision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FIX-003-B</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sprint 2 / Tenancy Hygiene</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>S2-05 + S2-08 + S2-10 + S2-12</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Sprint 2 hygiene batch: enrich_decisions tenant guard, contacts.type index, register race, active-workflow lock-in</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>S2-05 defense-in-depth: enrich_decision(s) now filter task_ids/created_by lookups by tenant_id; batch inference for single-tenant callers who forget; explicit at all 6 caller sites. S2-08: contacts index was on dead field `kind` (the collection uses `type`); replaced + drops legacy. S2-10: register handler was find_one-then-insert_one with orphan-tenant risk on concurrent race; now catches DuplicateKeyError, rolls back the orphan tenant, returns friendly 400. S2-12: verified S2-12 was fully closed by FIX-001-F and locked it in with a regression test guarding against ['delivered','paid'] reappearing anywhere in server.py.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>server.py (enrich_decision(s) + know360 caller + owner_brief caller + contacts index in bootstrap); routers/decisions.py (6 enrich_decision callers); routers/brief.py (awaiting_approval); routers/auth.py (register DuplicateKeyError handling + orphan tenant rollback)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>tests/test_tenancy_hygiene_batch.py - 10 tests (4x enrich_decision tenant guard incl. batch inference + mixed-batch + creator lookup, 2x contacts.type index bootstrap, 2x register DuplicateKeyError + rollback + email unique index invariant, 2x active-workflow lock-in)</t>
+        </is>
+      </c>
+      <c r="H50" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>f18bbc3</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Bundled 4 small Sprint 2 items. All P1/P2, no go-live blocker individually; bundled for efficiency. S2-12 was already implemented by FIX-001-F; this ship formalized the regression guard.</t>
         </is>
       </c>
     </row>
@@ -7604,9 +7713,9 @@
 (Scale/Ops)</t>
         </is>
       </c>
-      <c r="C9" s="56" t="inlineStr">
-        <is>
-          <t>[S2-05] Fix unfiltered enrich_decisions fetch
+      <c r="C9" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-05] Fix unfiltered enrich_decisions fetch
 (Tenancy/Data)</t>
         </is>
       </c>
@@ -7688,9 +7797,9 @@
 (Security/Auth)</t>
         </is>
       </c>
-      <c r="C12" s="55" t="inlineStr">
-        <is>
-          <t>[S2-08] Fix dead contacts.kind index
+      <c r="C12" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-08] Fix dead contacts.kind index
 (Tenancy/Data)</t>
         </is>
       </c>
@@ -7740,9 +7849,9 @@
 (Security/Auth)</t>
         </is>
       </c>
-      <c r="C14" s="56" t="inlineStr">
-        <is>
-          <t>[S2-10] Handle concurrent-registration race
+      <c r="C14" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-10] Handle concurrent-registration race
 (Tenancy/Data)</t>
         </is>
       </c>
@@ -7774,9 +7883,9 @@
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
-      <c r="C16" s="56" t="inlineStr">
-        <is>
-          <t>[S2-12] Fix 'active workflows' hardcoded terminal stages
+      <c r="C16" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-12] Fix 'active workflows' hardcoded terminal stages
 (Tenancy/Data)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs(tracker): FIX-003-C done, Sprint 2 = 11/12 (S2-07 remains)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -3228,20 +3228,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J23" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J23" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K23" s="103" t="inlineStr"/>
-      <c r="L23" s="103" t="inlineStr"/>
-      <c r="M23" s="103" t="inlineStr"/>
+      <c r="L23" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M23" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N23" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O23" s="22" t="inlineStr"/>
+      <c r="O23" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-003-C (f48bd24). </t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="103" t="inlineStr">
@@ -3423,20 +3435,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J26" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J26" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K26" s="103" t="inlineStr"/>
-      <c r="L26" s="103" t="inlineStr"/>
-      <c r="M26" s="103" t="inlineStr"/>
+      <c r="L26" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M26" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N26" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O26" s="22" t="inlineStr"/>
+      <c r="O26" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-003-C (f48bd24). </t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="103" t="inlineStr">
@@ -3557,20 +3581,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J28" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J28" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K28" s="103" t="inlineStr"/>
-      <c r="L28" s="103" t="inlineStr"/>
-      <c r="M28" s="103" t="inlineStr"/>
+      <c r="L28" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M28" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N28" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O28" s="22" t="inlineStr"/>
+      <c r="O28" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-003-C (f48bd24). </t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="103" t="inlineStr">
@@ -5212,7 +5248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5345,7 +5381,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>IN PROGRESS. 8/12 shipped: tenant helpers (FIX-001-C), TENANT_COLLECTIONS wipe (FIX-001-E), OTP+WhatsApp tenant scoping (FIX-003-A, folds S2-04), hygiene batch (FIX-003-B: enrich_decisions guard, contacts.type index, register race, active-workflow lock-in). Remaining 4: S2-06 session invalidation, S2-07 email verif + password reset, S2-09 denormalized names, S2-11 AI setup failure flag.</t>
+          <t>IN PROGRESS. 11/12 shipped: tenant helpers (FIX-001-C), TENANT_COLLECTIONS wipe (FIX-001-E), OTP+WhatsApp tenant scoping (FIX-003-A, folds S2-04), hygiene batch (FIX-003-B), JWT revocation + contact rename cascade + AI regen status (FIX-003-C). Remaining 1: S2-07 email verification + password reset (green-field email service).</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5355,7 +5391,7 @@
       </c>
       <c r="E8" s="106" t="inlineStr">
         <is>
-          <t>8/12 shipped. 4 remaining (all P1 hygiene).</t>
+          <t>11/12 shipped. Only S2-07 remains (FIX-003-D).</t>
         </is>
       </c>
     </row>
@@ -7424,6 +7460,73 @@
       <c r="M50" t="inlineStr">
         <is>
           <t>Bundled 4 small Sprint 2 items. All P1/P2, no go-live blocker individually; bundled for efficiency. S2-12 was already implemented by FIX-001-F; this ship formalized the regression guard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>FIX-003-C</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Sprint 2 / Auth &amp; Hygiene</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>S2-06 + S2-09 + S2-11</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>JWT revocation on logout + contact rename cascade + AI regen failure flag</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>S2-06 (security): /logout only cleared browser cookie; JWT stayed valid until exp (7 days). Now: every access token gains a random jti; /logout records (jti, exp) in db.revoked_tokens; get_current_user checks is_revoked on every authenticated request. TTL index on revoked_tokens.exp keeps the table bounded. Fail-open on Mongo blip so a transient DB error doesn't lock everyone out. /logout has no auth dependency so a corrupted/already-revoked token can still clear the cookie. S2-09: contact_name is denormalized into invoices/payments/workflows.counterparty; renaming a contact left every existing row with stale display + search columns. update_contact now cascades: match by contact_id (recent rows) + fall back to exact old_name where contact_id is null (legacy rows). Every cascade update is tenant-scoped. S2-11: regenerate_operating_model + regenerate_finance_categories called AI generators directly, so silent AI degradation (timeout, malformed JSON, empty pipelines) left tenants with default configs and no signal. Now uses ai_setup._with_status wrappers, persists ai_setup_status on tenant, returns ai_setup_status_summary in response. On defaulted/failed run, preserves existing config instead of clobbering.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>services/session_revocation.py (new: revoke/is_revoked with fail-open); core.py (create_token adds jti, get_current_user checks is_revoked); routers/auth.py (/logout revokes current jti + Request import); server.py (bootstrap: revoked_tokens jti unique + exp TTL indexes; regenerate_operating_model + regenerate_finance_categories status-tracking; update_contact rename cascade)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>tests/test_session_revocation.py - 17 tests (6 revoke/is_revoked contract, 2 jti in create_token, 2 /logout revocation + no auth dep, 1 get_current_user revocation check, 1 bootstrap indexes, 2 contact rename cascade guards, 3 AI regen status tracking)</t>
+        </is>
+      </c>
+      <c r="H51" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>f48bd24</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>S2-06 is the real security fix in this batch. Sprint 2 now 11/12 shipped; only S2-07 (email verification + password reset, green-field email service) remains.</t>
         </is>
       </c>
     </row>
@@ -7745,9 +7848,9 @@
 (Scale/Ops)</t>
         </is>
       </c>
-      <c r="C10" s="55" t="inlineStr">
-        <is>
-          <t>[S2-06] Add session invalidation on logout/password-change
+      <c r="C10" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-06] Add session invalidation on logout/password-change
 (Tenancy/Data)</t>
         </is>
       </c>
@@ -7823,9 +7926,9 @@
 (Security/Auth)</t>
         </is>
       </c>
-      <c r="C13" s="56" t="inlineStr">
-        <is>
-          <t>[S2-09] Fix denormalized-name staleness
+      <c r="C13" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-09] Fix denormalized-name staleness
 (Tenancy/Data)</t>
         </is>
       </c>
@@ -7869,9 +7972,9 @@
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
-      <c r="C15" s="55" t="inlineStr">
-        <is>
-          <t>[S2-11] Flag AI-operating-model generation failures
+      <c r="C15" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-11] Flag AI-operating-model generation failures
 (Tenancy/Data)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs(tracker): FIX-003-D done -- SPRINT 2 COMPLETE (12/12)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -3301,20 +3301,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J24" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J24" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K24" s="103" t="inlineStr"/>
-      <c r="L24" s="103" t="inlineStr"/>
-      <c r="M24" s="103" t="inlineStr"/>
+      <c r="L24" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M24" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N24" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O24" s="22" t="inlineStr"/>
+      <c r="O24" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-003-D (4ef865e). </t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="103" t="inlineStr">
@@ -5248,7 +5260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5381,7 +5393,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>IN PROGRESS. 11/12 shipped: tenant helpers (FIX-001-C), TENANT_COLLECTIONS wipe (FIX-001-E), OTP+WhatsApp tenant scoping (FIX-003-A, folds S2-04), hygiene batch (FIX-003-B), JWT revocation + contact rename cascade + AI regen status (FIX-003-C). Remaining 1: S2-07 email verification + password reset (green-field email service).</t>
+          <t>DONE. 12/12 shipped: tenant helpers (FIX-001-C), TENANT_COLLECTIONS wipe (FIX-001-E), OTP+WhatsApp tenant scoping (FIX-003-A), hygiene batch (FIX-003-B), JWT revocation + contact rename + AI regen status (FIX-003-C), email verification + password reset (FIX-003-D).</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5391,7 +5403,7 @@
       </c>
       <c r="E8" s="106" t="inlineStr">
         <is>
-          <t>11/12 shipped. Only S2-07 remains (FIX-003-D).</t>
+          <t>12/12 shipped. Sprint 2 COMPLETE.</t>
         </is>
       </c>
     </row>
@@ -7527,6 +7539,183 @@
       <c r="M51" t="inlineStr">
         <is>
           <t>S2-06 is the real security fix in this batch. Sprint 2 now 11/12 shipped; only S2-07 (email verification + password reset, green-field email service) remains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>FIX-003-D</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sprint 2 / Email + Auth</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>S2-07</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Email verification + password reset (green-field)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>New auth flows built from scratch. services/auth_emails.py provides a single token model for both flows: auth_email_tokens keyed by URL-safe 32-char token (secrets.token_urlsafe(24) = ~192 bits entropy), single-use consume() with atomic filter on used_at:None, issue() idempotent within cooldown to prevent inbox flood. TTLs differ by kind: email_verify=3 days, password_reset=1 hour. 4 endpoints on routers/auth.py: POST /auth/email/send-verification (authenticated), GET /auth/email/verify/{token} (public), POST /auth/password/forgot (public, canonical response = no email enumeration), POST /auth/password/reset (public, single-use + invalidates sibling reset tokens). Register hook: verification email sent best-effort on /auth/register (SMTP down never fails registration). 3 bootstrap indexes: token unique, expires_at TTL, kind+email+used_at compound for issue reuse lookup. Passwordless (OTP-only) accounts get canonical /forgot response but no email + explicit refusal on /reset.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>services/auth_emails.py (new: token model + email templates); routers/auth.py (PasswordForgotInput/PasswordResetInput models, 4 new endpoints, register hook, _app_base_url helper); server.py (3 auth_email_tokens indexes in bootstrap)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>tests/test_email_verification_and_reset.py - 23 tests (8 issue contract, 5 consume single-use + failure modes, 1 invalidate isolation, 5 endpoint shape guards, 1 register best-effort, 1 bootstrap indexes, 2 email templates)</t>
+        </is>
+      </c>
+      <c r="H52" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>4ef865e</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>SPRINT 2 COMPLETE (12/12). Green-field build. Follow-ups: FIX-FUP-18 per-IP rate limit on /forgot; FIX-FUP-19 frontend /verify-email + /reset-password pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>FIX-FUP-18</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-003-D)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>(logged during 003-D)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Per-IP rate limit on /auth/password/forgot</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Today the throttle is per-account via services.auth_emails.issue() cooldown (60s). That prevents inbox spam for one target, but an attacker cycling emails can still overwhelm SMTP quota. Add IP-based rate limit (e.g. 10 requests/hour) via a middleware or a small in-process counter.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>middleware or routers/auth.py</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>test: 11 rapid requests from same IP -&gt; 11th returns 429</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Sprint 0/security territory; not a go-live blocker for controlled beta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>FIX-FUP-19</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-003-D)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>(logged during 003-D)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Frontend pages: /verify-email + /reset-password</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Backend links point at APP_BASE_URL/verify-email?token=... and APP_BASE_URL/reset-password?token=... but no frontend routes exist yet. Add: two lightweight pages that read the token from the query string, call GET /api/auth/email/verify/{token} or POST /api/auth/password/reset respectively, and show success/error UI.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>frontend/src/App.js routes; new components</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>manual: click a verification email link -&gt; success page renders</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Backend is complete and callable via curl; frontend pages are the last mile for users.</t>
         </is>
       </c>
     </row>
@@ -7874,9 +8063,9 @@
 (Security/Auth)</t>
         </is>
       </c>
-      <c r="C11" s="55" t="inlineStr">
-        <is>
-          <t>[S2-07] Add email verification + password reset
+      <c r="C11" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S2-07] Add email verification + password reset
 (Tenancy/Data)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-A done -- RBAC Wave 1 shipped (RBAC-01/02/03)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -461,7 +461,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -497,11 +497,55 @@
         <color rgb="00B4B4B4"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -791,6 +835,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1380,7 +1426,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
@@ -1424,7 +1469,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
@@ -1474,7 +1518,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
@@ -1505,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="B2:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1518,7 +1561,6 @@
     <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1533,7 +1575,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="16" t="inlineStr">
         <is>
@@ -1600,7 +1641,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
@@ -1612,7 +1652,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="26" customHeight="1">
       <c r="B14" s="20" t="inlineStr">
         <is>
@@ -5459,14 +5498,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J55" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-A (a44135f). </t>
         </is>
       </c>
     </row>
@@ -5516,14 +5570,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J56" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-A (a44135f). </t>
         </is>
       </c>
     </row>
@@ -5573,14 +5642,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J57" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-A (a44135f). </t>
         </is>
       </c>
     </row>
@@ -7205,7 +7289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9655,6 +9739,238 @@
       <c r="M54" t="inlineStr">
         <is>
           <t>Backend is complete and callable via curl; frontend pages are the last mile for users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>FIX-004-A</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>RBAC-01 + RBAC-02 + RBAC-03</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>RBAC Wave 1: HMAC-signed drafts + CAPTCHA/rate-limit register + SSRF-guarded signup AI</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>3 P0 public-endpoint gaps closed. RBAC-01: onboarding drafts were world-accessible by ID; now HMAC-signed X-Draft-Token required on GET/PATCH + per-IP rate limit on create. RBAC-02: /register was unauth + unlimited; now Turnstile/hCaptcha token verification + 3/hour/IP rate limit. RBAC-03: signup AI endpoints (website-intel, tts, stt, interview/*) were unauth credit-burners; now shared _guard_signup_endpoint dep runs hourly (30/IP) + burst (5/10s) rate-limit + CAPTCHA. website-intel gains SSRF guard blocking private v4/v6 ranges, loopback, link-local, cloud-metadata IPs (169.254.169.254), and non-http(s) schemes. Also introduces reusable infra: services/rate_limit.py (sliding-window, fail-open), services/captcha.py (Turnstile/hCaptcha with 3 env states), services/ssrf_guard.py (single choke-point URL validator), services/auth/draft_tokens.py (HMAC sign/verify). All will be reused by RBAC Waves 2-5.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>services/rate_limit.py (new); services/captcha.py (new); services/ssrf_guard.py (new); services/auth/draft_tokens.py (new); services/auth/__init__.py (exports); routers/onboarding.py (draft token + rate limit); routers/auth.py (register captcha + rate limit); routers/signup.py (guard + SSRF on 9 endpoints)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>tests/test_rbac_wave1.py - 41 tests (9 rate_limit contract + client_ip variants, 5 captcha env-state combos, 10 SSRF guard incl. v6 loopback + link-local, 7 draft tokens, 5 onboarding gate, 2 register gate, 3 signup AI gate)</t>
+        </is>
+      </c>
+      <c r="H55" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>a44135f</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Backend-complete. FIX-FUP-20 tracks the frontend integration (Turnstile widget, X-Draft-Token header, X-Captcha-Token header). Rate limiter is per-worker; Redis backend logged as FIX-FUP-21 for multi-worker deploys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>FIX-FUP-20</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-A)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>(logged during Wave 1)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Frontend integration for RBAC Wave 1 (CAPTCHA widget + auth headers)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Backend is complete but the frontend needs 3 updates: (a) onboarding wizard stores the draft_token returned from POST /onboarding/draft, sends X-Draft-Token on every subsequent GET/PATCH; (b) /register page renders a Cloudflare Turnstile widget (free, invisible for most users), passes the resulting captcha_token in the request body; (c) /signup wizard renders same widget on first AI call per session, passes the resulting token via X-Captcha-Token header. Without these, the frontend will fail against a prod backend that has CAPTCHA_REQUIRED=1.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>frontend/src pages: OnboardingWizard, Register, Signup</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>manual: form submits succeed; loading Turnstile in dev works</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Backend is deployed-ready in permissive mode today; frontend fix required before flipping CAPTCHA_REQUIRED=1 in prod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>FIX-FUP-21</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-A)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>(logged during Wave 1)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cross-process rate limiter (Redis backend)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Current services/rate_limit.py is in-process. With N uvicorn workers the effective per-IP ceiling is N*cap. Fine for the current unauth surface (a bot burst is spread across workers roughly evenly), but not correct. Replace with a Redis-backed sliding window using INCR + EXPIRE or a Lua script. Same public API so no caller changes.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>services/rate_limit.py</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>test: 3-worker simulation, verify shared counter</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Sprint 3+ territory when we scale beyond 1 worker per instance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>FIX-FUP-22</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-A)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>(logged during Wave 1)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>SSRF guard v2: pin resolved IP through httpx transport</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Current is_url_safe_for_fetch resolves hostname + checks IPs, then httpx.get re-resolves independently. In the ~100ms gap between check + fetch, a hostile DNS server could re-flip the record from public to private. Fix: use httpx transport with a custom Resolver that reuses the resolved IPs from is_url_safe_for_fetch (or pass resolved IP + Host header separately). Adds SNI + Host complexity.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>services/ssrf_guard.py, routers/signup.py</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>test: TOCTOU race simulator with a mock resolver flipping IPs mid-call</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Current guard is fine for the SME-scale threat model; hardening is nice-to-have.</t>
         </is>
       </c>
     </row>
@@ -11603,6 +11919,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="109" t="inlineStr">
         <is>
@@ -11610,6 +11927,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="111" t="inlineStr">
         <is>
@@ -11679,6 +11997,8 @@
         </is>
       </c>
       <c r="F8" s="113" t="inlineStr"/>
+      <c r="G8" s="119" t="n"/>
+      <c r="H8" s="120" t="n"/>
       <c r="I8" s="113" t="inlineStr">
         <is>
           <t>Simple, works. Only 8 endpoints use it.</t>
@@ -11712,6 +12032,8 @@
         </is>
       </c>
       <c r="F9" s="113" t="inlineStr"/>
+      <c r="G9" s="119" t="n"/>
+      <c r="H9" s="120" t="n"/>
       <c r="I9" s="113" t="inlineStr">
         <is>
           <t>Only ~35 route uses; most endpoints use bare get_current_user.</t>
@@ -11745,6 +12067,8 @@
         </is>
       </c>
       <c r="F10" s="113" t="inlineStr"/>
+      <c r="G10" s="119" t="n"/>
+      <c r="H10" s="120" t="n"/>
       <c r="I10" s="113" t="inlineStr">
         <is>
           <t>Owner is a magic god-role. No way to say 'owner minus finance'.</t>
@@ -11778,6 +12102,8 @@
         </is>
       </c>
       <c r="F11" s="113" t="inlineStr"/>
+      <c r="G11" s="119" t="n"/>
+      <c r="H11" s="120" t="n"/>
       <c r="I11" s="113" t="inlineStr">
         <is>
           <t>Sane starter set.</t>
@@ -11811,6 +12137,8 @@
         </is>
       </c>
       <c r="F12" s="113" t="inlineStr"/>
+      <c r="G12" s="119" t="n"/>
+      <c r="H12" s="120" t="n"/>
       <c r="I12" s="113" t="inlineStr">
         <is>
           <t>Custom roles created via /tenant/roles have NO way to add perms without editing each user.</t>
@@ -11844,6 +12172,8 @@
         </is>
       </c>
       <c r="F13" s="113" t="inlineStr"/>
+      <c r="G13" s="119" t="n"/>
+      <c r="H13" s="120" t="n"/>
       <c r="I13" s="113" t="inlineStr">
         <is>
           <t>Reasonable granularity. But 'approvals', 'leave_approve', 'inbox', 'tasks', 'ledger' are unused as decorators.</t>
@@ -11877,12 +12207,15 @@
         </is>
       </c>
       <c r="F14" s="113" t="inlineStr"/>
+      <c r="G14" s="119" t="n"/>
+      <c r="H14" s="120" t="n"/>
       <c r="I14" s="113" t="inlineStr">
         <is>
           <t>Silent inconsistency — tenants get 'operations' but permission logic expects 'production'.</t>
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="111" t="inlineStr">
         <is>
@@ -11952,6 +12285,8 @@
         </is>
       </c>
       <c r="F18" s="113" t="inlineStr"/>
+      <c r="G18" s="119" t="n"/>
+      <c r="H18" s="120" t="n"/>
       <c r="I18" s="113" t="inlineStr">
         <is>
           <t>One user = one workspace. Accountants/consultants who serve multiple SMEs cannot exist as a single user account — must register N times with N emails.</t>
@@ -11985,6 +12320,8 @@
         </is>
       </c>
       <c r="F19" s="113" t="inlineStr"/>
+      <c r="G19" s="119" t="n"/>
+      <c r="H19" s="120" t="n"/>
       <c r="I19" s="113" t="inlineStr">
         <is>
           <t>Blocks multi-tenant membership. Same anti-pattern we JUST fixed for phones (FIX-003-A). Email needs the same treatment.</t>
@@ -12018,6 +12355,8 @@
         </is>
       </c>
       <c r="F20" s="113" t="inlineStr"/>
+      <c r="G20" s="119" t="n"/>
+      <c r="H20" s="120" t="n"/>
       <c r="I20" s="113" t="inlineStr">
         <is>
           <t>Good for field employees without email discipline.</t>
@@ -12051,6 +12390,8 @@
         </is>
       </c>
       <c r="F21" s="113" t="inlineStr"/>
+      <c r="G21" s="119" t="n"/>
+      <c r="H21" s="120" t="n"/>
       <c r="I21" s="113" t="inlineStr">
         <is>
           <t>But: no 'accepted' vs 'pending' state tracking, and invited users are already listed in /users same as active ones (no visible pending state to admin).</t>
@@ -12084,6 +12425,8 @@
         </is>
       </c>
       <c r="F22" s="113" t="inlineStr"/>
+      <c r="G22" s="119" t="n"/>
+      <c r="H22" s="120" t="n"/>
       <c r="I22" s="113" t="inlineStr">
         <is>
           <t>But there's no session revocation on suspend — the token stays cryptographically valid until it expires (though get_current_user WILL 403 next request). Combine with FIX-003-C's jti revocation.</t>
@@ -12117,12 +12460,15 @@
         </is>
       </c>
       <c r="F23" s="113" t="inlineStr"/>
+      <c r="G23" s="119" t="n"/>
+      <c r="H23" s="120" t="n"/>
       <c r="I23" s="113" t="inlineStr">
         <is>
           <t>Good separation. But: platform admins can do cross-tenant reclassify/delete — no super-audit trail visible.</t>
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="111" t="inlineStr">
         <is>
@@ -12192,6 +12538,8 @@
         </is>
       </c>
       <c r="F27" s="113" t="inlineStr"/>
+      <c r="G27" s="119" t="n"/>
+      <c r="H27" s="120" t="n"/>
       <c r="I27" s="113" t="inlineStr">
         <is>
           <t>Good baseline.</t>
@@ -12225,6 +12573,8 @@
         </is>
       </c>
       <c r="F28" s="113" t="inlineStr"/>
+      <c r="G28" s="119" t="n"/>
+      <c r="H28" s="120" t="n"/>
       <c r="I28" s="113" t="inlineStr">
         <is>
           <t>Creating a 'warehouse_manager' role and expecting it to see finance requires editing EACH user's permissions[] override. No way to say 'this ROLE always gets finance perm'.</t>
@@ -12258,12 +12608,15 @@
         </is>
       </c>
       <c r="F29" s="113" t="inlineStr"/>
+      <c r="G29" s="119" t="n"/>
+      <c r="H29" s="120" t="n"/>
       <c r="I29" s="113" t="inlineStr">
         <is>
           <t>Fine as an escape hatch, but shouldn't be the ONLY way to grant a permission.</t>
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="109" t="inlineStr">
         <is>
@@ -12278,6 +12631,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="111" t="inlineStr">
         <is>
@@ -12350,6 +12704,8 @@
           <t>Any client can guess a draft ID and read/write another founder's onboarding data (industry, description, roles, phone). draft_id is a UUID but there's zero enumeration protection.</t>
         </is>
       </c>
+      <c r="F36" s="119" t="n"/>
+      <c r="G36" s="120" t="n"/>
       <c r="H36" s="113" t="inlineStr">
         <is>
           <t>onboarding.py:146, 156</t>
@@ -12387,6 +12743,8 @@
           <t>Anyone can spin up unlimited tenants. AI credit burn + storage cost + noisy dashboard.</t>
         </is>
       </c>
+      <c r="F37" s="119" t="n"/>
+      <c r="G37" s="120" t="n"/>
       <c r="H37" s="113" t="inlineStr">
         <is>
           <t>auth.py:96</t>
@@ -12424,6 +12782,8 @@
           <t>Server-side URL fetch (SSRF potential) + unauthenticated AI calls burning credits. Any attacker can drain quota.</t>
         </is>
       </c>
+      <c r="F38" s="119" t="n"/>
+      <c r="G38" s="120" t="n"/>
       <c r="H38" s="113" t="inlineStr">
         <is>
           <t>signup.py:125, tts, stt</t>
@@ -12461,6 +12821,8 @@
           <t>Any employee can create workflows. But DELETE /workflows/{id} requires owner. Asymmetric.</t>
         </is>
       </c>
+      <c r="F39" s="119" t="n"/>
+      <c r="G39" s="120" t="n"/>
       <c r="H39" s="113" t="inlineStr">
         <is>
           <t>server.py:2484 vs 2596</t>
@@ -12498,6 +12860,8 @@
           <t>Approving a captured draft turns it into real workflow/task data. Should be role/perm-gated.</t>
         </is>
       </c>
+      <c r="F40" s="119" t="n"/>
+      <c r="G40" s="120" t="n"/>
       <c r="H40" s="113" t="inlineStr">
         <is>
           <t>server.py:5167-5211</t>
@@ -12535,6 +12899,8 @@
           <t>Any employee can trigger a full tenant follow-up sweep (LLM cost, notification spam).</t>
         </is>
       </c>
+      <c r="F41" s="119" t="n"/>
+      <c r="G41" s="120" t="n"/>
       <c r="H41" s="113" t="inlineStr">
         <is>
           <t>server.py:3205</t>
@@ -12572,6 +12938,8 @@
           <t>Reassign, DELETE execution-plan, prioritize (LLM), bulk delete — all open to every logged-in user. Inline `role!=owner` check only on /tasks/{id} DELETE.</t>
         </is>
       </c>
+      <c r="F42" s="119" t="n"/>
+      <c r="G42" s="120" t="n"/>
       <c r="H42" s="113" t="inlineStr">
         <is>
           <t>tasks.py all</t>
@@ -12609,6 +12977,8 @@
           <t>Every employee can burn STT/LLM credits without any quota. Voice notes attach to any task by id.</t>
         </is>
       </c>
+      <c r="F43" s="119" t="n"/>
+      <c r="G43" s="120" t="n"/>
       <c r="H43" s="113" t="inlineStr">
         <is>
           <t>server.py:2141, 2161</t>
@@ -12646,6 +13016,8 @@
           <t>Decorator gives no auth signal at endpoint level — reviewers reading the route can't tell what's gated. Move to require_perm('leave_approve').</t>
         </is>
       </c>
+      <c r="F44" s="119" t="n"/>
+      <c r="G44" s="120" t="n"/>
       <c r="H44" s="113" t="inlineStr">
         <is>
           <t>team.py:322, 328, 335</t>
@@ -12683,6 +13055,8 @@
           <t>'ask' is the QUERY permission. Export = bulk data extraction, higher privilege.</t>
         </is>
       </c>
+      <c r="F45" s="119" t="n"/>
+      <c r="G45" s="120" t="n"/>
       <c r="H45" s="113" t="inlineStr">
         <is>
           <t>brain.py:64</t>
@@ -12720,6 +13094,8 @@
           <t>Any employee can insert into shared tenant memory. No 'memory_write' permission.</t>
         </is>
       </c>
+      <c r="F46" s="119" t="n"/>
+      <c r="G46" s="120" t="n"/>
       <c r="H46" s="113" t="inlineStr">
         <is>
           <t>server.py:3264</t>
@@ -12731,6 +13107,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="111" t="inlineStr">
         <is>
@@ -12803,6 +13180,8 @@
           <t>An accountant serving 5 SMEs must register 5 emails. Founders switching between their bakery + consulting workspace must log out/in. Standard SaaS SME buyers reject this.</t>
         </is>
       </c>
+      <c r="F50" s="119" t="n"/>
+      <c r="G50" s="120" t="n"/>
       <c r="H50" s="113" t="inlineStr">
         <is>
           <t>team.py:122, auth.py:136</t>
@@ -12840,6 +13219,8 @@
           <t>Blocks (B1) permanently. Cannot model 'is member of Tenant A as employee + Tenant B as owner'. Every fix downstream (invite, delete, list users) must be rewritten later — cheaper to do now.</t>
         </is>
       </c>
+      <c r="F51" s="119" t="n"/>
+      <c r="G51" s="120" t="n"/>
       <c r="H51" s="113" t="inlineStr">
         <is>
           <t>team.py:143 + all users.find_one users</t>
@@ -12877,6 +13258,8 @@
           <t>Founder creates 'warehouse_manager' role, must then edit each user's permissions[] individually. Role loses its meaning as a policy unit.</t>
         </is>
       </c>
+      <c r="F52" s="119" t="n"/>
+      <c r="G52" s="120" t="n"/>
       <c r="H52" s="113" t="inlineStr">
         <is>
           <t>core.py:358-361</t>
@@ -12914,6 +13297,8 @@
           <t>Cannot have 'Co-founder with everything EXCEPT finance visibility' — a common early-stage founder ask. No 'break-glass' pattern (grant admin temporarily, log it).</t>
         </is>
       </c>
+      <c r="F53" s="119" t="n"/>
+      <c r="G53" s="120" t="n"/>
       <c r="H53" s="113" t="inlineStr">
         <is>
           <t>core.py:365</t>
@@ -12951,6 +13336,8 @@
           <t>Any code that switches on ROLES silently misses tenants who got 'operations' as a default role.</t>
         </is>
       </c>
+      <c r="F54" s="119" t="n"/>
+      <c r="G54" s="120" t="n"/>
       <c r="H54" s="113" t="inlineStr">
         <is>
           <t>config.py:36 vs 44-48</t>
@@ -12988,6 +13375,8 @@
           <t>Admin cannot see 'you invited 3 people, 1 has accepted, 2 are pending'. Also blocks off-boarding: cannot uninvite before accept.</t>
         </is>
       </c>
+      <c r="F55" s="119" t="n"/>
+      <c r="G55" s="120" t="n"/>
       <c r="H55" s="113" t="inlineStr">
         <is>
           <t>team.py:158-165, GET /users</t>
@@ -13025,6 +13414,8 @@
           <t>Multi-branch SMEs are common in India (kirana chains, salon franchises). Blocks selling to any tenant with &gt;1 physical location.</t>
         </is>
       </c>
+      <c r="F56" s="119" t="n"/>
+      <c r="G56" s="120" t="n"/>
       <c r="H56" s="113" t="inlineStr">
         <is>
           <t>N/A (missing entirely)</t>
@@ -13062,6 +13453,8 @@
           <t>Cannot say 'all Regional Managers get inventory perm' — must edit 12 individual users.</t>
         </is>
       </c>
+      <c r="F57" s="119" t="n"/>
+      <c r="G57" s="120" t="n"/>
       <c r="H57" s="113" t="inlineStr">
         <is>
           <t>N/A (missing entirely)</t>
@@ -13073,6 +13466,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="111" t="inlineStr">
         <is>
@@ -13136,6 +13530,9 @@
           <t>SOC2/DPDP/GDPR compliance + 'who deleted this decision?' operational forensics. Today log_activity is human-readable free text, not queryable, and can be deleted with a normal update.</t>
         </is>
       </c>
+      <c r="E61" s="119" t="n"/>
+      <c r="F61" s="119" t="n"/>
+      <c r="G61" s="120" t="n"/>
       <c r="H61" s="113" t="inlineStr">
         <is>
           <t>Standard in QuickBooks / Zoho One / Odoo.</t>
@@ -13168,6 +13565,9 @@
           <t>User needs to see 'I'm logged in on 3 devices, revoke the phone I lost'. Backend has FIX-003-C jti revocation infra — no UI endpoint exposes it.</t>
         </is>
       </c>
+      <c r="E62" s="119" t="n"/>
+      <c r="F62" s="119" t="n"/>
+      <c r="G62" s="120" t="n"/>
       <c r="H62" s="113" t="inlineStr">
         <is>
           <t>Every consumer + B2B tool for 10 years.</t>
@@ -13200,6 +13600,9 @@
           <t>Departing employee must: revoke all sessions, reassign owned tasks, transfer decisions in-flight, mark authored contacts as reassigned, revoke invite tokens. Today only role-change/suspend/delete exist — the cleanup is manual.</t>
         </is>
       </c>
+      <c r="E63" s="119" t="n"/>
+      <c r="F63" s="119" t="n"/>
+      <c r="G63" s="120" t="n"/>
       <c r="H63" s="113" t="inlineStr">
         <is>
           <t>Enterprise-must-have; SMEs benefit too.</t>
@@ -13232,6 +13635,9 @@
           <t>Insurance, banking-adjacent, finance-team users demand it. Also 'sign-in from a new device' second-factor.</t>
         </is>
       </c>
+      <c r="E64" s="119" t="n"/>
+      <c r="F64" s="119" t="n"/>
+      <c r="G64" s="120" t="n"/>
       <c r="H64" s="113" t="inlineStr">
         <is>
           <t>Universal.</t>
@@ -13264,6 +13670,9 @@
           <t>Founder leaves the company. Today, delete owner blocks 'last owner'; there's no clean promote-then-demote sequence with tenant billing rebind.</t>
         </is>
       </c>
+      <c r="E65" s="119" t="n"/>
+      <c r="F65" s="119" t="n"/>
+      <c r="G65" s="120" t="n"/>
       <c r="H65" s="113" t="inlineStr">
         <is>
           <t>Common at series-A/B.</t>
@@ -13296,6 +13705,9 @@
           <t>DPDP-2023 requires explicit consent for AI processing of PII. Today the app just sends employee names/tasks to Anthropic without a per-tenant consent gate.</t>
         </is>
       </c>
+      <c r="E66" s="119" t="n"/>
+      <c r="F66" s="119" t="n"/>
+      <c r="G66" s="120" t="n"/>
       <c r="H66" s="113" t="inlineStr">
         <is>
           <t>Legal requirement for India.</t>
@@ -13328,6 +13740,9 @@
           <t>On-leave approvers block the workflow. Should be able to say 'while I'm out, X approves for me'. FIX-001-D and team.py have plumbing but no delegation surface.</t>
         </is>
       </c>
+      <c r="E67" s="119" t="n"/>
+      <c r="F67" s="119" t="n"/>
+      <c r="G67" s="120" t="n"/>
       <c r="H67" s="113" t="inlineStr">
         <is>
           <t>Standard in HRIS / procurement.</t>
@@ -13360,6 +13775,9 @@
           <t>Contractor gets finance perm for month-end close, auto-revokes at end of month. Today it's manual add/remove.</t>
         </is>
       </c>
+      <c r="E68" s="119" t="n"/>
+      <c r="F68" s="119" t="n"/>
+      <c r="G68" s="120" t="n"/>
       <c r="H68" s="113" t="inlineStr">
         <is>
           <t>Nice-to-have.</t>
@@ -13392,6 +13810,9 @@
           <t>Enterprise gate. Most SMEs don't ask, but any 50+ employee prospect will.</t>
         </is>
       </c>
+      <c r="E69" s="119" t="n"/>
+      <c r="F69" s="119" t="n"/>
+      <c r="G69" s="120" t="n"/>
       <c r="H69" s="113" t="inlineStr">
         <is>
           <t>SAML for enterprise; Google/MS OAuth for SME.</t>
@@ -13424,6 +13845,9 @@
           <t>Programmatic access (Zapier, custom scripts). Today the only path is JWT extraction from a browser session.</t>
         </is>
       </c>
+      <c r="E70" s="119" t="n"/>
+      <c r="F70" s="119" t="n"/>
+      <c r="G70" s="120" t="n"/>
       <c r="H70" s="113" t="inlineStr">
         <is>
           <t>Standard.</t>
@@ -13456,6 +13880,9 @@
           <t>Share a workflow status with a customer without giving them a full account. Common ask from procurement flow.</t>
         </is>
       </c>
+      <c r="E71" s="119" t="n"/>
+      <c r="F71" s="119" t="n"/>
+      <c r="G71" s="120" t="n"/>
       <c r="H71" s="113" t="inlineStr">
         <is>
           <t>Common for procurement / support tools.</t>
@@ -13467,6 +13894,7 @@
         </is>
       </c>
     </row>
+    <row r="72"/>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="109" t="inlineStr">
         <is>
@@ -13481,6 +13909,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="112" t="inlineStr">
         <is>
@@ -14938,6 +15367,7 @@
         </is>
       </c>
     </row>
+    <row r="107"/>
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="109" t="inlineStr">
         <is>
@@ -14952,6 +15382,7 @@
         </is>
       </c>
     </row>
+    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="112" t="inlineStr">
         <is>
@@ -15013,6 +15444,9 @@
           <t>RBAC-04..11, 14, 15, 16</t>
         </is>
       </c>
+      <c r="F112" s="119" t="n"/>
+      <c r="G112" s="119" t="n"/>
+      <c r="H112" s="120" t="n"/>
       <c r="I112" s="113" t="inlineStr">
         <is>
           <t>100% pass on the matrix. New route = new row in the matrix (enforced by a test that greps for @router decorators).</t>
@@ -15045,6 +15479,9 @@
           <t>RBAC-12, 13</t>
         </is>
       </c>
+      <c r="F113" s="119" t="n"/>
+      <c r="G113" s="119" t="n"/>
+      <c r="H113" s="120" t="n"/>
       <c r="I113" s="113" t="inlineStr">
         <is>
           <t>Test creates user X in tenant A and B, verifies /me/workspaces returns both, /tasks in A does not leak B.</t>
@@ -15077,6 +15514,9 @@
           <t>RBAC-17</t>
         </is>
       </c>
+      <c r="F114" s="119" t="n"/>
+      <c r="G114" s="119" t="n"/>
+      <c r="H114" s="120" t="n"/>
       <c r="I114" s="113" t="inlineStr">
         <is>
           <t>All 3 paths pass.</t>
@@ -15109,6 +15549,9 @@
           <t>RBAC-01</t>
         </is>
       </c>
+      <c r="F115" s="119" t="n"/>
+      <c r="G115" s="119" t="n"/>
+      <c r="H115" s="120" t="n"/>
       <c r="I115" s="113" t="inlineStr">
         <is>
           <t>All 3 cases + rate-limit test.</t>
@@ -15141,6 +15584,9 @@
           <t>RBAC-02, 03</t>
         </is>
       </c>
+      <c r="F116" s="119" t="n"/>
+      <c r="G116" s="119" t="n"/>
+      <c r="H116" s="120" t="n"/>
       <c r="I116" s="113" t="inlineStr">
         <is>
           <t>Bot simulation blocked at expected threshold.</t>
@@ -15173,6 +15619,9 @@
           <t>RBAC-03</t>
         </is>
       </c>
+      <c r="F117" s="119" t="n"/>
+      <c r="G117" s="119" t="n"/>
+      <c r="H117" s="120" t="n"/>
       <c r="I117" s="113" t="inlineStr">
         <is>
           <t>All private ranges blocked.</t>
@@ -15205,6 +15654,9 @@
           <t>RBAC-20</t>
         </is>
       </c>
+      <c r="F118" s="119" t="n"/>
+      <c r="G118" s="119" t="n"/>
+      <c r="H118" s="120" t="n"/>
       <c r="I118" s="113" t="inlineStr">
         <is>
           <t>Random-sampled 20 mutating endpoints all leave audit trails.</t>
@@ -15237,6 +15689,9 @@
           <t>RBAC-21</t>
         </is>
       </c>
+      <c r="F119" s="119" t="n"/>
+      <c r="G119" s="119" t="n"/>
+      <c r="H119" s="120" t="n"/>
       <c r="I119" s="113" t="inlineStr">
         <is>
           <t>All 3 flows pass.</t>
@@ -15269,6 +15724,9 @@
           <t>RBAC-22</t>
         </is>
       </c>
+      <c r="F120" s="119" t="n"/>
+      <c r="G120" s="119" t="n"/>
+      <c r="H120" s="120" t="n"/>
       <c r="I120" s="113" t="inlineStr">
         <is>
           <t>Zero owned entities remain; second call returns 'already deprovisioned' cleanly.</t>
@@ -15301,6 +15759,9 @@
           <t>RBAC-23</t>
         </is>
       </c>
+      <c r="F121" s="119" t="n"/>
+      <c r="G121" s="119" t="n"/>
+      <c r="H121" s="120" t="n"/>
       <c r="I121" s="113" t="inlineStr">
         <is>
           <t>All 4 flows pass.</t>
@@ -15333,6 +15794,9 @@
           <t>RBAC-25</t>
         </is>
       </c>
+      <c r="F122" s="119" t="n"/>
+      <c r="G122" s="119" t="n"/>
+      <c r="H122" s="120" t="n"/>
       <c r="I122" s="113" t="inlineStr">
         <is>
           <t>3 states all pass.</t>
@@ -15365,6 +15829,9 @@
           <t>RBAC-14</t>
         </is>
       </c>
+      <c r="F123" s="119" t="n"/>
+      <c r="G123" s="119" t="n"/>
+      <c r="H123" s="120" t="n"/>
       <c r="I123" s="113" t="inlineStr">
         <is>
           <t>Propagation confirmed on next request.</t>
@@ -15397,12 +15864,16 @@
           <t>RBAC-15</t>
         </is>
       </c>
+      <c r="F124" s="119" t="n"/>
+      <c r="G124" s="119" t="n"/>
+      <c r="H124" s="120" t="n"/>
       <c r="I124" s="113" t="inlineStr">
         <is>
           <t>One denied endpoint + one allowed endpoint confirm behavior.</t>
         </is>
       </c>
     </row>
+    <row r="125"/>
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="109" t="inlineStr">
         <is>
@@ -15417,6 +15888,7 @@
         </is>
       </c>
     </row>
+    <row r="128"/>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="111" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-B done -- RBAC Wave 2 shipped (RBAC-12/13 + 3 follow-ups)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -6170,9 +6170,19 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J66" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -6182,7 +6192,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>Depends on RBAC-13</t>
+          <t>Shipped in FIX-004-B (56399d6). Depends on RBAC-13</t>
         </is>
       </c>
     </row>
@@ -6232,14 +6242,29 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J67" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-B (56399d6). </t>
         </is>
       </c>
     </row>
@@ -7289,7 +7314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9855,9 +9880,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
           <t>Backend is deployed-ready in permissive mode today; frontend fix required before flipping CAPTCHA_REQUIRED=1 in prod.</t>
@@ -9910,9 +9932,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>Sprint 3+ territory when we scale beyond 1 worker per instance.</t>
@@ -9965,12 +9984,241 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
           <t>Current guard is fine for the SME-scale threat model; hardening is nice-to-have.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>FIX-004-B</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 2</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>RBAC-12 + RBAC-13</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Memberships collection + email-per-person (many-to-many user↔tenant)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Big data-model refactor that unblocks every remaining multi-workspace fix. Before: user.tenant_id single FK + users.email globally unique = one email = one person = one workspace forever. After: new memberships collection (user_id, tenant_id, role, permissions, status, invite metadata) with compound unique. users.email still globally unique (one PERSON per email) but that person can belong to N workspaces via N membership rows. Unlocks accountants serving multiple SMEs, founders with 2 businesses, employee invited to 2nd workspace. get_current_user projects role/permissions from CURRENT membership onto user dict — ~430 downstream call sites keep working unchanged (compat layer). Only login + register + user CRUD + invite flow have real logic changes. Bootstrap: 3 new indexes + backfill_memberships_v1 migration (via FIX-002-C ledger). New endpoints: GET /me/workspaces + POST /me/switch-workspace. Login gains optional tenant_id in body; multi-membership + no hint returns ambiguity payload for the frontend picker.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>services/auth/membership.py (new: full service + compat helper); services/auth/__init__.py (exports); core.py (get_current_user resolves membership + projects onto user + legacy fallback); server.py (bootstrap: 3 indexes + backfill migration); routers/auth.py (register creates owner membership + rollback; login ambiguity; /me/workspaces; /me/switch-workspace); routers/team.py (create_user creates membership; update_user mirrors role/perm changes)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>tests/test_memberships_wave2.py — 29 tests (5 create incl. idempotent + reactivate, 2 find + status filter, 2 list-for-user, 3 resolve_login_choices, 2 update, 2 remove soft-delete, 2 project, 1 bootstrap, 1 register+rollback, 2 login flow, 3 workspace endpoints, 2 get_current_user, 2 team mirroring)</t>
+        </is>
+      </c>
+      <c r="H59" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>56399d6</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Blocks-go-live P0. Sprint 2.5 now 5/20 shipped (Waves 1 + 2). Compat layer keeps 349/349 offline regression green — downstream refactor is optional and can happen incrementally. Frontend integration (workspace switcher UI, ambiguity picker on login) is FIX-FUP-25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>FIX-FUP-23</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-B)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>(logged during Wave 2)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>OTP verify: read role from membership directly (not via compat)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Today OTP verify still reads user.role via the get_current_user compat layer projection. Correct behavior, but the code reads clearer if we look up the membership explicitly for role. Small cleanup — trivial once every downstream reader is migrated off user.tenant_id/role.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>server.py verify_otp handler</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>test: OTP verify returns correct role when user has multi-tenant</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Cosmetic; correct behavior today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>FIX-FUP-24</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-B)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>(logged during Wave 2)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Cascade: delete memberships on user delete</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Currently memberships are soft-deleted (status=removed) when a tenant admin removes an employee. There's no path yet to delete the USER (person) — that comes with RBAC-22 (off-boarding wizard) in Wave 4. When we get there, need to decide: delete all their memberships? preserve for audit? Also cascade rules if a TENANT is deleted (currently TENANT_COLLECTIONS wipe should include memberships).</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>routers/admin.py TENANT_COLLECTIONS, routers/team.py user delete path</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>test: tenant delete wipes all memberships for that tenant</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Blocks RBAC-22 off-boarding (Wave 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>FIX-FUP-25</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-B)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>(logged during Wave 2)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Frontend: workspace switcher UI + login ambiguity picker</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Backend is ready. Frontend needs: (a) login page handles the {ambiguous: true, choices: [...]} response and renders a workspace-picker; (b) top-bar workspace switcher calls GET /me/workspaces and POST /me/switch-workspace; (c) invited-user landing UI (post-OTP) if a person now holds multiple memberships. Also update the frontend register form: when a user with an existing email hits /register, show the friendly 'log in first + then Settings &gt; Create Workspace' message.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>frontend/src pages: Login, TopBar, Settings, Register</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>manual: log in as user with 2 memberships, verify picker + switch</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Backend accepts current single-membership frontend unchanged; frontend can ship this incrementally.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-C done -- Wave 3 sub-batch A (RBAC-04..11)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -5714,14 +5714,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J58" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -5771,14 +5786,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J59" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -5828,14 +5858,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J60" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -5885,14 +5930,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J61" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -5942,14 +6002,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J62" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -5999,14 +6074,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J63" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -6056,14 +6146,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J64" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -6113,14 +6218,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J65" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-C (9b3a1c3). </t>
         </is>
       </c>
     </row>
@@ -7314,7 +7434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10103,9 +10223,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
           <t>Cosmetic; correct behavior today.</t>
@@ -10158,9 +10275,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>Blocks RBAC-22 off-boarding (Wave 4).</t>
@@ -10213,12 +10327,76 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
           <t>Backend accepts current single-membership frontend unchanged; frontend can ship this incrementally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>FIX-004-C</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 3 sub-batch A</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>RBAC-04..11 (8 items)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Wave 3 endpoint gates: 8 auth-only endpoints upgraded to role/perm gated</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Closes every 'auth-only endpoint that should be role/perm-gated' finding from the RBAC audit sweep. 8 items in one commit because they share the same testing infrastructure (cross-role permission matrix). RBAC-04 /workflows POST -&gt; require_perm(workflows) [symmetric with DELETE which was already owner]. RBAC-05 /captures/{id}/approve|reject|reassign|clarify -&gt; require_perm(approvals). RBAC-06 /follow-up/run -&gt; require_perm(team_manage). RBAC-07 4 of 17 tasks endpoints upgraded (delete_task role(owner), reassign/delete-plan/prioritize require_perm(team_manage)); other 13 remain auth-only with inline scope checks because widening would break normal workflow. RBAC-08 /meetings + /meetings/text -&gt; require_perm(voice_capture) [matches /voice-notes]. RBAC-09 /leaves approve/reject/request-info -&gt; require_perm(leave_approve) [decorator gate; inline _can_approve_leave stays as defense-in-depth]. RBAC-10 /brain/export -&gt; require_perm(brain_export) [NEW permission key added to config; NOT in _BASE_PERMS so owner-only or explicit grant]. RBAC-11 /memory POST -&gt; require_perm(brain) [read stays open].</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>config.py (brain_export in PERMISSION_KEYS); server.py (create_workflow, 4 captures, followup_run, 2 meetings, add_memory); routers/tasks.py (delete_task, reassign_task, delete_execution_plan, prioritize_tasks + require_role/require_perm imports); routers/team.py (3 leaves endpoints); routers/brain.py (/brain/export)</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>tests/test_rbac_wave3_gates.py — 22 tests (3 config lock-in incl. brain_export not-in-base, 11 per-endpoint dep verification for all 8 RBAC-IDs, 6 cross-role permission matrix incl. owner all-perms + sales/finance defaults + custom role fallback + explicit grant override + brain_export explicit-grant-only, 2 regression on existing gates)</t>
+        </is>
+      </c>
+      <c r="H63" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>9b3a1c3</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 now 13/20 shipped (Waves 1+2 + Wave 3 sub-batch A). Sub-batches B (per-role perm editor + owner exclusion + ROLES fix) and C (pending-invite visibility) remain. Cross-role matrix test is the regression harness — any new endpoint added later must add a matrix row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-D done -- Wave 3 sub-batch B (RBAC-14/15/16)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -6434,9 +6434,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J68" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -6446,7 +6456,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Depends on RBAC-13</t>
+          <t>Shipped in FIX-004-D (f440c33). Depends on RBAC-13</t>
         </is>
       </c>
     </row>
@@ -6496,14 +6506,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J69" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-D (f440c33). </t>
         </is>
       </c>
     </row>
@@ -6553,14 +6578,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J70" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-D (f440c33). </t>
         </is>
       </c>
     </row>
@@ -7434,7 +7474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10397,6 +10437,128 @@
       <c r="M63" t="inlineStr">
         <is>
           <t>Sprint 2.5 now 13/20 shipped (Waves 1+2 + Wave 3 sub-batch A). Sub-batches B (per-role perm editor + owner exclusion + ROLES fix) and C (pending-invite visibility) remain. Cross-role matrix test is the regression harness — any new endpoint added later must add a matrix row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>FIX-004-D</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 3 sub-batch B</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>RBAC-14 + RBAC-15 + RBAC-16</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Role model: per-role permission editor + owner exclusions + production→operations canonical rename</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Wave 2 memberships made these possible; this fix ships them. RBAC-14: tenant.roles[i].permissions[] carries role-level perms. NEW endpoint PATCH /tenant/roles/{key}/permissions (team_manage). user_perms() 5-tier precedence: owner all-minus-exclusions -&gt; user override -&gt; tenant role map -&gt; ROLE_DEFAULT_PERMS -&gt; _BASE_PERMS. Custom roles ('warehouse_manager') can now carry finance/ledger/team_manage etc. without editing each user individually — a role is a policy unit again. RBAC-15: tenant.owner_exclusions:[str] lets a tenant deny specific perms to owner(s). NEW endpoint PUT /tenant/owner-exclusions (owner-only). Backward compat: empty list = classic all-perms owner. Solves 'co-founder with everything except finance visibility'. RBAC-16: canonical role name = 'operations' (matches DEFAULT_ROLES). config.ROLES rewritten. Bootstrap migration rename_production_role_v1 (via FIX-002-C ledger) rewrites tenant.roles[].key + users.role + memberships.role. Idempotent.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>config.py (ROLES canonical); core.py (get_current_user fetches tenant roles + owner_exclusions + populates _role_perms_map/_owner_exclusions on user; user_perms rewritten with 5-tier precedence); server.py (2 new endpoints: PATCH /tenant/roles/{key}/permissions + PUT /tenant/owner-exclusions; bootstrap rename_production_role_v1 migration)</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>tests/test_rbac_wave3_role_model.py — 16 tests (8 per-role perms incl. precedence + endpoint gates, 5 owner exclusions incl. backward compat + PUT semantic + owner-only, 2 canonical rename + migration wiring, 1 get_current_user enrichment)</t>
+        </is>
+      </c>
+      <c r="H64" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>f440c33</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 now 16/20 shipped (Waves 1+2 + Wave 3 A+B). Only Wave 3 sub-batch C (RBAC-17) remains in Wave 3. Frontend Settings UI logged as FIX-FUP-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>FIX-FUP-26</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-D)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>(logged during Wave 3-B)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Frontend Settings UI: per-role permission editor + owner exclusions</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Backend endpoints ship in FIX-004-D. Frontend needs: (a) Team &amp; Roles settings page adds a permission-checkbox matrix per tenant role, POSTs to PATCH /tenant/roles/{key}/permissions; (b) Owner settings page adds an exclusion-checkbox list, PUTs to /tenant/owner-exclusions. Admins can already call the endpoints via curl but the UX story isn't complete until the UI ships.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>frontend/src pages: Settings, Team, Roles</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>manual: edit a role's perms in UI, verify a member's effective perms reflect the change on next request</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Backend is deploy-ready; UI blocks non-technical admin usage.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-E done -- Wave 3 COMPLETE (RBAC-17 pending invite)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -6650,14 +6650,29 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J71" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-E (1541439). </t>
         </is>
       </c>
     </row>
@@ -7474,7 +7489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10553,12 +10568,76 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
           <t>Backend is deploy-ready; UI blocks non-technical admin usage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>FIX-004-E</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 3 sub-batch C</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>RBAC-17</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Pending-invite visibility on GET /users + POST /users/{id}/uninvite</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Small ship that surfaces what Wave 2 already made possible. GET /users now merges membership.status onto each user (pending|active|suspended|removed excluded) + invited_at + accepted_at so admin UI can render a Pending badge. Legacy users without membership rows default to 'active'. NEW endpoint POST /users/{id}/uninvite (team_manage) revokes a pending invite: soft-deletes membership + wipes invite_token on user doc so the invite URL stops resolving. Refuses non-pending targets (use suspend/delete instead). Emits log_activity('user_uninvited').</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>routers/team.py (list_users enrichment + new uninvite_user endpoint)</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>tests/test_rbac_wave3_invite_status.py — 8 tests (3 list enrichment, 5 uninvite gate/refusal/token-invalidation/logging)</t>
+        </is>
+      </c>
+      <c r="H66" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>1541439</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 now 17/20 shipped. RBAC Wave 3 COMPLETE. Remaining: RBAC-18 department scope (Sprint 4), RBAC-19 user groups (Sprint 4), RBAC-30 customer portal (Sprint 5).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-F done -- audit log (RBAC-20)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -6846,14 +6846,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J74" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-F (cc7c698). </t>
         </is>
       </c>
     </row>
@@ -7489,7 +7504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10638,6 +10653,183 @@
       <c r="M66" t="inlineStr">
         <is>
           <t>Sprint 2.5 now 17/20 shipped. RBAC Wave 3 COMPLETE. Remaining: RBAC-18 department scope (Sprint 4), RBAC-19 user groups (Sprint 4), RBAC-30 customer portal (Sprint 5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>FIX-004-F</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 4-A</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>RBAC-20</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Immutable audit log (SOC2/DPDP/GDPR compliance)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>New services/audit_log.py: append-only, best-effort record() + tenant-scoped query() + context_from() request/user extractor. Fail-open by design — Mongo hiccup during audit write must not fail user action. NEVER raises. 35 canonical action names in ACTIONS registry for review-time typo catch. Bootstrap creates 3 indexes: (tenant_id, ts DESC), (actor_id, ts DESC), (tenant_id, entity_type, entity_id). NO TTL (rows live forever for compliance). NO PATCH/DELETE endpoints — API-layer append-only; tampering requires DB access. GET /admin/audit-log endpoint (owner-only) supports action/actor_id/entity_type/entity_id/since_ts/before_ts filters + limit (capped 500) + cursor paging. High-value events wired to record() this ship: login_success + login_failure (captures attempted email on unknown user), logout (records even on invalid token), tenant_created + user_created on register, owner_exclusions_updated with before/after diff. Expanding call-site coverage to user_deleted / role_deleted / decision_approved / etc. logged as FIX-FUP-27 — 3-line change per event, non-blocker.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>services/audit_log.py (new); server.py (bootstrap: 3 indexes + GET /admin/audit-log endpoint + owner_exclusions audit wire); routers/auth.py (login success + failure audit, logout audit, register tenant+user audit)</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>tests/test_audit_log.py — 24 tests (5 record contract incl. fail-open + string caps, 6 query contract incl. tenant isolation + paging, 4 context_from variants, 1 bootstrap, 3 endpoint incl. no-PATCH/DELETE guard, 5 wire-up on login/logout/register/owner-exclusions)</t>
+        </is>
+      </c>
+      <c r="H67" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>cc7c698</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 now 18/20 shipped. Wave 4 sub-batch 1/3 done — sub-batches G (session mgmt UI, RBAC-21) and H (off-boarding wizard, RBAC-22) remain. Blocks-go-live P0 requirement for SOC 2 / DPDP compliance now met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>FIX-FUP-27</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-F)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>(logged during Wave 4-A)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Expand audit_log.record() call-site coverage across mutating events</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Wave 4-A ships the audit-log service + 4 high-value event call sites (login, logout, register, owner-exclusions). Progressive coverage needed on the rest of the ACTIONS registry: user_deleted, user_uninvited, role_deleted, role_permissions_updated, decision_approved/rejected, capture_approved/rejected, workflow_deleted, task_deleted, tenant_deleted (from admin.py), platform_admin_tenant_wipe, ai_key_updated. Each is a 3-line change: audit_log.context_from(request, user) + await record(db, action='...', entity_type='...', entity_id='...', before/after, **ctx). Non-blocker — infra is ready, incremental fill-in.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>routers/admin.py, routers/team.py, routers/decisions.py, routers/tasks.py, server.py</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>test: each new call site verified via grep + one integration assertion per event</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>Post-FIX-004-F incremental. Ship as batches of 3-4 events per commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>FIX-FUP-28</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-F)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>(logged during Wave 4-A)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Audit log retention policy (TTL + off-hot-storage archive)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Currently audit_log has NO TTL — rows live forever. Compliance regimes (SOC 2, DPDP) require min retention (12-24 months typically) but max retention is a business decision (privacy vs forensics tradeoff). Also: hot Mongo isn't the cheapest place to keep 5-year audit history. Plan an archive path: TTL on hot rows + cold storage (S3 / obj_store) for archived tail. Blocks nothing today; revisit before we sell to a customer whose contract requires a retention SLA.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>services/audit_log.py + scheduler job + obj_store integration</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>test: TTL wipes rows past retention window; archive job moves them intact</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>Sprint 5 (DevOps + compliance) territory.</t>
         </is>
       </c>
     </row>
@@ -16746,6 +16938,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="85" t="inlineStr">
         <is>
@@ -17230,6 +17423,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-G done -- session mgmt UI (RBAC-21)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -6918,14 +6918,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J75" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-004-G (d95ae44). </t>
         </is>
       </c>
     </row>
@@ -7504,7 +7519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10769,9 +10784,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
           <t>Post-FIX-004-F incremental. Ship as batches of 3-4 events per commit.</t>
@@ -10824,12 +10836,131 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
           <t>Sprint 5 (DevOps + compliance) territory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>FIX-004-G</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 4-B</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>RBAC-21</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Session-management UI (/me/sessions list + revoke by device)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>New services/auth/session_tracking.py extends the FIX-003-C revocation infra with device metadata (ua, ip, last_seen_at). NEW active_sessions collection with jti unique index + user_id/created_at index + exp TTL for auto-purge. record_session/touch_session/list_sessions/revoke_one_session/revoke_all_sessions_for_user (with tenant_id + keep_jti knobs). get_current_user gained touch_session call so /me/sessions shows accurate last-seen. login + register + switch-workspace all record the new jti. 3 new endpoints: GET /me/sessions (marks current session), DELETE /me/sessions/{jti} (ownership-guarded), DELETE /me/sessions (revoke all except current).</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>services/auth/session_tracking.py (new); services/auth/__init__.py (exports); core.py (get_current_user calls touch_session); server.py (bootstrap: 3 active_sessions indexes); routers/auth.py (login + register + switch-workspace record + 3 new endpoints)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>tests/test_session_mgmt.py — 20 tests (4 record contract incl. fail-open + UA cap, 3 list incl. user isolation + tenant filter, 3 revoke_one incl. ownership guard, 2 revoke_all incl. keep_jti + tenant filter, 1 bootstrap indexes, 3 endpoint source guards, 1 get_current_user touch, 3 wire-up on login/register/switch)</t>
+        </is>
+      </c>
+      <c r="H70" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>d95ae44</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>Sprint 2.5: 19/20. Only RBAC-22 (off-boarding wizard) left. Backend done — frontend /settings/sessions UI logged as FIX-FUP-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>FIX-FUP-29</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-G)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>(logged during Wave 4-B)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Frontend Settings &gt; Sessions UI</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Backend ships GET/DELETE /me/sessions + DELETE /me/sessions/{jti}. Frontend needs Settings page listing sessions with UA/IP/last-seen + revoke buttons (individual + 'sign out other devices'). Row for current session should be marked distinct (grey out revoke).</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>frontend/src pages: Settings/Sessions</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>manual: log in on 2 devices, revoke the other from device 1, verify device 2 401s</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>Backend deploy-ready; UI blocks user self-serve session control.</t>
         </is>
       </c>
     </row>
@@ -16938,7 +17069,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="85" t="inlineStr">
         <is>
@@ -17423,7 +17553,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tracker): FIX-004-H done -- RBAC Wave 4 COMPLETE (RBAC-22 off-boarding)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -6990,9 +6990,19 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J76" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -7002,7 +7012,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>Depends on RBAC-21</t>
+          <t>Shipped in FIX-004-H (309ef84). Depends on RBAC-21</t>
         </is>
       </c>
     </row>
@@ -7519,7 +7529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10955,12 +10965,241 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
           <t>Backend deploy-ready; UI blocks user self-serve session control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>FIX-004-H</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sprint 2.5 / RBAC Wave 4-C</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>RBAC-22</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Off-boarding wizard (deprovisioning) — RBAC Wave 4 COMPLETE</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>New services/deprovisioning.py orchestrates 6 idempotent steps into one call: last-owner guard + tenant-scoped session revoke + soft-remove membership + invalidate invite_token + reassign owned tasks + reassign authored contacts + audit_log entry. New endpoint POST /users/{id}/deprovision {reassign_to_user_id?} — owner-only. Self-deprovision refused. Replacement user validated as LIVE member. Returns per-step report for UI confirmation. Session revoke is TENANT-SCOPED — a user's sessions in other tenants they belong to survive. Task reassignment updates denormalized assignee_role. No reassign target = null the fields.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>services/deprovisioning.py (new); routers/team.py (new POST /users/{id}/deprovision endpoint + DeprovisionInput model + BaseModel import)</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>tests/test_deprovisioning.py — 11 tests (2 fresh full-run with + without replacement, 1 idempotent, 2 last-owner guard, 1 tenant scoping, 1 audit entry, 4 endpoint gates)</t>
+        </is>
+      </c>
+      <c r="H72" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>309ef84</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>RBAC WAVE 4 COMPLETE — 3/3 sub-batches shipped (F+G+H). Sprint 2.5 now 20/20. Full RBAC roadmap Waves 1-4 COMPLETE — 20 of 30 audit items shipped. Remaining 10 are Sprint 4/5 items: RBAC-18 (department scope), RBAC-19 (user groups), RBAC-23..28 (2FA, ownership transfer, DPDP consent, delegation, time-bounded perms, SSO, API keys), RBAC-30 (customer portal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>FIX-FUP-30</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-H)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>(logged during Wave 4-C)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Ownership transfer wizard (owner-to-owner)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Deprovisioning's last-owner guard is correct behavior — it blocks removing the only owner. But it leaves no path out. Need a separate 'transfer ownership' flow: promote another member to owner, then optionally deprovision the previous owner. 2FA confirmation recommended for the promoting owner.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>new endpoint POST /tenant/transfer-ownership + service</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>test: two-owner state achieved, previous owner deprovisions cleanly</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>RBAC-24 in the audit — Sprint 3 territory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>FIX-FUP-31</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-H)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>(logged during Wave 4-C)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Cascade decisions in deprovision</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Today deprovision reassigns tasks + contacts but NOT decisions where created_by = target. Small addition — same pattern as tasks. Decision-approver relationships also worth considering: if target was designated approver for pending decisions, they need routing to the replacement.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>services/deprovisioning.py</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>test: fresh deprovision reassigns created_by decisions + approver_id decisions</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Incremental improvement on FIX-004-H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>FIX-FUP-32</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-004-H)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>(logged during Wave 4-C)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Frontend off-boarding wizard UI</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Backend done. Frontend needs: Team &gt; Member detail page adds 'Remove from workspace' button that opens a wizard: pick replacement member (dropdown of live members), preview count of items to reassign, confirm modal, POST /users/{id}/deprovision, show report summary.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>frontend/src pages: Team/MemberDetail, Team/OffboardWizard</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>manual: off-board a test member, verify counts match backend report</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>Backend deploy-ready via curl.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-005-A done -- S3-02 plan fields + S3-03 per-tenant AI keys
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -4034,20 +4034,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J31" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J31" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K31" s="103" t="inlineStr"/>
-      <c r="L31" s="103" t="inlineStr"/>
-      <c r="M31" s="103" t="inlineStr"/>
+      <c r="L31" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M31" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N31" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O31" s="22" t="inlineStr"/>
+      <c r="O31" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-005-A (afbf9b8). </t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="103" t="inlineStr">
@@ -4095,20 +4107,32 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J32" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J32" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K32" s="103" t="inlineStr"/>
-      <c r="L32" s="103" t="inlineStr"/>
-      <c r="M32" s="103" t="inlineStr"/>
+      <c r="L32" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M32" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N32" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O32" s="22" t="inlineStr"/>
+      <c r="O32" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-005-A (afbf9b8). </t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="103" t="inlineStr">
@@ -7529,7 +7553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11084,9 +11108,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
           <t>RBAC-24 in the audit — Sprint 3 territory.</t>
@@ -11139,9 +11160,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
           <t>Incremental improvement on FIX-004-H.</t>
@@ -11194,12 +11212,186 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
           <t>Backend deploy-ready via curl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>FIX-005-A</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Sprint 3 / Billing + AI Keys</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>S3-02 + S3-03</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Plan/entitlement fields + per-tenant AI keys</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Two Sprint 3 items shipped together — both pure data-model + resolver changes, no external integration. S3-02: services/plans.py with 5 plans (trial/starter/business/enterprise/grandfathered), each carries seat_limit + quotas (llm_tokens/stt_minutes/storage/brain_docs) + features (whatsapp/sso/api_keys). effective_plan(tenant) merges base + tenant overrides. new_tenant_plan_fields() called in register for trial+14d. enforce_seat_limit raises 402 with upgrade prompt. Bootstrap migration backfill_grandfathered_plans_v1 marks pre-plan tenants — same generous shape as business, retained forever, zero user-visible change. team.py create_user calls enforce_seat_limit BEFORE any writes. S3-03: services/tenant_ai_keys.py resolves keys with precedence tenant-&gt;platform-&gt;none. 3 owner-only endpoints on /tenant/ai-keys (GET list with masked previews, PUT replace map with audit_log per-provider-change rotation events, DELETE revert to platform pool). Never logs the raw key value — regression-guarded in tests.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>services/plans.py (new: plan model + effective_plan + enforce_seat_limit); services/tenant_ai_keys.py (new: resolve_ai_key + normalize + summarize); server.py (GET /tenant/plan + 3 /tenant/ai-keys endpoints + backfill migration); routers/auth.py (register initializes plan fields via new_tenant_plan_fields); routers/team.py (create_user enforces seat limit)</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>tests/test_plans_and_ai_keys.py — 38 tests (7 effective_plan, 3 trial expiry, 3 has_feature, 1 defaults, 3 enforce_seat_limit, 1 register wire, 1 bootstrap migration, 5 resolve_ai_key precedence, 2 source, 3 normalize, 1 no-secret-leak, 4 endpoint gates, 3 PUT audit + no-leak guard, 1 delete revert, 1 seat-limit BEFORE-insert order)</t>
+        </is>
+      </c>
+      <c r="H76" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>afbf9b8</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Sprint 3: 2/5 shipped (+ 3 RBAC items TBD). Billing provider = Razorpay (India-primary). S3-01 deferred until we're ready for external integration. Follow-ups: FIX-FUP-33 (secrets manager for ai_keys), FIX-FUP-34 (provider outage transparent fallback).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>FIX-FUP-33</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-A)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>(logged during S3-03)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Move tenant.ai_keys to a real secrets manager</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>tenant.ai_keys stored plain-text in Mongo. Fine for MVP, red flag on a security review. Move to AWS Secrets Manager / HashiCorp Vault / Cloudflare Secrets Store. Wrap services/tenant_ai_keys.resolve_ai_key to fetch from the secrets manager instead of the tenant doc; keep the current in-doc storage as a fallback during migration.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>services/tenant_ai_keys.py + new services/secrets_manager.py</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>test: rotate key in secrets manager, verify resolve returns new value on next call</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>Sprint 5 (DevOps/security). Blocks enterprise-tier sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>FIX-FUP-34</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-A)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>(logged during S3-03)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>AI provider outage transparent fallback (tenant key -&gt; platform)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>When a tenant's key returns 429/500, transparently fall back to the platform pool for that request + notify the tenant. Improves reliability without exposing platform quota to abuse (rate-limit the fallback to a low ceiling per tenant/hr).</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>core.py LLM wrappers + services/tenant_ai_keys.py</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>test: mock 429 on tenant key, verify fallback + notification + rate-limit on fallback</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>Depends on RBAC-23 (2FA) being live so admin can rotate the key confidently after an outage.</t>
         </is>
       </c>
     </row>
@@ -11285,6 +11477,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -11380,9 +11573,9 @@
 (Tenancy/Data)</t>
         </is>
       </c>
-      <c r="D6" s="55" t="inlineStr">
-        <is>
-          <t>[S3-02] Add plan / entitlement fields to tenant doc
+      <c r="D6" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S3-02] Add plan / entitlement fields to tenant doc
 (Billing/AI-Keys)</t>
         </is>
       </c>
@@ -11418,9 +11611,9 @@
 (Tenancy/Data)</t>
         </is>
       </c>
-      <c r="D7" s="54" t="inlineStr">
-        <is>
-          <t>[S3-03] Per-tenant AI key resolver
+      <c r="D7" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S3-03] Per-tenant AI key resolver
 (Billing/AI-Keys)</t>
         </is>
       </c>
@@ -11665,6 +11858,8 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="57" t="inlineStr">
         <is>
@@ -13148,7 +13343,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="109" t="inlineStr">
         <is>
@@ -13156,7 +13350,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="111" t="inlineStr">
         <is>
@@ -13444,7 +13637,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="111" t="inlineStr">
         <is>
@@ -13697,7 +13889,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="111" t="inlineStr">
         <is>
@@ -13845,7 +14036,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="109" t="inlineStr">
         <is>
@@ -13860,7 +14050,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="111" t="inlineStr">
         <is>
@@ -14336,7 +14525,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="111" t="inlineStr">
         <is>
@@ -14695,7 +14883,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="111" t="inlineStr">
         <is>
@@ -15123,7 +15310,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="109" t="inlineStr">
         <is>
@@ -15138,7 +15324,6 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="112" t="inlineStr">
         <is>
@@ -16596,7 +16781,6 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="109" t="inlineStr">
         <is>
@@ -16611,7 +16795,6 @@
         </is>
       </c>
     </row>
-    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="112" t="inlineStr">
         <is>
@@ -17102,7 +17285,6 @@
         </is>
       </c>
     </row>
-    <row r="125"/>
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="109" t="inlineStr">
         <is>
@@ -17117,7 +17299,6 @@
         </is>
       </c>
     </row>
-    <row r="128"/>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="111" t="inlineStr">
         <is>
@@ -17308,6 +17489,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="85" t="inlineStr">
         <is>
@@ -17563,12 +17745,12 @@
       </c>
       <c r="C15" s="92" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="D15" s="88" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+          <t>Sprint 3 | FIX-005-A (afbf9b8) — services/tenant_ai_keys.resolve_ai_key + services/plans.py</t>
+        </is>
+      </c>
+      <c r="D15" s="104" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -17585,12 +17767,12 @@
       </c>
       <c r="C16" s="92" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="D16" s="88" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+          <t>Sprint 3 | FIX-005-A (afbf9b8) — services/tenant_ai_keys.resolve_ai_key + services/plans.py</t>
+        </is>
+      </c>
+      <c r="D16" s="104" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -17792,6 +17974,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tracker): FIX-005-B done -- S3-04 usage quotas
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -4180,20 +4180,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J33" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J33" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K33" s="103" t="inlineStr"/>
-      <c r="L33" s="103" t="inlineStr"/>
-      <c r="M33" s="103" t="inlineStr"/>
+      <c r="L33" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M33" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="N33" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O33" s="22" t="inlineStr"/>
+      <c r="O33" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-005-B (29d2238). </t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="103" t="inlineStr">
@@ -7553,7 +7565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M78"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11331,9 +11343,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
           <t>Sprint 5 (DevOps/security). Blocks enterprise-tier sales.</t>
@@ -11386,12 +11395,131 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
           <t>Depends on RBAC-23 (2FA) being live so admin can rotate the key confidently after an outage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>FIX-005-B</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Sprint 3 / Usage Quotas</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>S3-04</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Usage-quota enforcement (402 on exceed)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>New services/quotas.py: check_quota reads current-month usage_events aggregation, compares to plan cap from FIX-005-A. cost param lets caller pre-block a request that would push over. Fail-open on Mongo blip — quota infra failure never blocks AI. 4 resources: llm_tokens_total (sums usage_events.tokens_total), stt_minutes (sums usage_events.units where unit_type=minutes), storage_bytes (sums files.size), brain_docs (counts brain_documents). Aggregation window = current UTC calendar month, resets on 1st. guarded_llm now reads _ctx_tenant contextvar and enforces quota BEFORE taking semaphore slot — raises HTTPException(402) with structured detail {code, resource, message, usage, cap, plan}. NEW skip_quota_check kwarg bypasses check for admin key-probe (would be user-hostile). GET /tenant/usage returns every quota with usage/cap/percent/over — powers frontend dashboard.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>services/quotas.py (new); services/ai/llm_limits.py (guarded_llm quota check + skip_quota_check kwarg); server.py (GET /tenant/usage endpoint); routers/admin.py (probe passes skip_quota_check=True)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>tests/test_quotas.py — 16 tests (6 check_quota incl. unlimited/under/over/cost-projection/last-month/tenant-isolation, 2 storage + brain_docs sources, 2 status shape, 1 status_all row-per-quota, 4 guarded_llm wiring incl. fail-open, 1 endpoint)</t>
+        </is>
+      </c>
+      <c r="H79" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>29d2238</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Sprint 3: 3/5 shipped (S3-02, S3-03, S3-04). Only S3-01 (Razorpay billing, deferred) + 3 RBAC items (23/24/25) remain. FIX-FUP-35 logged for soft-limit warning emails (75/90/100% thresholds).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>FIX-FUP-35</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-B)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>(logged during S3-04)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Soft-limit warning emails at 75/90/100% quota thresholds</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Backend reports percent + over flag via quota_status. A scheduler task should sweep daily, compare current percent to previously-notified threshold on tenant (persist last_notified_thresholds dict), and send an email at each crossing so tenants hit the cap with warning not surprise. Templates in services/auth_emails.py.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>new services/quota_alerts.py + scheduler hook</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>test: 75% threshold triggers email once, subsequent runs don't re-send unless dropped + re-crossed</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Post-Wave-5 polish; not go-live blocker but big UX improvement.</t>
         </is>
       </c>
     </row>
@@ -11649,9 +11777,9 @@
 (Tenancy/Data)</t>
         </is>
       </c>
-      <c r="D8" s="55" t="inlineStr">
-        <is>
-          <t>[S3-04] Enforce usage quotas (402 on exceed)
+      <c r="D8" s="108" t="inlineStr">
+        <is>
+          <t>[DONE][S3-04] Enforce usage quotas (402 on exceed)
 (Billing/AI-Keys)</t>
         </is>
       </c>
@@ -17745,7 +17873,7 @@
       </c>
       <c r="C15" s="92" t="inlineStr">
         <is>
-          <t>Sprint 3 | FIX-005-A (afbf9b8) — services/tenant_ai_keys.resolve_ai_key + services/plans.py</t>
+          <t>Sprint 3 | FIX-005-A (afbf9b8) — services/tenant_ai_keys.resolve_ai_key + services/plans.py | FIX-005-B (29d2238) — services/quotas.py + guarded_llm enforcement + /tenant/usage endpoint</t>
         </is>
       </c>
       <c r="D15" s="104" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): FIX-005-C done -- RBAC-25 DPDP consent tracking
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -7217,14 +7217,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J79" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-005-C (4115624). </t>
         </is>
       </c>
     </row>
@@ -7565,7 +7580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11514,12 +11529,186 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
           <t>Post-Wave-5 polish; not go-live blocker but big UX improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>FIX-005-C</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Sprint 3 / Compliance</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>RBAC-25</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>DPDP AI-consent tracking (India-mandatory)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>New services/ai_consent.py: tenant.ai_consent = {granted_at, granted_by_user_id, granted_by_email, ip, ua, version, revoked_at}. CURRENT_CONSENT_VERSION='1.0' — bump when scope changes, tenants must re-consent. has_active_consent hot-path reader. consent_status frontend shape deliberately OMITS IP/UA (audit-only). needs_reconsent flag for version-drift. require_ai_consent raises HTTPException(451 'Unavailable For Legal Reasons') with structured detail — frontend maps to consent modal. 3 endpoints: GET (any user, banner state), POST (owner grants + captures IP/UA/UA/version), DELETE (owner flips revoked_at + preserves grant history). Both mutations emit audit_log rows. Enforcement wired at guarded_llm BEFORE quota check — single tenants.find_one reused for both consent + plan-quota reads (no double round-trip). Fail-open on Mongo blip, skip_quota_check bypasses (admin probe).</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>services/ai_consent.py (new: has_active_consent + require_ai_consent + build_grant/revoke + consent_status); services/ai/llm_limits.py (guarded_llm calls require_ai_consent BEFORE quota check, reuses tenant fetch); server.py (3 /tenant/ai-consent endpoints + AiConsentGrantInput model)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>tests/test_ai_consent.py — 23 tests (5 has_active_consent state matrix, 3 consent_status incl. no-IP-leak, 3 require_ai_consent, 2 build_grant, 1 build_revoke, 7 endpoint gates + audit emission, 2 guarded_llm gate + fetch reuse)</t>
+        </is>
+      </c>
+      <c r="H81" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>4115624</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Sprint 3: 4/5 shipped. India DPDP-blocker closed. FIX-005-D (RBAC-23 2FA + RBAC-24 ownership transfer) next — the two go together since transfer needs 2FA confirm. S3-01 (Razorpay billing) deferred. FIX-FUP-36 (email nudge on version bump) + FIX-FUP-37 (extend gate to STT/vision) logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>FIX-FUP-36</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-C)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>(logged during RBAC-25)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Consent-doc versioning UX: email nudge on version bump</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>When CURRENT_CONSENT_VERSION bumps, consent_status flags needs_reconsent=True but nothing emails the owner. Add scheduler task that sweeps tenants where ai_consent.version &lt; CURRENT and sends a re-consent email once per version bump. Suppress duplicate sends via last_reconsent_notified_version on tenant doc.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>new services/consent_alerts.py + scheduler hook + services/auth_emails.py template</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>test: bump version, sweep sends email once per tenant, not on subsequent sweeps</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>Non-blocker; adds compliance smoothness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>FIX-FUP-37</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-C)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>(logged during RBAC-25)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Extend AI consent gate to non-LLM paths (Sarvam STT/TTS + Gemini vision)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>guarded_llm is the choke point for LLM calls but Sarvam STT/TTS (server.py transcribe_audio_full, signup /tts /stt) and Gemini vision calls (services/tasks OCR paths) don't route through it. Extend the consent check to those code paths so all AI processing is uniformly gated.</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>server.py transcribe_audio_full + routers/signup.py tts/stt + Gemini vision call sites</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>test: STT call without consent returns 451; consented STT returns 200</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Compliance completeness — DPDP considers STT + vision as AI processing too.</t>
         </is>
       </c>
     </row>
@@ -11605,7 +11794,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -11986,8 +12174,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="57" t="inlineStr">
         <is>
@@ -13471,6 +13657,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="109" t="inlineStr">
         <is>
@@ -13478,6 +13665,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="111" t="inlineStr">
         <is>
@@ -13765,6 +13953,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="111" t="inlineStr">
         <is>
@@ -14017,6 +14206,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="111" t="inlineStr">
         <is>
@@ -14164,6 +14354,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="109" t="inlineStr">
         <is>
@@ -14178,6 +14369,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="111" t="inlineStr">
         <is>
@@ -14653,6 +14845,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="111" t="inlineStr">
         <is>
@@ -15011,6 +15204,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="111" t="inlineStr">
         <is>
@@ -15438,6 +15632,7 @@
         </is>
       </c>
     </row>
+    <row r="72"/>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="109" t="inlineStr">
         <is>
@@ -15452,6 +15647,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="112" t="inlineStr">
         <is>
@@ -16909,6 +17105,7 @@
         </is>
       </c>
     </row>
+    <row r="107"/>
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="109" t="inlineStr">
         <is>
@@ -16923,6 +17120,7 @@
         </is>
       </c>
     </row>
+    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="112" t="inlineStr">
         <is>
@@ -17413,6 +17611,7 @@
         </is>
       </c>
     </row>
+    <row r="125"/>
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="109" t="inlineStr">
         <is>
@@ -17427,6 +17626,7 @@
         </is>
       </c>
     </row>
+    <row r="128"/>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="111" t="inlineStr">
         <is>
@@ -17617,7 +17817,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="85" t="inlineStr">
         <is>
@@ -18102,7 +18301,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tracker): FIX-005-D done -- Sprint 3 COMPLETE (minus S3-01 Razorpay)
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -7098,14 +7098,29 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J77" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-005-D (a8da19b). </t>
         </is>
       </c>
     </row>
@@ -7155,9 +7170,19 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J78" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -7167,7 +7192,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>Depends on RBAC-13</t>
+          <t>Shipped in FIX-005-D (a8da19b). Depends on RBAC-13</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M83"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11648,9 +11673,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
           <t>Non-blocker; adds compliance smoothness.</t>
@@ -11703,12 +11725,241 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
           <t>Compliance completeness — DPDP considers STT + vision as AI processing too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>FIX-005-D</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Sprint 3 / Security + Auth</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>RBAC-23 + RBAC-24</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>TOTP 2FA + tenant ownership transfer</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>RBAC-23: pyotp-based TOTP flow. services/auth/totp.py: begin_enrollment (secret + provisioning URI for QR), confirm_enrollment (verify pending + generate 10 bcrypt-hashed backup codes returned once), verify_totp (valid_window=1 = 30s drift), consume_backup_code (single-use), disable_totp, regenerate_backup_codes (requires current TOTP not backup). 5 endpoints on /auth/2fa: enroll, confirm, verify-login, disable, regenerate-backup-codes. All emit audit_log events (two_factor_enabled/success/failure/disabled/backup_regenerated/challenge_issued). Login flow: when user.two_factor.enabled_secret set, /login returns {two_factor_required:True, challenge_token} instead of session JWT. 5-min challenge JWT encodes {sub, tenant_id, role, type=2fa_challenge}. Client calls /2fa/verify-login with challenge+code. RBAC-24: POST /auth/tenant/transfer-ownership. Owner-only inline check. Refuses self-transfer + validates target is live member. If caller has 2FA enabled, MUST supply totp_code (prevents session-theft workspace seizure); non-2FA callers still allowed but audit marks two_fa_used=false. Atomic promote+demote in memberships (target-&gt;owner, caller-&gt;sales safe default). Legacy user.role fields synced too. Audits tenant_ownership_transferred with before/after {owner_id}.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>services/auth/totp.py (new: pyotp-based TOTP + bcrypt-hashed backup codes); services/auth/__init__.py (exports); routers/auth.py (5 2FA endpoints + transfer-ownership + login 2FA gate + _mint_challenge/_decode_challenge helpers + 4 input models); requirements.txt (pyotp==2.10.0)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>tests/test_totp_and_ownership.py — 26 tests (3 enrollment flow, 4 backup codes incl. regen invalidates, 1 disable wipes, 3 is_enabled state, 2 login challenge shape, 2 challenge token roundtrip + type-guard, 5 endpoint guards, 6 ownership transfer incl. self-refuse + live-member validation + 2FA gate + atomic swap + audit)</t>
+        </is>
+      </c>
+      <c r="H84" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>a8da19b</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>SPRINT 3 COMPLETE (minus S3-01 Razorpay billing, deferred). 5/5 backlog items shipped this sprint: S3-02, S3-03, S3-04 + RBAC-23, RBAC-24, RBAC-25. 3 follow-ups logged: SMS 2FA fallback (FIX-FUP-38), tenant-level enforce-2FA policy (FIX-FUP-39), Razorpay subscription rebind on transfer (FIX-FUP-40).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>FIX-FUP-38</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-D)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 3)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>SMS 2FA fallback + WhatsApp OTP fallback</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Many Indian SME employees don't use authenticator apps. Add SMS-OTP as an alternative second factor (integrate Twilio + Razorpay MSG91 or Sarvam) and/or a WhatsApp OTP path (we already have WA infra from FIX-002-A). Same user.two_factor storage, new services/auth/sms_2fa.py.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>services/auth/* + relevant routers</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>test: integration with the new provider / policy</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>Post-Sprint 3 improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>FIX-FUP-39</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-D)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 3)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Tenant-level enforce-2FA policy</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Add tenant.security_policy.require_2fa_for_owners (bool) + require_2fa_for_admins. When set, login for a matching role refuses to complete without 2FA enrolled first — user is prompted to enroll before session issued. Enterprise-grade compliance ask.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>services/auth/* + relevant routers</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>test: integration with the new provider / policy</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>Post-Sprint 3 improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>FIX-FUP-40</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-005-D)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 3)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Razorpay subscription rebind on ownership transfer</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Ownership transfer currently changes DB state only. When S3-01 lands (Razorpay integration), the transfer must also re-point the subscription billing contact to the new owner. Coupled with S3-01.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>services/auth/* + relevant routers</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>test: integration with the new provider / policy</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Post-Sprint 3 improvement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-006-A done -- Sprint 0 batch A (S0-01/08/09/10)
Auth credential hardening: 4 launch-blockers shipped in c57b550.
Task Backlog rows for S0-01/08/09/10 marked Done. Fix Log entry
FIX-006-A appended.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -2053,20 +2053,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J2" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J2" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K2" s="103" t="inlineStr"/>
-      <c r="L2" s="103" t="inlineStr"/>
-      <c r="M2" s="103" t="inlineStr"/>
+      <c r="L2" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="M2" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="N2" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O2" s="22" t="inlineStr"/>
+      <c r="O2" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-A (c57b550). </t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="103" t="inlineStr">
@@ -2480,20 +2492,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J9" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J9" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K9" s="103" t="inlineStr"/>
-      <c r="L9" s="103" t="inlineStr"/>
-      <c r="M9" s="103" t="inlineStr"/>
+      <c r="L9" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="M9" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="N9" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O9" s="22" t="inlineStr"/>
+      <c r="O9" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-A (c57b550). </t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="103" t="inlineStr">
@@ -2541,20 +2565,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J10" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J10" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K10" s="103" t="inlineStr"/>
-      <c r="L10" s="103" t="inlineStr"/>
-      <c r="M10" s="103" t="inlineStr"/>
+      <c r="L10" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="M10" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="N10" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O10" s="22" t="inlineStr"/>
+      <c r="O10" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-A (c57b550). </t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="103" t="inlineStr">
@@ -2602,20 +2638,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J11" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J11" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K11" s="103" t="inlineStr"/>
-      <c r="L11" s="103" t="inlineStr"/>
-      <c r="M11" s="103" t="inlineStr"/>
+      <c r="L11" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="M11" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="N11" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O11" s="22" t="inlineStr"/>
+      <c r="O11" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-A (c57b550). </t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="103" t="inlineStr">
@@ -7605,7 +7653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11844,9 +11892,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
           <t>Post-Sprint 3 improvement.</t>
@@ -11899,9 +11944,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
           <t>Post-Sprint 3 improvement.</t>
@@ -11954,12 +11996,76 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
           <t>Post-Sprint 3 improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>FIX-006-A</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Sprint 0 / Security P0</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>S0-01 + S0-08 + S0-09 + S0-10</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Auth credential hardening (4 launch-blockers)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>S0-01: seed_platform_admin no longer ships hardcoded default creds. Prod (ENV=prod) refuses to boot when SUPERADMIN_EMAIL/PASSWORD missing. Existing admin hash is NEVER overwritten on restart -- refresh path requires an explicit SUPERADMIN_ALLOW_HASH_REFRESH=1 one-off flag. S0-08: login / register / switch-workspace / 2fa-verify-login / admin-login / OTP-verify (6 sites) no longer include the raw JWT in the JSON body when AUTH_RETURN_TOKEN is off. HttpOnly cookie is the source of truth. Env defaults: off in prod, on elsewhere. New login_response() helper centralises the shape. S0-09: Platform-admin tokens now signed + verified with PLATFORM_ADMIN_JWT_SECRET (falls back to JWT_SECRET when unset for dev back-compat). A compromise of the tenant JWT_SECRET can no longer forge platform-admin sessions. type='platform_admin' claim remains as second gate either way. S0-10: verify_otp invalidates invite_token + expiry on successful accept, so the invite link stops resolving on /auth/invite/{token} (no more leaked name / masked phone) and a second /auth/invite/{token}/start can't bomb the invitee's phone with fresh SMS OTPs. Records invite_consumed_at for the paper trail.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>config.py (PLATFORM_ADMIN_JWT_SECRET, AUTH_RETURN_TOKEN, SUPERADMIN_ALLOW_HASH_REFRESH env plumbing + env-driven defaults); core.py (create_admin_token + get_platform_admin use admin secret; new login_response() helper); server.py (seed_platform_admin prod refuse + no-silent-refresh + verify_otp invite invalidation + login_response wiring; login_response import); routers/auth.py (register + login + switch-workspace + 2fa-verify-login all route through login_response); routers/admin.py (admin_login routes through login_response)</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>tests/test_auth_hardening.py -- 23 tests: 4 login_response helper (flag on/off/kwargs/no-shared-state); 5 AUTH_RETURN_TOKEN env semantics (prod default off, dev default on, explicit overrides, truthy/falsy accepted); 4 platform-admin secret split (fallback, distinct, admin verifies with admin secret, tenant secret cannot forge admin); 6 seed_platform_admin (prod refuses, dev fallback, env creds, hash NOT overwritten by default, opt-in refreshes, opt-in noop when password matches); 2 invite invalidation source-inspection guards; 2 no-raw-token endpoint guards (grep-style regression backstop)</t>
+        </is>
+      </c>
+      <c r="H88" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>c57b550</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Sprint 0 batch A. 4 launch-blockers shipped together. 337 pre-existing auth/RBAC/session/plans/consent/totp tests still green (zero regressions). Deployment note for ops: set PLATFORM_ADMIN_JWT_SECRET + SUPERADMIN_EMAIL + SUPERADMIN_PASSWORD as distinct high-entropy env values before flipping ENV=prod. AUTH_RETURN_TOKEN defaults off in prod; explicitly set =1 only if a native-mobile client needs the bearer path.</t>
         </is>
       </c>
     </row>
@@ -13908,7 +14014,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="109" t="inlineStr">
         <is>
@@ -13916,7 +14021,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="111" t="inlineStr">
         <is>
@@ -14204,7 +14308,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="111" t="inlineStr">
         <is>
@@ -14457,7 +14560,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="111" t="inlineStr">
         <is>
@@ -14605,7 +14707,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="109" t="inlineStr">
         <is>
@@ -14620,7 +14721,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="111" t="inlineStr">
         <is>
@@ -15096,7 +15196,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="111" t="inlineStr">
         <is>
@@ -15455,7 +15554,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="111" t="inlineStr">
         <is>
@@ -15883,7 +15981,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="109" t="inlineStr">
         <is>
@@ -15898,7 +15995,6 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="112" t="inlineStr">
         <is>
@@ -17356,7 +17452,6 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="109" t="inlineStr">
         <is>
@@ -17371,7 +17466,6 @@
         </is>
       </c>
     </row>
-    <row r="110"/>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="112" t="inlineStr">
         <is>
@@ -17862,7 +17956,6 @@
         </is>
       </c>
     </row>
-    <row r="125"/>
     <row r="126" ht="26" customHeight="1">
       <c r="A126" s="109" t="inlineStr">
         <is>
@@ -17877,7 +17970,6 @@
         </is>
       </c>
     </row>
-    <row r="128"/>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="111" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(tracker): FIX-006-B done -- S0-02 CORS + CSRF shipped
Sprint 0 progress: 5/10 (S0-01/02/08/09/10 done). Fix Log entry
FIX-006-B appended; S0-02 marked Done in Task Backlog. Two
follow-ups logged: FIX-FUP-41 (test-suite asyncio-loop flakiness)
+ FIX-FUP-42 (frontend to send X-CSRF-Token, then flip CSRF_ENFORCE=1).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -2126,20 +2126,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J3" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J3" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K3" s="103" t="inlineStr"/>
-      <c r="L3" s="103" t="inlineStr"/>
-      <c r="M3" s="103" t="inlineStr"/>
+      <c r="L3" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M3" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="N3" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O3" s="22" t="inlineStr"/>
+      <c r="O3" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-B (ababc06). </t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="103" t="inlineStr">
@@ -7653,7 +7665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M88"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12066,6 +12078,183 @@
       <c r="M88" t="inlineStr">
         <is>
           <t>Sprint 0 batch A. 4 launch-blockers shipped together. 337 pre-existing auth/RBAC/session/plans/consent/totp tests still green (zero regressions). Deployment note for ops: set PLATFORM_ADMIN_JWT_SECRET + SUPERADMIN_EMAIL + SUPERADMIN_PASSWORD as distinct high-entropy env values before flipping ENV=prod. AUTH_RETURN_TOKEN defaults off in prod; explicitly set =1 only if a native-mobile client needs the bearer path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>FIX-006-B</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Sprint 0 / Security P0</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>S0-02</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Strict CORS allow-list + CSRF double-submit cookie</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>CORS lockdown: removed allow_origin_regex='.*'+allow_credentials=True combo that echoed back any origin and let evil.com make credentialed cross-origin calls carrying the user's auth cookie. CORS_ORIGINS env is now required in prod (unset or containing '*' makes config.py raise at boot). Dev defaults to local frontend origins. CSRF (double-submit cookie): set_auth_cookie + set_admin_cookie now also set a non-HttpOnly dos_csrf cookie carrying a fresh secrets.token_urlsafe(32) token. Frontend JS reads it and echoes as X-CSRF-Token on every mutating request. New services/csrf.py middleware compares header (constant-time) to cookie on each cookie-authed mutating request. Safe verbs, exempt paths (webhooks + login), and bearer-authed requests bypass. Rollout via CSRF_ENFORCE env -- defaults OFF so this batch ships without a breaking frontend change; middleware logs match/mismatch metrics so ops watches adoption before flipping enforcement on.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>config.py (CORS_ORIGINS strict allow-list parser + prod boot refusal; CSRF_COOKIE_NAME/HEADER_NAME/EXEMPT_PATHS/ENFORCE env plumbing); core.py (set_csrf_cookie/clear_csrf_cookie helpers; set_auth_cookie + set_admin_cookie now mint CSRF cookie; clear paths also clear CSRF); server.py (replaced regex-CORS block with strict allow-list + CSRFMiddleware registration + startup log); services/csrf.py (new: CSRFMiddleware + _check + metrics counters)</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>tests/test_cors_csrf.py -- 31 tests: 7 CORS parsing (prod refuses empty/wildcard/wildcard-mixed, accepts explicit list, strips whitespace/empty, dev fallback, dev override); 6 CSRF cookie minting (auth/admin sets, fresh token per call, clear also clears CSRF, explicit token); 8 check contract (safe verbs, exempt paths, bearer bypass, missing cookie/header, value mismatch, admin cookie equivalence); 3 metrics (counter shape, reset, snapshot returns copy); 4 enforce toggle parsing; 5 middleware dispatch (shadow passes, enforce 403s, matching passes, bearer bypasses, exempt-path bypasses). test_auth_hardening.py refactored to use monkeypatch.setattr on module attrs instead of importlib.reload(config) -- kills the cross-test config pollution that surfaced when TestClient closes shared asyncio loop.</t>
+        </is>
+      </c>
+      <c r="H89" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>ababc06</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Sprint 0 batch B. 405/405 pass across adjacent auth/RBAC/session/plans/consent/totp/tenancy/dockerfile surfaces. test_workflows_dynamic excluded from regression -- pre-existing asyncio.run() vs get_event_loop() interaction is unrelated to this batch (FIX-FUP-41 logged). Deployment: set CORS_ORIGINS to comma-separated exact origins before ENV=prod. Frontend follow-up (FIX-FUP-42): read dos_csrf cookie in JS, send X-CSRF-Token header on mutating requests, then flip CSRF_ENFORCE=1 in prod once staging shows ~100% match rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>FIX-FUP-41</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-006-B)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 0)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Kill test-suite asyncio-loop flakiness</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>test_workflows_dynamic.py uses asyncio.run() which closes the shared event loop, breaking test_deprovisioning/quotas/email_verification that use asyncio.get_event_loop(). Under xdist loadscope both can land on the same worker in an order that trips this. Fix: standardize on asyncio.new_event_loop() everywhere (or asyncio.run everywhere).</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>tests/* (FUP-41) or frontend/src/api (FUP-42)</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>test: cross-worker asyncio stability / frontend integration</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Post-FIX-006-B improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>FIX-FUP-42</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-006-B)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 0)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Frontend: read dos_csrf, send X-CSRF-Token, flip CSRF_ENFORCE</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Read the dos_csrf cookie via document.cookie (non-HttpOnly). Wrap fetch/axios to send X-CSRF-Token header on every POST/PUT/PATCH/DELETE. Watch staging csrf_check_failed logs. Once ~100% match rate, set CSRF_ENFORCE=1 in prod. Middleware will start returning 403 on mismatch.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>tests/* (FUP-41) or frontend/src/api (FUP-42)</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>test: cross-worker asyncio stability / frontend integration</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Post-FIX-006-B improvement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-006-C done -- S0-03/04/05 endpoint P0s shipped
Sprint 0 progress: 8/10 done. Fix Log entry FIX-006-C appended;
S0-03/04/05 marked Done in Task Backlog.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -2199,20 +2199,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J4" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J4" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K4" s="103" t="inlineStr"/>
-      <c r="L4" s="103" t="inlineStr"/>
-      <c r="M4" s="103" t="inlineStr"/>
+      <c r="L4" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M4" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="N4" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O4" s="22" t="inlineStr"/>
+      <c r="O4" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-C (685141d). </t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="103" t="inlineStr">
@@ -2260,20 +2272,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J5" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J5" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K5" s="103" t="inlineStr"/>
-      <c r="L5" s="103" t="inlineStr"/>
-      <c r="M5" s="103" t="inlineStr"/>
+      <c r="L5" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M5" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="N5" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O5" s="22" t="inlineStr"/>
+      <c r="O5" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-C (685141d). </t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="103" t="inlineStr">
@@ -2321,20 +2345,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J6" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J6" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K6" s="103" t="inlineStr"/>
-      <c r="L6" s="103" t="inlineStr"/>
-      <c r="M6" s="103" t="inlineStr"/>
+      <c r="L6" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M6" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="N6" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O6" s="22" t="inlineStr"/>
+      <c r="O6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-C (685141d). </t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="103" t="inlineStr">
@@ -7665,7 +7701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12194,9 +12230,6 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
           <t>Post-FIX-006-B improvement.</t>
@@ -12249,12 +12282,76 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
           <t>Post-FIX-006-B improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>FIX-006-C</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Sprint 0 / Security P0</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>S0-03 + S0-04 + S0-05</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Endpoint P0s (files / OTP / WhatsApp)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>S0-03: GET /api/files/{fname} legacy local-disk fallback is now off-by-default. The old branch served any file on disk to any authenticated caller -- no tenant-ownership check on the legacy path. Gated behind SERVE_LEGACY_LOCAL_DISK env (default False); denied hits logged for observability. S0-04: /auth/otp/request no longer surfaces dev_otp in the JSON body unless DEV_OTP_IN_RESPONSE=1 is explicitly set. server.py now refuses to boot in prod when neither APM_SMS_API_KEY nor TWILIO_* is configured -- silent dev-mode fall-through would hand working login codes to any /auth/otp/request caller. S0-05: WhatsApp webhook rejects (403) on X-Hub-Signature-256 mismatch instead of logging + processing. Also refuses missing WA_APP_SECRET in prod (dev/staging accept with WARN so local tunnels work). hmac.compare_digest preserved for constant-time compare.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>config.py (SERVE_LEGACY_LOCAL_DISK + DEV_OTP_IN_RESPONSE env parsing); server.py (get_file legacy-branch gate + logging; _issue_otp dev_otp gate; TWILIO/APM boot-check raise; whatsapp_webhook 403 on mismatch + prod refuses missing WA_APP_SECRET)</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>tests/test_endpoint_hardening.py -- 14 tests: 4 legacy-disk fallback (source has gate, default off, opt-in works, tenant scope preserved on non-legacy branches); 5 dev-OTP (source gates on flag, default off, opt-in works, prod-boot check exists, end-to-end prod-without-SMS refuses to boot); 5 WhatsApp signature (rejects on mismatch not processes, constant-time compare stays, missing secret rejected in prod, not-configured branch unchanged, HMAC recomputes correctly)</t>
+        </is>
+      </c>
+      <c r="H92" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>685141d</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Sprint 0 batch C. 419/419 pass across adjacent auth/RBAC/session/plans/consent/totp/tenancy surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: set APM_SMS_API_KEY (India) or TWILIO_* (global) before ENV=prod. Set WA_APP_SECRET whenever WhatsApp ingestion is enabled in prod. Leave SERVE_LEGACY_LOCAL_DISK unset in prod.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-006-D done -- SPRINT 0 COMPLETE (10/10)
Sprint 0 launch-blockers all shipped:
  A: superadmin (S0-01) + JWT-in-body (S0-08) + admin JWT split (S0-09)
     + invite invalidation (S0-10)
  B: CORS + CSRF (S0-02)
  C: file downloads (S0-03) + dev-OTP leak (S0-04) + WA signature (S0-05)
  D: unauth-AI guard (S0-06) + login lockout (S0-07)

Fix Log entry FIX-006-D appended; S0-06/07 marked Done in Task Backlog.
One follow-up logged: FIX-FUP-43 (TTL index on user_login_attempts).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -2418,20 +2418,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J7" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J7" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K7" s="103" t="inlineStr"/>
-      <c r="L7" s="103" t="inlineStr"/>
-      <c r="M7" s="103" t="inlineStr"/>
+      <c r="L7" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M7" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="N7" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O7" s="22" t="inlineStr"/>
+      <c r="O7" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-D (93a9f1c). </t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="103" t="inlineStr">
@@ -2479,20 +2491,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J8" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J8" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K8" s="103" t="inlineStr"/>
-      <c r="L8" s="103" t="inlineStr"/>
-      <c r="M8" s="103" t="inlineStr"/>
+      <c r="L8" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M8" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="N8" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O8" s="22" t="inlineStr"/>
+      <c r="O8" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-006-D (93a9f1c). </t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="103" t="inlineStr">
@@ -7701,7 +7725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12352,6 +12376,128 @@
       <c r="M92" t="inlineStr">
         <is>
           <t>Sprint 0 batch C. 419/419 pass across adjacent auth/RBAC/session/plans/consent/totp/tenancy surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: set APM_SMS_API_KEY (India) or TWILIO_* (global) before ENV=prod. Set WA_APP_SECRET whenever WhatsApp ingestion is enabled in prod. Leave SERVE_LEGACY_LOCAL_DISK unset in prod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>FIX-006-D</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Sprint 0 / Security P0</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>S0-06 + S0-07</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Unauth-AI rate-limit/captcha + tenant login lockout</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>S0-06: new shared services.rate_limit.guard_unauth_ai_endpoint() extracts the 3-check pattern (hourly quota + burst quota + CAPTCHA) that signup.py already used, and applies it to the two /api/onboarding/* endpoints that were still unguarded. Both call claude_chat unauthenticated, so drive-by traffic burns real LLM credit. onboarding/os-blueprint is the biggest per-call spend on the pre-auth surface. Per-(service, kind) buckets so signup-drained quotas don't affect onboarding and vice-versa. S0-07: tenant /api/auth/login now has a 5-attempt / 15-min lockout -- parity with admin login. db.user_login_attempts keyed by (IP, email), X-Forwarded-For preferred for real client IP. Lock check runs BEFORE db.users.find_one so timing doesn't leak whether an email exists. Cool-down clears on natural expiry AND on successful login so a slow attacker can't share the cooldown with the legitimate user. Emits login_locked_out audit event.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>services/rate_limit.py (new public guard_unauth_ai_endpoint() with per-service, per-kind buckets + configurable quotas + require_captcha opt-out); routers/onboarding.py (import shared helper; apply guard to onboarding_suggest + onboarding_os_blueprint; both handlers gain request: Request param); routers/auth.py (LOGIN_MAX_ATTEMPTS=5, LOGIN_LOCKOUT_MIN=15 constants; _login_ident/_login_locked_out/_login_record_failure/_login_clear_attempts helpers; login endpoint wires lock check + record-on-fail + clear-on-success + audit login_locked_out event)</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>tests/test_ratelimit_and_lockout.py -- 23 tests: 7 unauth-AI guard (first hit ok, hourly 429, burst 429, captcha required, service isolation, kind isolation, captcha opt-out); 3 endpoint wire-up guards (both onboarding endpoints call shared helper, module imports it); 7 lockout unit tests (ident shape, XFF preference, below/at threshold, window expiry clears, increment upserts, clear wipes, bad iso doesn't perma-lock); 4 login source-inspection guards (lock check before DB find, records on failure, clears on success, 429 not 401, parity numbers with admin login)</t>
+        </is>
+      </c>
+      <c r="H93" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>P0/P1</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>93a9f1c</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Sprint 0 batch D. CLOSES SPRINT 0. 442/442 pass across all adjacent auth/RBAC/session/plans/consent/totp/tenancy/dockerfile test surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: consider adding a Mongo TTL index on user_login_attempts.last (mirrors platform_login_attempts) so expired rows auto-clean -- logged as FIX-FUP-43. In prod, set CAPTCHA_REQUIRED=1 + TURNSTILE_SECRET to hard-enforce captcha on all pre-auth AI endpoints (currently permissive in dev/staging where no secret is set).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>FIX-FUP-43</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-006-D)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 0)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>TTL index on user_login_attempts.last</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Mirror the scheduler_locks / platform_login_attempts TTL pattern: create index on db.user_login_attempts.last with expireAfterSeconds = LOGIN_LOCKOUT_MIN * 60 * 2 (double the window so a fresh row can still exist for its full useful life). Kills row buildup for attackers who spray many (IP, email) pairs.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>server.py bootstrap indexes block; services/auth or routers/auth (where LOGIN_LOCKOUT_MIN is defined)</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>test: index exists on collection after bootstrap; row inserted at T=0 gone after T=LOGIN_LOCKOUT_MIN*2</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Post-Sprint-0 hygiene.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-007-A done -- Sprint 4 hygiene batch shipped
S4-01 (text-index stemming + memory index), S4-03 (brain_contexts
rename), S4-11 (tenant/industry vocab) all Done in Task Backlog;
FIX-007-A row appended to Fix Log.

Sprint 4 Brain: 3/11 done. Ready for FIX-007-B (write coverage:
S4-02 + S4-10) next.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -4373,20 +4373,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J34" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J34" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K34" s="103" t="inlineStr"/>
-      <c r="L34" s="103" t="inlineStr"/>
-      <c r="M34" s="103" t="inlineStr"/>
+      <c r="L34" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M34" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="N34" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O34" s="22" t="inlineStr"/>
+      <c r="O34" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-007-A (c4f3f88). </t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="A35" s="103" t="inlineStr">
@@ -4495,20 +4507,32 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J36" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J36" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K36" s="103" t="inlineStr"/>
-      <c r="L36" s="103" t="inlineStr"/>
-      <c r="M36" s="103" t="inlineStr"/>
+      <c r="L36" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M36" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="N36" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O36" s="22" t="inlineStr"/>
+      <c r="O36" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-007-A (c4f3f88). </t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="32" customHeight="1">
       <c r="A37" s="103" t="inlineStr">
@@ -4983,20 +5007,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J44" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J44" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K44" s="103" t="inlineStr"/>
-      <c r="L44" s="103" t="inlineStr"/>
-      <c r="M44" s="103" t="inlineStr"/>
+      <c r="L44" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M44" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="N44" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O44" s="22" t="inlineStr"/>
+      <c r="O44" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-007-A (c4f3f88). </t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="32" customHeight="1">
       <c r="A45" s="103" t="inlineStr">
@@ -7725,7 +7761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M94"/>
+  <dimension ref="A1:M95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12492,12 +12528,76 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
           <t>Post-Sprint-0 hygiene.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>FIX-007-A</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Sprint 4 / Brain hygiene</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>S4-01 + S4-03 + S4-11</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Brain hygiene: text-index stemming, brain_contexts rename, tenant/industry vocab</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>S4-01: brain_context_text_v1 and brain_documents_text_v1 rebuilt with default_language='english' (was 'none') so Mongo's snowball stemmer kicks in -- 'refund' now matches 'refunds'/'refunded'. NEW memory_text_v1 text index on db.memory. Mongo doesn't let you mutate default_language on an existing text index, so drop_none_language_text_indexes_v1 migration drops stale 'none' indexes once; create_index rebuilds them with english. S4-03: brain_contexts (plural /ask query-plan cache) renamed to brain_query_cache -- the singular/plural collision with brain_context (decision-provenance store) was a silent-corruption foot-gun. rename_brain_contexts_to_query_cache_v1 migration uses Mongo's atomic renameCollection; guarded on source-has-data + target-absent. All 3 hot-path call sites in routers/brain.py updated. TENANT_COLLECTIONS wipe list carries BOTH names during transition. S4-11: _TAG_VOCAB was 10 hardcoded manufacturing patterns -- clinics, restaurants, agencies, retail were silently under-tagged. Renamed to _BASE_TAG_VOCAB (compat alias kept). New INDUSTRY_VOCAB for 11 industries (manufacturing, healthcare, clinic, restaurant, restaurant/hospitality, agency, retail, services, logistics, education, construction). Tenants override via tenant.brain_tag_vocab = [{tag, pattern}]. Precedence: tenant custom &gt; industry &gt; base (dedup by tag key). record_context reads tenant.industry + brain_tag_vocab at record time. Malformed regexes skipped silently. 100% backward compatible.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>server.py (2 migrations added + english default_language on 2 text indexes + new memory text index + brain_query_cache indexes); routers/brain.py (3 db call sites: brain_contexts -&gt; brain_query_cache); routers/admin.py (TENANT_COLLECTIONS carries both names); services/ai/brain_context.py (_BASE_TAG_VOCAB rename + INDUSTRY_VOCAB for 11 industries + _industry_key resolver + _resolve_vocab precedence chain + _load_tenant_vocab_shape helper + record_context wired to pass industry+custom into auto_tags)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>tests/test_brain_hygiene.py -- 27 tests: S4-01 (6): source guards for english language on brain_context / brain_documents / memory + memory_text_v1 weights + drop-migration registered + runs before rebuild. S4-03 (7): no hot-path calls to old collection + new indexes created + wipe list carries both + rename migration checks source/target + uses Mongo renameCollection. S4-11 (14): base vocab shape + legacy alias points at base + no-industry back-compat + clinic/restaurant/agency/healthcare alias industries + unknown industry fall-back + fuzzy key match + tenant custom wins over base + tenant adds new tag + malformed regex tolerated + half-written entries tolerated + precedence chain + industry ordered before base + record_context wiring + fail-open on DB blip</t>
+        </is>
+      </c>
+      <c r="H95" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>P1/P2</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>c4f3f88</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Sprint 4 batch A (Brain hygiene). 469/469 pass across all adjacent brain-hygiene / rate-limit / endpoint-hardening / cors-csrf / auth-hardening / totp / email-verify / memberships / session-revocation / rbac-wave-1/3 / audit-log / session-mgmt / deprovisioning / plans / quotas / ai-consent / tenancy-hygiene / dockerfile surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: migrations auto-run on first boot via ledger. The rename uses Mongo's renameCollection admin command -- Atlas + Railway MongoDB both grant this by default. No data migration for S4-11: tenants with industry set start getting industry-aware tags on the next record_context write. Old rows stay as-is.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-007-B done -- Sprint 4 write coverage shipped
S4-02 (task provenance / execution-plan gap + decision_id linkage)
and S4-10 (finance + workflow + meetings Brain writes) both Done
in Task Backlog. FIX-007-B row appended to Fix Log. One follow-up
logged: FIX-FUP-44 (WhatsApp + doc-upload ingestion coverage).

Sprint 4 Brain: 5/11 done. Ready for FIX-007-C (retrieval
unification: S4-04) next.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -4446,20 +4446,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J35" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J35" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K35" s="103" t="inlineStr"/>
-      <c r="L35" s="103" t="inlineStr"/>
-      <c r="M35" s="103" t="inlineStr"/>
+      <c r="L35" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M35" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="N35" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O35" s="22" t="inlineStr"/>
+      <c r="O35" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-007-B (8ad22fd). </t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="103" t="inlineStr">
@@ -4946,20 +4958,32 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J43" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J43" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K43" s="103" t="inlineStr"/>
-      <c r="L43" s="103" t="inlineStr"/>
-      <c r="M43" s="103" t="inlineStr"/>
+      <c r="L43" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M43" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="N43" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O43" s="22" t="inlineStr"/>
+      <c r="O43" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-007-B (8ad22fd). </t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="32" customHeight="1">
       <c r="A44" s="103" t="inlineStr">
@@ -7761,7 +7785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M95"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12598,6 +12622,128 @@
       <c r="M95" t="inlineStr">
         <is>
           <t>Sprint 4 batch A (Brain hygiene). 469/469 pass across all adjacent brain-hygiene / rate-limit / endpoint-hardening / cors-csrf / auth-hardening / totp / email-verify / memberships / session-revocation / rbac-wave-1/3 / audit-log / session-mgmt / deprovisioning / plans / quotas / ai-consent / tenancy-hygiene / dockerfile surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: migrations auto-run on first boot via ledger. The rename uses Mongo's renameCollection admin command -- Atlas + Railway MongoDB both grant this by default. No data migration for S4-11: tenants with industry set start getting industry-aware tags on the next record_context write. Old rows stay as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>FIX-007-B</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Sprint 4 / Brain write coverage</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>S4-02 + S4-10</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Brain write coverage: task-provenance + finance/workflow/meetings</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>S4-02: record_context() gained first-class decision_id + related_ids params so decision -&gt; task -&gt; outcome chains are queryable. Stored only when present (no null spam). The gap this fixed: save_execution_plan auto-transitioned tasks to done when their plan hit 100%, but was the ONE completion path skipping record_context. Now parity with the PATCH /tasks/{id} status=done path. All 3 existing task-lifecycle sites (task_done / approve / reject) thread t.get('decision_id') through. S4-10: five new event kinds captured (workflow, finance, meeting, ingestion added to KIND_VALUES). advance_workflow drops a workflow row on every stage advance (terminal stage -&gt; outcome=completed). process_meeting writes one Brain row when notes finalize. create_expense + create_income write finance rows (non-manual only, manual entries stay Brain-invisible unless write_brain=True). reconcile_payment writes AFTER the no-match early return so unmatched payments don't spam the Brain. All 5 sites wrapped in try/except -- fail-open, never 500 the parent operation.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>services/ai/brain_context.py (record_context signature + KIND_VALUES); routers/tasks.py (3 call sites thread decision_id + save_execution_plan gains the missing record_context); server.py (advance_workflow + process_meeting Brain writes); routers/ledger.py (import brain_context + create_expense/create_income/reconcile_payment Brain writes)</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>tests/test_brain_write_coverage.py -- 23 tests: S4-02 (11): signature has decision_id+related_ids as keyword-only with None defaults; decision_id only stored when provided + length-capped; related_ids only stored when non-empty + None values dropped; KIND_VALUES expanded; old kinds preserved; unknown kind falls back to note; 3 task call sites thread decision_id; save_execution_plan writes record_context; write inside status=done branch. S4-10 (9): advance_workflow calls record_context + kind=workflow + terminal outcome=completed + decision_id passthrough + fail-open; process_meeting writes kind=meeting; create_expense writes kind=finance inside write_brain gate; create_income writes kind=finance; reconcile_payment writes AFTER no-match return; all 3 ledger writes wrapped in try. E2E (2): full workflow-row shape lands with all new fields; record_context never raises on Mongo blip.</t>
+        </is>
+      </c>
+      <c r="H96" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>8ad22fd</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Sprint 4 batch B (Brain write coverage). 492/492 pass across all adjacent test surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: additive change to record_context signature is 100% backward compatible. Existing DB indexes cover the new rows since brain_context is already indexed by (tenant_id, created_at) + (tenant_id, kind, created_at). Future query pattern 'downstream of decision X' -- consider indexing (tenant_id, decision_id) once S4-04 unifies /ask and /brain/agent retrieval reach in batch C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>FIX-FUP-44</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Follow-up (from FIX-007-B)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>(logged during Sprint 4)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Extend Brain write coverage to WhatsApp + doc-upload ingestion</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>process_whatsapp_message (server.py:5112) branches text / document / audio through persist_capture_draft -- each promotion to a decision or capture_draft should also drop a brain_context row of kind=ingestion so 'what was that WhatsApp message about the Sharma delivery?' resolves. Same for the two direct db.ingestions.insert_one sites (server.py:4381 and 4437) that back the doc-upload endpoint. Worth its own targeted batch rather than a scatter of adds during S4-10 -- design pass first so we don't double-write (capture_draft -&gt; decision -&gt; record_context).</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>server.py (process_whatsapp_message + doc-ingest endpoints); possibly a new helper in services/ai/brain_context.py for the ingestion -&gt; decision promotion path so both channels share one shape</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>test: text/document/audio inbound WA messages each land a brain_context row; doc-upload also lands one; no duplicate rows for a WA capture that later promotes to a decision</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Post-FIX-007-B improvement. Covers the 'ingestion' KIND value that FIX-007-B added to KIND_VALUES but doesn't yet emit anywhere.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FIX-007-C done -- Sprint 4 retrieval unification shipped
S4-04 marked Done in Task Backlog; FIX-007-C row appended to Fix Log.

Sprint 4 Brain: 6/11 done. Ready for FIX-007-D (batch D: embeddings +
hybrid retrieval — S4-05/06) next.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -4592,20 +4592,32 @@
           <t>M</t>
         </is>
       </c>
-      <c r="J37" s="37" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="J37" s="104" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K37" s="103" t="inlineStr"/>
-      <c r="L37" s="103" t="inlineStr"/>
-      <c r="M37" s="103" t="inlineStr"/>
+      <c r="L37" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M37" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="N37" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O37" s="22" t="inlineStr"/>
+      <c r="O37" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shipped in FIX-007-C (c9e4916). </t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="32" customHeight="1">
       <c r="A38" s="103" t="inlineStr">
@@ -7785,7 +7797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M97"/>
+  <dimension ref="A1:M98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12738,12 +12750,76 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
           <t>Post-FIX-007-B improvement. Covers the 'ingestion' KIND value that FIX-007-B added to KIND_VALUES but doesn't yet emit anywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>FIX-007-C</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Sprint 4 / Brain retrieval unification</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>S4-04</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>/ask and /brain/agent now share one retrieval code path</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Before: /ask only queried domain tables (tasks/invoices/decisions/etc.) -- completely blind to brain_context (provenance) and brain_documents (policies). Dex was the only surface where 'how did we handle the last vendor delay?' returned real answers. Two problems: product surface inconsistency (same question, different answer quality) + code drift risk (Mongo queries duplicated between the two routers). Fix: new services/ai/brain_retrieval.py with search_documents() + search_context() + cites_from_hits(). Both routers hit this shared entrypoint -- future S4-05/06 embedding upgrades land in one place and both surfaces benefit. /ask now enriches every answer with top-N brain_context + brain_documents hits keyed by plan keywords. INSUFFICIENT_DATA short-circuit updated to check Brain extras so /ask no longer says 'no data' when the Brain has provenance/document matches.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>services/ai/brain_retrieval.py (NEW: search_documents + search_context + cites_from_hits, shared retrieval layer); routers/brain.py (import brain_retrieval; new _enrich_with_brain helper; _retrieve gains optional user=None param; _answer accepts knowledge_hits + document_hits; /ask endpoint merges domain + Brain citations; INSUFFICIENT_DATA respects extras); routers/brain_router.py (_tool_metadata_search + _tool_knowledge_lookup collapsed from ~40 lines to 3-line delegations to the shared service; runtime dict shape unchanged)</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>tests/test_brain_retrieval_unified.py -- 20 tests: Service (10): search_documents text-index path + empty-query fallback + fail-open + owner bypasses visibility; search_context delegates correctly + fail-open; cites_from_hits shapes docs/context + merges docs-first + fallback title chain. /ask wiring (4): _enrich_with_brain calls both stores; handles keywords list vs string; _retrieve signature backward-compat; _answer signature accepts hits. /brain/agent (4): both tools use shared service; direct Mongo hits removed; runtime dict shape unchanged for both. E2E (2): /ask merges extras into sources; INSUFFICIENT_DATA short-circuit respects Brain hits.</t>
+        </is>
+      </c>
+      <c r="H98" s="106" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>c9e4916</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Sprint 4 batch C (retrieval unification). 512/512 pass across all adjacent test surfaces. test_workflows_dynamic still excluded per FIX-FUP-41. Deployment: additive change -- the enrichment pass is best-effort and fails open; no schema migrations, no index changes needed beyond what S4-01 already delivered. Prod behaviour: /ask answers gain 2 new signal streams (past_context + policies) in the LLM prompt, so answer quality improves for provenance / policy questions without any config toggle. Downstream setup: batch D (S4-05 + S4-06) now has one code path to upgrade -- embeddings + hybrid rerank land inside services/ai/brain_retrieval.search_documents and both surfaces get vector search for free.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): FUP-48 — workflow board doesn't advance when tasks complete
Live multi-user E2E test on 2026-08-13 (Kapoor Cotton Mills / Delhi
Retail Corp order) surfaced the exact bug the workflow-engine spec
was written for. 3 users completed all 3 tasks belonging to a
workflow card. brain_context correctly linked each task_done row
to the parent decision_id (FIX-007-B working). But the workflow
card stayed stuck at stage 'order_received' -- no auto-advance,
history=1. Founder sees a stuck kanban even though every underlying
task is done.

Fix is the 3-phase rebuild already scoped in docs/DecisionOS_
Workflow_Engine_Spec.pptx (+ Testing_Plan.pptx). Tracker entry
carries the live repro + points at the spec/test deck.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
+++ b/docs/DecisionOS_SaaS_Stability_Tracker.xlsx
@@ -1910,7 +1910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O87"/>
+  <dimension ref="A1:O88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7923,6 +7923,63 @@
       <c r="O87" t="inlineStr">
         <is>
           <t>LIVE-TEST EXAMPLE (2026-08-13): Kapoor Retail decision spawned 3 tasks - all had assignee_role (production/sales/finance) but assignee_id was null. /ask response flagged 'immediate risk of missing deadlines' because ownership was unassigned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>FUP-48</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Data model / UX</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Workflow engine rebuild -- wire task completion to workflow advance</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Tasks + workflows are two collections with no lifecycle link. Completing a task never advances the parent workflow card. Founder sees a stuck kanban. Full spec + test plan already in docs/DecisionOS_Workflow_Engine_Spec.pptx + Testing_Plan.pptx (3 phases, 4-6 sessions).</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Live E2E 2026-08-13 + Workflow Engine Spec</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>LIVE-TEST EXAMPLE (2026-08-13): 3 users completed all 3 Delhi Retail tasks. Every task = done. brain_context linked all 3 back to parent decision. But the pipeline card for 'Delhi Retail Corp -- 2000m Mixed Cotton &amp; Silk Fabric' stayed at 'order_received'. Needs 4 manual Advance clicks to move through the stages even though the underlying work is finished. Also blocks FIX-001-B auto-expense (only fires on terminal-stage advance).</t>
         </is>
       </c>
     </row>
@@ -7968,7 +8025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M101"/>
+  <dimension ref="A1:M102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13040,9 +13097,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
           <t>LIVE-TEST EXAMPLE (2026-08-13, Kapoor Cotton Mills tenant): typed 'Confirmed a bulk order from Kapoor Retail...' in Decision Desk, clicked 'Structure it'. Nothing happened on screen. Network tab showed POST /api/capture/clarify -&gt; 451, voice-note persisted but no AI output. Only after granting consent via curl did retry succeed. Real user would think the app is broken. Spawned chip task_e8077ebe also tracks this.</t>
@@ -13095,9 +13149,6 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
           <t>LIVE-TEST EXAMPLE (2026-08-13): I signed up 'Kapoor Cotton Mills' with email amit@kapoorcotton.test. Wizard completed, blueprint generated, clicked 'Looks good - Enter DecisionOS'. Nothing visible happened. Backend network trace showed 422 {'value is not a valid email address: The part after the @-sign is a special-use or reserved name that cannot be used with email.'}. Had to open DevTools to know why. First-time signups with typo'd or corporate-firewall-blocked email domains will hit this and silently drop off.</t>
@@ -13150,12 +13201,64 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
           <t>LIVE-TEST EXAMPLE (2026-08-13): the Kapoor decision approval created 3 tasks (Allocate stock -&gt; production, Confirm delivery slot -&gt; sales, Raise GST invoice -&gt; finance). All three had assignee_role set correctly but assignee_id was null. The /ask response called this out as a risk: 'all 3 tasks remain unassigned and in To Do status. No tasks are overdue yet, but with no assignees in place, there is an immediate risk of missing these deadlines. Ownership needs to be assigned urgently across Finance, Sales, and Production.'  Real founders will find this friction and blame the AI instead of the onboarding gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>FIX-FUP-48</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Follow-up (from live multi-user E2E 2026-08-13)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>(matches workflow-engine spec deck)</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Workflow board does NOT advance when its tasks complete</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>The workflow-engine spec I authored earlier (docs/DecisionOS_Workflow_Engine_Spec.pptx) identified 'tasks and workflows are strangers' as the core bug. This E2E test proves it is live and customer-visible: 3 people finished all 3 tasks belonging to a workflow card, brain_context correctly linked each task_done row back to the parent decision_id, but the workflow card stayed stuck at stage 1 because nothing wires task completion to workflow advance. The founder opens the board and sees 'nothing moved' -- exactly the trust-breaker the spec warned about. Fix = the 3-phase rebuild in the spec: Phase 1 unify data model (add tasks.workflow_id + stage_key), Phase 2 workflow_engine.py transition operations (on_stage_enter, check_stage_ready, advance), Phase 3 joined My-Work + Workflow view with stage chips. Not a small item -- 4-6 sessions per the spec's timeline -- but the ONE change that converts DecisionOS from 'AI captures tasks' to 'AI runs the operation'.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>See docs/DecisionOS_Workflow_Engine_Spec.pptx sections 03 (backend) + 04 (UI); planned modules: services/workflow_engine.py (new), routers/workflows.py, routers/tasks.py, server.py, migration ledger (3 new migrations)</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>See docs/DecisionOS_Workflow_Engine_Testing_Plan.pptx -- full test plan already written. Golden-path E2E: capture -&gt; approve -&gt; assignee closes task -&gt; card auto-advances -&gt; next stage tasks auto-spawn -&gt; repeat to terminal -&gt; side-effect fires.</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>LIVE-TEST EXAMPLE (2026-08-13, Kapoor Cotton Mills / Delhi Retail Corp order): Owner Amit captured 'Big rush order from Delhi Retail Corp -- 2000m mixed cotton and silk...' Decision approved, 3 tasks auto-assigned (Priya finance, Neha production, Rahul sales). All 3 logged in, marked their task done. brain_context correctly recorded 3 task_done rows all linked back to decision_id=8add0963. But the 'Delhi Retail Corp -- 2000m Mixed Cotton &amp; Silk Fabric' workflow card STAYED at stage 'order_received' with history=1. It requires 4 manual Advance clicks (Order Received -&gt; Confirmed -&gt; In Production -&gt; Ready) to move through, even though every underlying task is done. Also related: FIX-001-B finance auto-expense on terminal-stage advance NEVER fires unless someone manually clicks Advance all the way through. Silent revenue-tracking gap.</t>
         </is>
       </c>
     </row>

</xml_diff>